<commit_message>
Atualiza Superestrutura · 2026-09-10T14:46:06.425-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="192" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{989A7F9E-5B93-400A-BFE0-2756F5F80232}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{398FB898-2747-4987-A581-7EEB61709DD9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3128,12 +3128,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3159,6 +3153,12 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3724,38 +3724,6 @@
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="ENTRADA"/>
-      <sheetName val="CURVAS"/>
-      <sheetName val="HISTOGRAMA"/>
-      <sheetName val="SERVIÇOS NOTÁVEIS"/>
-      <sheetName val="LASTRO"/>
-      <sheetName val="MATERIAIS"/>
-      <sheetName val="PONTOS DE ATENÇÃO"/>
-      <sheetName val="PLANO DE AÇÃO"/>
-      <sheetName val="Modelo Acompanhamento Super2 - "/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
@@ -3904,6 +3872,42 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="ENTRADA"/>
+      <sheetName val="CURVAS"/>
+      <sheetName val="HISTOGRAMA"/>
+      <sheetName val="SERVIÇOS NOTÁVEIS"/>
+      <sheetName val="LASTRO"/>
+      <sheetName val="MATERIAIS"/>
+      <sheetName val="PONTOS DE ATENÇÃO"/>
+      <sheetName val="PLANO DE AÇÃO"/>
+      <sheetName val="Modelo Acompanhamento Super2 - "/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4149,56 +4153,56 @@
   <sheetData>
     <row r="1" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="196" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="197"/>
-      <c r="D2" s="197"/>
-      <c r="E2" s="197"/>
-      <c r="F2" s="197"/>
-      <c r="G2" s="197"/>
+      <c r="B2" s="194" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="195"/>
+      <c r="D2" s="195"/>
+      <c r="E2" s="195"/>
+      <c r="F2" s="195"/>
+      <c r="G2" s="195"/>
     </row>
     <row r="3" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="198" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="199"/>
-      <c r="D3" s="199"/>
-      <c r="E3" s="199"/>
-      <c r="F3" s="199"/>
-      <c r="G3" s="200"/>
+      <c r="B3" s="196" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="197"/>
+      <c r="D3" s="197"/>
+      <c r="E3" s="197"/>
+      <c r="F3" s="197"/>
+      <c r="G3" s="198"/>
     </row>
     <row r="4" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="201"/>
-      <c r="C4" s="197"/>
-      <c r="D4" s="197"/>
-      <c r="E4" s="197"/>
-      <c r="F4" s="197"/>
-      <c r="G4" s="202"/>
+      <c r="B4" s="199"/>
+      <c r="C4" s="195"/>
+      <c r="D4" s="195"/>
+      <c r="E4" s="195"/>
+      <c r="F4" s="195"/>
+      <c r="G4" s="200"/>
     </row>
     <row r="5" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="201"/>
-      <c r="C5" s="197"/>
-      <c r="D5" s="197"/>
-      <c r="E5" s="197"/>
-      <c r="F5" s="197"/>
-      <c r="G5" s="202"/>
+      <c r="B5" s="199"/>
+      <c r="C5" s="195"/>
+      <c r="D5" s="195"/>
+      <c r="E5" s="195"/>
+      <c r="F5" s="195"/>
+      <c r="G5" s="200"/>
     </row>
     <row r="6" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="201"/>
-      <c r="C6" s="197"/>
-      <c r="D6" s="197"/>
-      <c r="E6" s="197"/>
-      <c r="F6" s="197"/>
-      <c r="G6" s="202"/>
+      <c r="B6" s="199"/>
+      <c r="C6" s="195"/>
+      <c r="D6" s="195"/>
+      <c r="E6" s="195"/>
+      <c r="F6" s="195"/>
+      <c r="G6" s="200"/>
     </row>
     <row r="7" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="203"/>
-      <c r="C7" s="204"/>
-      <c r="D7" s="204"/>
-      <c r="E7" s="204"/>
-      <c r="F7" s="204"/>
-      <c r="G7" s="205"/>
+      <c r="B7" s="201"/>
+      <c r="C7" s="202"/>
+      <c r="D7" s="202"/>
+      <c r="E7" s="202"/>
+      <c r="F7" s="202"/>
+      <c r="G7" s="203"/>
     </row>
     <row r="8" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4301,7 +4305,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="80">
-        <v>93100</v>
+        <v>95540</v>
       </c>
       <c r="E15" s="79"/>
       <c r="F15" s="80"/>
@@ -4324,7 +4328,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="80">
-        <v>79240</v>
+        <v>82860</v>
       </c>
       <c r="E16" s="79"/>
       <c r="F16" s="80"/>
@@ -4347,7 +4351,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="80">
-        <v>80880</v>
+        <v>82860</v>
       </c>
       <c r="E17" s="79"/>
       <c r="F17" s="80"/>
@@ -4430,7 +4434,7 @@
         <v>23000</v>
       </c>
       <c r="F20" s="80">
-        <v>45000</v>
+        <v>47100</v>
       </c>
       <c r="G20" s="79">
         <v>60160</v>
@@ -4526,8 +4530,12 @@
       <c r="F23" s="80">
         <v>31650</v>
       </c>
-      <c r="G23" s="79"/>
-      <c r="H23" s="80"/>
+      <c r="G23" s="79">
+        <v>34980</v>
+      </c>
+      <c r="H23" s="80">
+        <v>36700</v>
+      </c>
       <c r="I23" s="79"/>
       <c r="J23" s="80"/>
       <c r="K23" s="79"/>
@@ -4640,7 +4648,7 @@
         <v>11607</v>
       </c>
       <c r="F27" s="80">
-        <v>19269</v>
+        <v>23792</v>
       </c>
       <c r="G27" s="79"/>
       <c r="H27" s="80"/>
@@ -6222,31 +6230,31 @@
         <v>55</v>
       </c>
       <c r="B22" s="87">
-        <f>[2]HISTOGRAMA!C33</f>
+        <f>[1]HISTOGRAMA!C33</f>
         <v>5</v>
       </c>
       <c r="C22" s="87">
-        <f>[2]HISTOGRAMA!E33</f>
+        <f>[1]HISTOGRAMA!E33</f>
         <v>89</v>
       </c>
       <c r="D22" s="87">
-        <f>[2]HISTOGRAMA!G33</f>
+        <f>[1]HISTOGRAMA!G33</f>
         <v>127</v>
       </c>
       <c r="E22" s="87">
-        <f>[2]HISTOGRAMA!I33</f>
+        <f>[1]HISTOGRAMA!I33</f>
         <v>150</v>
       </c>
       <c r="F22" s="87">
-        <f>[2]HISTOGRAMA!K33</f>
+        <f>[1]HISTOGRAMA!K33</f>
         <v>144</v>
       </c>
       <c r="G22" s="87">
-        <f>[2]HISTOGRAMA!M33</f>
+        <f>[1]HISTOGRAMA!M33</f>
         <v>194</v>
       </c>
       <c r="H22" s="87">
-        <f>[2]HISTOGRAMA!O33</f>
+        <f>[1]HISTOGRAMA!O33</f>
         <v>198</v>
       </c>
       <c r="I22" s="87">
@@ -6451,35 +6459,35 @@
         <v>55</v>
       </c>
       <c r="B27" s="87">
-        <f>[2]HISTOGRAMA!C79</f>
+        <f>[1]HISTOGRAMA!C79</f>
         <v>4</v>
       </c>
       <c r="C27" s="87">
-        <f>[2]HISTOGRAMA!E79</f>
+        <f>[1]HISTOGRAMA!E79</f>
         <v>34</v>
       </c>
       <c r="D27" s="87">
-        <f>[2]HISTOGRAMA!G79</f>
+        <f>[1]HISTOGRAMA!G79</f>
         <v>56</v>
       </c>
       <c r="E27" s="87">
-        <f>[2]HISTOGRAMA!I79</f>
+        <f>[1]HISTOGRAMA!I79</f>
         <v>64</v>
       </c>
       <c r="F27" s="87">
-        <f>[2]HISTOGRAMA!K79</f>
+        <f>[1]HISTOGRAMA!K79</f>
         <v>72</v>
       </c>
       <c r="G27" s="87">
-        <f>[2]HISTOGRAMA!M79</f>
+        <f>[1]HISTOGRAMA!M79</f>
         <v>84</v>
       </c>
       <c r="H27" s="87">
-        <f>[2]HISTOGRAMA!O79</f>
+        <f>[1]HISTOGRAMA!O79</f>
         <v>88</v>
       </c>
       <c r="I27" s="87">
-        <f>[2]HISTOGRAMA!Q79</f>
+        <f>[1]HISTOGRAMA!Q79</f>
         <v>102</v>
       </c>
       <c r="J27" s="88">
@@ -6681,35 +6689,35 @@
         <v>55</v>
       </c>
       <c r="B32" s="87">
-        <f>[2]HISTOGRAMA!C116</f>
+        <f>[1]HISTOGRAMA!C116</f>
         <v>1</v>
       </c>
       <c r="C32" s="87">
-        <f>[2]HISTOGRAMA!E116</f>
+        <f>[1]HISTOGRAMA!E116</f>
         <v>11</v>
       </c>
       <c r="D32" s="87">
-        <f>[2]HISTOGRAMA!G116</f>
+        <f>[1]HISTOGRAMA!G116</f>
         <v>17</v>
       </c>
       <c r="E32" s="87">
-        <f>[2]HISTOGRAMA!I116</f>
+        <f>[1]HISTOGRAMA!I116</f>
         <v>21</v>
       </c>
       <c r="F32" s="87">
-        <f>[2]HISTOGRAMA!K116</f>
+        <f>[1]HISTOGRAMA!K116</f>
         <v>26</v>
       </c>
       <c r="G32" s="87">
-        <f>[2]HISTOGRAMA!M116</f>
+        <f>[1]HISTOGRAMA!M116</f>
         <v>32</v>
       </c>
       <c r="H32" s="87">
-        <f>[2]HISTOGRAMA!O116</f>
+        <f>[1]HISTOGRAMA!O116</f>
         <v>38</v>
       </c>
       <c r="I32" s="87">
-        <f>[2]HISTOGRAMA!Q116</f>
+        <f>[1]HISTOGRAMA!Q116</f>
         <v>44</v>
       </c>
       <c r="J32" s="88">
@@ -6911,35 +6919,35 @@
         <v>55</v>
       </c>
       <c r="B37" s="87">
-        <f>[2]HISTOGRAMA!C90</f>
+        <f>[1]HISTOGRAMA!C90</f>
         <v>0</v>
       </c>
       <c r="C37" s="87">
-        <f>[2]HISTOGRAMA!E90</f>
+        <f>[1]HISTOGRAMA!E90</f>
         <v>13</v>
       </c>
       <c r="D37" s="87">
-        <f>[2]HISTOGRAMA!G90</f>
+        <f>[1]HISTOGRAMA!G90</f>
         <v>25</v>
       </c>
       <c r="E37" s="87">
-        <f>[2]HISTOGRAMA!I90</f>
+        <f>[1]HISTOGRAMA!I90</f>
         <v>25</v>
       </c>
       <c r="F37" s="87">
-        <f>[2]HISTOGRAMA!K90</f>
+        <f>[1]HISTOGRAMA!K90</f>
         <v>38</v>
       </c>
       <c r="G37" s="87">
-        <f>[2]HISTOGRAMA!M90</f>
+        <f>[1]HISTOGRAMA!M90</f>
         <v>41</v>
       </c>
       <c r="H37" s="87">
-        <f>[2]HISTOGRAMA!O90</f>
+        <f>[1]HISTOGRAMA!O90</f>
         <v>42</v>
       </c>
       <c r="I37" s="87">
-        <f>[2]HISTOGRAMA!Q90</f>
+        <f>[1]HISTOGRAMA!Q90</f>
         <v>47</v>
       </c>
       <c r="J37" s="88">
@@ -12486,7 +12494,7 @@
       <c r="O34" s="15"/>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A35" s="206" t="s">
+      <c r="A35" s="204" t="s">
         <v>97</v>
       </c>
       <c r="B35" s="90">
@@ -12652,7 +12660,7 @@
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A36" s="207"/>
+      <c r="A36" s="205"/>
       <c r="B36" s="97" t="s">
         <v>63</v>
       </c>
@@ -19934,7 +19942,7 @@
       <c r="O80" s="15"/>
     </row>
     <row r="81" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A81" s="206" t="s">
+      <c r="A81" s="204" t="s">
         <v>140</v>
       </c>
       <c r="B81" s="90">
@@ -20100,7 +20108,7 @@
       </c>
     </row>
     <row r="82" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A82" s="208"/>
+      <c r="A82" s="206"/>
       <c r="B82" s="97" t="s">
         <v>63</v>
       </c>
@@ -21726,7 +21734,7 @@
       <c r="O91" s="15"/>
     </row>
     <row r="92" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A92" s="206" t="s">
+      <c r="A92" s="204" t="s">
         <v>145</v>
       </c>
       <c r="B92" s="90">
@@ -21892,7 +21900,7 @@
       </c>
     </row>
     <row r="93" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A93" s="207"/>
+      <c r="A93" s="205"/>
       <c r="B93" s="97" t="s">
         <v>63</v>
       </c>
@@ -58557,7 +58565,7 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <f>SUM([2]LASTRO!D2,[2]LASTRO!G2)/1.39</f>
+        <f>SUM([1]LASTRO!D2,[1]LASTRO!G2)/1.39</f>
         <v>189335.95683453238</v>
       </c>
       <c r="N15" s="72">
@@ -58589,25 +58597,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="209" t="s">
+      <c r="A1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="209" t="s">
+      <c r="B1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="209" t="s">
+      <c r="C1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="209" t="s">
+      <c r="D1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="209" t="s">
+      <c r="E1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="F1" s="209" t="s">
+      <c r="F1" s="207" t="s">
         <v>251</v>
       </c>
-      <c r="G1" s="209" t="s">
+      <c r="G1" s="207" t="s">
         <v>251</v>
       </c>
     </row>
@@ -59142,43 +59150,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="194" t="s">
+      <c r="A1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="B1" s="194" t="s">
+      <c r="B1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="C1" s="194" t="s">
+      <c r="C1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="D1" s="194" t="s">
+      <c r="D1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="E1" s="194" t="s">
+      <c r="E1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="F1" s="194" t="s">
+      <c r="F1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="G1" s="194" t="s">
+      <c r="G1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="H1" s="194" t="s">
+      <c r="H1" s="208" t="s">
         <v>319</v>
       </c>
-      <c r="J1" s="195" t="s">
+      <c r="J1" s="209" t="s">
         <v>320</v>
       </c>
-      <c r="K1" s="195" t="s">
+      <c r="K1" s="209" t="s">
         <v>320</v>
       </c>
-      <c r="L1" s="195" t="s">
+      <c r="L1" s="209" t="s">
         <v>320</v>
       </c>
-      <c r="M1" s="195" t="s">
+      <c r="M1" s="209" t="s">
         <v>320</v>
       </c>
-      <c r="N1" s="195" t="s">
+      <c r="N1" s="209" t="s">
         <v>320</v>
       </c>
     </row>
@@ -59821,7 +59829,7 @@
         <v>46251</v>
       </c>
       <c r="F28" s="189">
-        <f>[1]!PlanoAcaoCoordTable4[[#This Row],[Data da atualização]]</f>
+        <f>[2]!PlanoAcaoCoordTable4[[#This Row],[Data da atualização]]</f>
         <v>46251</v>
       </c>
       <c r="G28" s="188" t="s">
@@ -59829,7 +59837,7 @@
       </c>
       <c r="H28" s="188"/>
     </row>
-    <row r="29" spans="1:8" ht="52.7" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>393</v>
       </c>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-15T14:04:04.140-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="308" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39355A31-D4C9-46EC-8695-F6F3301DB543}"/>
+  <xr:revisionPtr revIDLastSave="315" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497CD170-9539-4296-A718-7705D99A8C67}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -3858,9 +3858,6 @@
           <cell r="D2">
             <v>106810.56</v>
           </cell>
-          <cell r="G2">
-            <v>156366.41999999998</v>
-          </cell>
         </row>
       </sheetData>
       <sheetData sheetId="6"/>
@@ -5032,10 +5029,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AM37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="24" width="9.140625" style="7"/>
+    <col min="1" max="1" width="27.42578125" style="7" customWidth="1"/>
+    <col min="2" max="10" width="0" style="7" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="9.140625" style="7" collapsed="1"/>
+    <col min="12" max="24" width="9.140625" style="7"/>
     <col min="25" max="39" width="9.140625" style="83"/>
   </cols>
   <sheetData>
@@ -6246,7 +6245,7 @@
       <c r="J22" s="87">
         <v>239</v>
       </c>
-      <c r="K22" s="87">
+      <c r="K22" s="86">
         <v>241</v>
       </c>
       <c r="L22" s="62"/>
@@ -6710,7 +6709,7 @@
       <c r="J32" s="87">
         <v>46</v>
       </c>
-      <c r="K32" s="87">
+      <c r="K32" s="86">
         <v>46</v>
       </c>
       <c r="L32" s="62"/>
@@ -58758,8 +58757,7 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <f>SUM([1]LASTRO!D2,[1]LASTRO!G2)/1.39</f>
-        <v>189335.95683453238</v>
+        <v>306532</v>
       </c>
       <c r="N15" s="72">
         <v>282288.96999999997</v>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-16T10:56:59.051-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="315" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{497CD170-9539-4296-A718-7705D99A8C67}"/>
+  <xr:revisionPtr revIDLastSave="338" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDF44F8E-26C4-4541-A32C-57C28E0AC2D0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4711,10 +4711,10 @@
         <v>31</v>
       </c>
       <c r="C36" s="81">
-        <v>110100</v>
+        <v>104520</v>
       </c>
       <c r="D36" s="81">
-        <v>110680</v>
+        <v>104980</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4722,25 +4722,33 @@
         <v>32</v>
       </c>
       <c r="C37" s="81">
-        <v>113700</v>
+        <v>105020</v>
       </c>
       <c r="D37" s="81">
-        <v>114720</v>
+        <v>105160</v>
       </c>
     </row>
     <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="192" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="81"/>
-      <c r="D38" s="81"/>
+      <c r="C38" s="81">
+        <v>110100</v>
+      </c>
+      <c r="D38" s="81">
+        <v>110680</v>
+      </c>
     </row>
     <row r="39" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="192" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="81"/>
-      <c r="D39" s="81"/>
+      <c r="C39" s="81">
+        <v>113700</v>
+      </c>
+      <c r="D39" s="81">
+        <v>114720</v>
+      </c>
     </row>
     <row r="40" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="192" t="s">
@@ -58184,11 +58192,12 @@
         <v>37087.89</v>
       </c>
       <c r="M2" s="72">
-        <v>13557.49</v>
+        <v>20095.73</v>
       </c>
       <c r="N2" s="72">
-        <v>6204.96</v>
-      </c>
+        <v>7778.88</v>
+      </c>
+      <c r="P2" s="29"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="166" t="s">
@@ -58228,13 +58237,13 @@
         <v>509033</v>
       </c>
       <c r="M3" s="72">
-        <v>228789</v>
+        <v>285583</v>
       </c>
       <c r="N3" s="72">
-        <v>156686</v>
+        <v>162068</v>
       </c>
       <c r="O3" s="4"/>
-      <c r="P3" s="168"/>
+      <c r="P3" s="29"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="166" t="s">
@@ -58278,8 +58287,9 @@
       </c>
       <c r="N4" s="72">
         <f>M3*4</f>
-        <v>915156</v>
-      </c>
+        <v>1142332</v>
+      </c>
+      <c r="P4" s="29"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="166" t="s">
@@ -58319,11 +58329,12 @@
         <v>1018066</v>
       </c>
       <c r="M5" s="72">
-        <v>309535</v>
+        <v>397675</v>
       </c>
       <c r="N5" s="72">
         <v>319386</v>
       </c>
+      <c r="P5" s="29"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="166" t="s">
@@ -58363,11 +58374,12 @@
         <v>2036132</v>
       </c>
       <c r="M6" s="72">
-        <v>622250</v>
+        <v>795977</v>
       </c>
       <c r="N6" s="72">
         <v>642561</v>
       </c>
+      <c r="P6" s="29"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="166" t="s">
@@ -58412,6 +58424,7 @@
       <c r="N7" s="72">
         <v>557904</v>
       </c>
+      <c r="P7" s="29"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="166" t="s">
@@ -58454,6 +58467,7 @@
       <c r="N8" s="72">
         <v>962</v>
       </c>
+      <c r="P8" s="29"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="166" t="s">
@@ -58498,6 +58512,7 @@
       <c r="N9" s="72">
         <v>3432</v>
       </c>
+      <c r="P9" s="29"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="166" t="s">
@@ -58542,6 +58557,7 @@
       <c r="N10" s="72">
         <v>7</v>
       </c>
+      <c r="P10" s="29"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="166" t="s">
@@ -58586,6 +58602,7 @@
       <c r="N11" s="72">
         <v>0</v>
       </c>
+      <c r="P11" s="29"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="166" t="s">
@@ -58630,6 +58647,7 @@
       <c r="N12" s="72">
         <v>6</v>
       </c>
+      <c r="P12" s="29"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="166" t="s">
@@ -58674,6 +58692,7 @@
       <c r="N13" s="72">
         <v>0</v>
       </c>
+      <c r="P13" s="29"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="166" t="s">
@@ -58716,8 +58735,9 @@
         <v>1592</v>
       </c>
       <c r="N14" s="72">
-        <v>447</v>
-      </c>
+        <v>459</v>
+      </c>
+      <c r="P14" s="29"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="166" t="s">
@@ -58757,12 +58777,12 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <v>306532</v>
+        <v>314543.35700000002</v>
       </c>
       <c r="N15" s="72">
-        <v>282288.96999999997</v>
-      </c>
-      <c r="P15" s="168"/>
+        <v>293604.81</v>
+      </c>
+      <c r="P15" s="29"/>
     </row>
     <row r="17" spans="14:14" x14ac:dyDescent="0.25">
       <c r="N17" s="168"/>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-22T10:26:19.649-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="338" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDF44F8E-26C4-4541-A32C-57C28E0AC2D0}"/>
+  <xr:revisionPtr revIDLastSave="441" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FC64A70-3345-4C47-94D2-65CC3B4648C3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -4206,7 +4206,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="80">
-        <v>46277</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="12" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4283,8 +4283,12 @@
       <c r="J14" s="79">
         <v>99500</v>
       </c>
-      <c r="K14" s="78"/>
-      <c r="L14" s="79"/>
+      <c r="K14" s="78">
+        <v>100086</v>
+      </c>
+      <c r="L14" s="79">
+        <v>100292</v>
+      </c>
       <c r="M14" s="78"/>
       <c r="N14" s="79"/>
     </row>
@@ -4296,7 +4300,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="79">
-        <v>96610</v>
+        <v>102500</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79"/>
@@ -4317,7 +4321,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="79">
-        <v>82860</v>
+        <v>85240</v>
       </c>
       <c r="E16" s="78"/>
       <c r="F16" s="79"/>
@@ -4338,7 +4342,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="79">
-        <v>82860</v>
+        <v>85220</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79"/>
@@ -4367,8 +4371,12 @@
       <c r="F18" s="79">
         <v>78560</v>
       </c>
-      <c r="G18" s="78"/>
-      <c r="H18" s="79"/>
+      <c r="G18" s="78">
+        <v>83420</v>
+      </c>
+      <c r="H18" s="79">
+        <v>85220</v>
+      </c>
       <c r="I18" s="78">
         <v>65400</v>
       </c>
@@ -4419,7 +4427,7 @@
         <v>23000</v>
       </c>
       <c r="F20" s="79">
-        <v>47100</v>
+        <v>51460</v>
       </c>
       <c r="G20" s="78">
         <v>60160</v>
@@ -4525,13 +4533,13 @@
         <v>40100</v>
       </c>
       <c r="L23" s="79">
-        <v>40500</v>
+        <v>41500</v>
       </c>
       <c r="M23" s="78">
         <v>41500</v>
       </c>
       <c r="N23" s="79">
-        <v>43400</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="24" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4631,7 +4639,7 @@
         <v>11607</v>
       </c>
       <c r="F27" s="79">
-        <v>26668</v>
+        <v>31464</v>
       </c>
       <c r="G27" s="78"/>
       <c r="H27" s="79"/>
@@ -4679,8 +4687,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="81">
-        <f>D14</f>
-        <v>96640</v>
+        <v>103820</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4688,11 +4695,10 @@
         <v>29</v>
       </c>
       <c r="C34" s="81">
-        <v>97140</v>
+        <v>104000</v>
       </c>
       <c r="D34" s="81">
-        <f>F14</f>
-        <v>98340</v>
+        <v>104980</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4700,10 +4706,10 @@
         <v>30</v>
       </c>
       <c r="C35" s="81">
-        <v>101220</v>
+        <v>105020</v>
       </c>
       <c r="D35" s="81">
-        <v>104500</v>
+        <v>105160</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4711,10 +4717,10 @@
         <v>31</v>
       </c>
       <c r="C36" s="81">
-        <v>104520</v>
+        <v>107440</v>
       </c>
       <c r="D36" s="81">
-        <v>104980</v>
+        <v>108500</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4722,10 +4728,10 @@
         <v>32</v>
       </c>
       <c r="C37" s="81">
-        <v>105020</v>
+        <v>110100</v>
       </c>
       <c r="D37" s="81">
-        <v>105160</v>
+        <v>110700</v>
       </c>
     </row>
     <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4733,22 +4739,18 @@
         <v>33</v>
       </c>
       <c r="C38" s="81">
-        <v>110100</v>
+        <v>112720</v>
       </c>
       <c r="D38" s="81">
-        <v>110680</v>
+        <v>114720</v>
       </c>
     </row>
     <row r="39" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="192" t="s">
         <v>34</v>
       </c>
-      <c r="C39" s="81">
-        <v>113700</v>
-      </c>
-      <c r="D39" s="81">
-        <v>114720</v>
-      </c>
+      <c r="C39" s="81"/>
+      <c r="D39" s="81"/>
     </row>
     <row r="40" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="192" t="s">
@@ -6256,7 +6258,9 @@
       <c r="K22" s="86">
         <v>241</v>
       </c>
-      <c r="L22" s="62"/>
+      <c r="L22" s="86">
+        <v>237</v>
+      </c>
       <c r="M22" s="62"/>
       <c r="N22" s="62"/>
       <c r="O22" s="62"/>
@@ -6488,7 +6492,9 @@
       <c r="K27" s="87">
         <v>113</v>
       </c>
-      <c r="L27" s="62"/>
+      <c r="L27" s="86">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="M27" s="62"/>
       <c r="N27" s="62"/>
       <c r="O27" s="62"/>
@@ -6720,7 +6726,9 @@
       <c r="K32" s="86">
         <v>46</v>
       </c>
-      <c r="L32" s="62"/>
+      <c r="L32" s="86">
+        <v>46</v>
+      </c>
       <c r="M32" s="62"/>
       <c r="N32" s="62"/>
       <c r="O32" s="62"/>
@@ -6952,7 +6960,9 @@
       <c r="K37" s="87">
         <v>48</v>
       </c>
-      <c r="L37" s="62"/>
+      <c r="L37" s="87">
+        <v>48</v>
+      </c>
       <c r="M37" s="62"/>
       <c r="N37" s="62"/>
       <c r="O37" s="62"/>
@@ -7583,7 +7593,7 @@
         <v>96</v>
       </c>
       <c r="U4" s="103">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="V4" s="102">
         <v>96</v>
@@ -8399,7 +8409,7 @@
         <v>5</v>
       </c>
       <c r="U9" s="13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="V9" s="12">
         <v>5</v>
@@ -9703,7 +9713,7 @@
         <v>23</v>
       </c>
       <c r="U17" s="13">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="V17" s="12">
         <v>23</v>
@@ -12339,7 +12349,7 @@
       </c>
       <c r="U33" s="113">
         <f t="shared" si="8"/>
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="V33" s="113">
         <f t="shared" si="8"/>
@@ -14119,7 +14129,7 @@
         <v>16</v>
       </c>
       <c r="U44" s="103">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="V44" s="102">
         <v>16</v>
@@ -14443,7 +14453,7 @@
         <v>6</v>
       </c>
       <c r="U46" s="103">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V46" s="102">
         <v>6</v>
@@ -17715,7 +17725,7 @@
         <v>8</v>
       </c>
       <c r="U66" s="103">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V66" s="102">
         <v>8</v>
@@ -19183,7 +19193,7 @@
         <v>3</v>
       </c>
       <c r="U75" s="13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V75" s="12">
         <v>3</v>
@@ -19855,7 +19865,7 @@
       </c>
       <c r="U79" s="112">
         <f t="shared" si="18"/>
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="V79" s="112">
         <f t="shared" si="18"/>
@@ -27176,7 +27186,7 @@
         <v>1105</v>
       </c>
       <c r="I5" s="68">
-        <v>570</v>
+        <v>880</v>
       </c>
       <c r="J5" s="68"/>
       <c r="K5" s="68"/>
@@ -27233,7 +27243,7 @@
         <v>21</v>
       </c>
       <c r="I6" s="69">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J6" s="69"/>
       <c r="K6" s="69"/>
@@ -27283,7 +27293,7 @@
       </c>
       <c r="I7" s="69">
         <f t="shared" si="2"/>
-        <v>51.81818181818182</v>
+        <v>51.764705882352942</v>
       </c>
       <c r="J7" s="69"/>
       <c r="K7" s="69"/>
@@ -27347,37 +27357,37 @@
         <v>1051</v>
       </c>
       <c r="I8" s="147">
-        <v>1415.1000000000004</v>
+        <v>1402.1999999999998</v>
       </c>
       <c r="J8" s="147">
-        <v>1365.1999999999998</v>
+        <v>1370.6999999999998</v>
       </c>
       <c r="K8" s="147">
-        <v>1235.1999999999998</v>
+        <v>1240.1000000000004</v>
       </c>
       <c r="L8" s="147">
-        <v>910.10000000000036</v>
+        <v>913.79999999999927</v>
       </c>
       <c r="M8" s="147">
-        <v>1235.2000000000007</v>
+        <v>1240.1000000000004</v>
       </c>
       <c r="N8" s="147">
-        <v>1300.2000000000007</v>
+        <v>1305.3999999999996</v>
       </c>
       <c r="O8" s="147">
-        <v>1495.2000000000007</v>
+        <v>1501.2000000000007</v>
       </c>
       <c r="P8" s="147">
-        <v>1430.2000000000007</v>
+        <v>1435.8999999999996</v>
       </c>
       <c r="Q8" s="147">
-        <v>1365.2000000000007</v>
+        <v>1370.7000000000007</v>
       </c>
       <c r="R8" s="147">
-        <v>1430.1999999999989</v>
+        <v>1435.8999999999996</v>
       </c>
       <c r="S8" s="147">
-        <v>1100.5999999999985</v>
+        <v>1066.0999999999985</v>
       </c>
       <c r="T8" s="147">
         <v>0</v>
@@ -27520,47 +27530,47 @@
       </c>
       <c r="I10" s="69">
         <f t="shared" si="5"/>
-        <v>56.604000000000013</v>
+        <v>56.087999999999994</v>
       </c>
       <c r="J10" s="69">
         <f t="shared" si="5"/>
-        <v>50.562962962962956</v>
+        <v>50.766666666666659</v>
       </c>
       <c r="K10" s="69">
         <f t="shared" si="5"/>
-        <v>49.407999999999994</v>
+        <v>49.604000000000013</v>
       </c>
       <c r="L10" s="69">
         <f t="shared" si="5"/>
-        <v>56.881250000000023</v>
+        <v>57.112499999999955</v>
       </c>
       <c r="M10" s="69">
         <f t="shared" si="5"/>
-        <v>51.466666666666697</v>
+        <v>51.670833333333348</v>
       </c>
       <c r="N10" s="69">
         <f t="shared" si="5"/>
-        <v>54.175000000000033</v>
+        <v>54.391666666666652</v>
       </c>
       <c r="O10" s="69">
         <f t="shared" si="5"/>
-        <v>55.377777777777801</v>
+        <v>55.60000000000003</v>
       </c>
       <c r="P10" s="69">
         <f t="shared" si="5"/>
-        <v>55.007692307692338</v>
+        <v>55.226923076923065</v>
       </c>
       <c r="Q10" s="69">
         <f t="shared" si="5"/>
-        <v>52.507692307692338</v>
+        <v>52.719230769230798</v>
       </c>
       <c r="R10" s="69">
         <f t="shared" si="5"/>
-        <v>55.007692307692267</v>
+        <v>55.226923076923065</v>
       </c>
       <c r="S10" s="69">
         <f t="shared" si="5"/>
-        <v>40.762962962962909</v>
+        <v>39.485185185185131</v>
       </c>
       <c r="T10" s="69">
         <f t="shared" si="5"/>
@@ -27941,7 +27951,7 @@
         <v>20537</v>
       </c>
       <c r="I16" s="153">
-        <v>4925</v>
+        <v>9855</v>
       </c>
       <c r="J16" s="153"/>
       <c r="K16" s="153"/>
@@ -27984,7 +27994,7 @@
         <v>16</v>
       </c>
       <c r="I17" s="69">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="J17" s="69"/>
       <c r="K17" s="69"/>
@@ -28034,7 +28044,7 @@
       </c>
       <c r="I18" s="69">
         <f t="shared" si="7"/>
-        <v>615.625</v>
+        <v>758.07692307692309</v>
       </c>
       <c r="J18" s="69"/>
       <c r="K18" s="69"/>
@@ -28082,31 +28092,31 @@
         <v>16832</v>
       </c>
       <c r="I19" s="147">
-        <v>22925.699999999997</v>
+        <v>19957.899999999994</v>
       </c>
       <c r="J19" s="147">
-        <v>19802.599999999991</v>
+        <v>19826</v>
       </c>
       <c r="K19" s="147">
-        <v>16248.100000000006</v>
+        <v>16325.200000000012</v>
       </c>
       <c r="L19" s="147">
-        <v>12826</v>
+        <v>12810.299999999988</v>
       </c>
       <c r="M19" s="147">
-        <v>17763.700000000012</v>
+        <v>17729.700000000012</v>
       </c>
       <c r="N19" s="147">
         <v>18617.200000000012</v>
       </c>
       <c r="O19" s="147">
-        <v>21413.200000000012</v>
+        <v>21409.799999999988</v>
       </c>
       <c r="P19" s="147">
-        <v>20527.899999999994</v>
+        <v>20513.899999999994</v>
       </c>
       <c r="Q19" s="147">
-        <v>19826.700000000012</v>
+        <v>19843.299999999988</v>
       </c>
       <c r="R19" s="147">
         <v>20484.799999999988</v>
@@ -28115,7 +28125,7 @@
         <v>20484.799999999988</v>
       </c>
       <c r="T19" s="147">
-        <v>8318.7999999999302</v>
+        <v>11236.599999999977</v>
       </c>
       <c r="U19" s="147">
         <v>0</v>
@@ -28234,23 +28244,23 @@
       </c>
       <c r="I21" s="69">
         <f t="shared" si="10"/>
-        <v>917.02799999999991</v>
+        <v>798.3159999999998</v>
       </c>
       <c r="J21" s="69">
         <f t="shared" si="10"/>
-        <v>733.42962962962929</v>
+        <v>734.2962962962963</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="10"/>
-        <v>649.92400000000021</v>
+        <v>653.00800000000049</v>
       </c>
       <c r="L21" s="69">
         <f t="shared" si="10"/>
-        <v>801.625</v>
+        <v>800.64374999999927</v>
       </c>
       <c r="M21" s="69">
         <f t="shared" si="10"/>
-        <v>740.15416666666715</v>
+        <v>738.73750000000052</v>
       </c>
       <c r="N21" s="69">
         <f t="shared" si="10"/>
@@ -28258,15 +28268,15 @@
       </c>
       <c r="O21" s="69">
         <f t="shared" si="10"/>
-        <v>793.08148148148189</v>
+        <v>792.95555555555518</v>
       </c>
       <c r="P21" s="69">
         <f t="shared" si="10"/>
-        <v>789.53461538461511</v>
+        <v>788.99615384615367</v>
       </c>
       <c r="Q21" s="69">
         <f t="shared" si="10"/>
-        <v>762.56538461538503</v>
+        <v>763.20384615384569</v>
       </c>
       <c r="R21" s="69">
         <f t="shared" si="10"/>
@@ -28278,7 +28288,7 @@
       </c>
       <c r="T21" s="69">
         <f t="shared" si="10"/>
-        <v>319.95384615384347</v>
+        <v>432.17692307692221</v>
       </c>
       <c r="U21" s="69">
         <f t="shared" si="10"/>
@@ -28609,7 +28619,7 @@
         <v>41202</v>
       </c>
       <c r="I27" s="68">
-        <v>13227</v>
+        <v>25071</v>
       </c>
       <c r="J27" s="68" t="s">
         <v>196</v>
@@ -28678,7 +28688,7 @@
         <v>13</v>
       </c>
       <c r="I28" s="69">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="J28" s="69"/>
       <c r="K28" s="69"/>
@@ -28728,7 +28738,7 @@
       </c>
       <c r="I29" s="69">
         <f t="shared" si="12"/>
-        <v>1889.5714285714287</v>
+        <v>2279.181818181818</v>
       </c>
       <c r="J29" s="69"/>
       <c r="K29" s="69"/>
@@ -28776,40 +28786,40 @@
         <v>41202</v>
       </c>
       <c r="I30" s="147">
-        <v>47573.600000000006</v>
+        <v>51643.799999999988</v>
       </c>
       <c r="J30" s="147">
-        <v>49997.800000000017</v>
+        <v>85090.700000000012</v>
       </c>
       <c r="K30" s="147">
-        <v>45378.099999999977</v>
+        <v>40690.900000000023</v>
       </c>
       <c r="L30" s="147">
-        <v>40451.099999999977</v>
+        <v>21151</v>
       </c>
       <c r="M30" s="147">
-        <v>56267.099999999977</v>
+        <v>34574</v>
       </c>
       <c r="N30" s="147">
-        <v>39979.799999999988</v>
+        <v>37784.700000000012</v>
       </c>
       <c r="O30" s="147">
-        <v>45290.099999999977</v>
+        <v>50217.700000000012</v>
       </c>
       <c r="P30" s="147">
-        <v>51371.599999999977</v>
+        <v>45950.599999999977</v>
       </c>
       <c r="Q30" s="147">
-        <v>54032.100000000035</v>
+        <v>51976.699999999953</v>
       </c>
       <c r="R30" s="147">
-        <v>34898.699999999953</v>
+        <v>45354</v>
       </c>
       <c r="S30" s="147">
-        <v>43009.599999999977</v>
+        <v>38685.5</v>
       </c>
       <c r="T30" s="147">
-        <v>50567</v>
+        <v>50592.099999999977</v>
       </c>
       <c r="U30" s="147">
         <v>0</v>
@@ -28928,51 +28938,51 @@
       </c>
       <c r="I32" s="69">
         <f t="shared" si="15"/>
-        <v>1902.9440000000002</v>
+        <v>2065.7519999999995</v>
       </c>
       <c r="J32" s="69">
         <f t="shared" si="15"/>
-        <v>1851.770370370371</v>
+        <v>3151.5074074074078</v>
       </c>
       <c r="K32" s="69">
         <f t="shared" si="15"/>
-        <v>1815.1239999999991</v>
+        <v>1627.6360000000009</v>
       </c>
       <c r="L32" s="69">
         <f t="shared" si="15"/>
-        <v>2528.1937499999985</v>
+        <v>1321.9375</v>
       </c>
       <c r="M32" s="69">
         <f t="shared" si="15"/>
-        <v>2344.4624999999992</v>
+        <v>1440.5833333333333</v>
       </c>
       <c r="N32" s="69">
         <f t="shared" si="15"/>
-        <v>1665.8249999999996</v>
+        <v>1574.3625000000004</v>
       </c>
       <c r="O32" s="69">
         <f t="shared" si="15"/>
-        <v>1677.4111111111104</v>
+        <v>1859.9148148148151</v>
       </c>
       <c r="P32" s="69">
         <f t="shared" si="15"/>
-        <v>1975.8307692307683</v>
+        <v>1767.3307692307683</v>
       </c>
       <c r="Q32" s="69">
         <f t="shared" si="15"/>
-        <v>2078.1576923076937</v>
+        <v>1999.1038461538444</v>
       </c>
       <c r="R32" s="69">
         <f t="shared" si="15"/>
-        <v>1342.2576923076906</v>
+        <v>1744.3846153846155</v>
       </c>
       <c r="S32" s="69">
         <f t="shared" si="15"/>
-        <v>1592.9481481481473</v>
+        <v>1432.7962962962963</v>
       </c>
       <c r="T32" s="69">
         <f t="shared" si="15"/>
-        <v>1944.8846153846155</v>
+        <v>1945.849999999999</v>
       </c>
       <c r="U32" s="69">
         <f t="shared" si="15"/>
@@ -29303,7 +29313,7 @@
         <v>57</v>
       </c>
       <c r="I38" s="68">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="J38" s="68" t="s">
         <v>196</v>
@@ -29372,7 +29382,7 @@
         <v>17</v>
       </c>
       <c r="I39" s="69">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J39" s="69"/>
       <c r="K39" s="69"/>
@@ -29422,7 +29432,7 @@
       </c>
       <c r="I40" s="69">
         <f t="shared" si="17"/>
-        <v>3.4</v>
+        <v>3.625</v>
       </c>
       <c r="J40" s="69"/>
       <c r="K40" s="69"/>
@@ -29470,46 +29480,46 @@
         <v>57</v>
       </c>
       <c r="I41" s="147">
-        <v>197.79999999999995</v>
+        <v>152.10000000000002</v>
       </c>
       <c r="J41" s="147">
-        <v>221.20000000000005</v>
+        <v>238.19999999999993</v>
       </c>
       <c r="K41" s="147">
-        <v>186.20000000000005</v>
+        <v>197.29999999999995</v>
       </c>
       <c r="L41" s="147">
-        <v>152.40000000000009</v>
+        <v>153.5</v>
       </c>
       <c r="M41" s="147">
-        <v>194.20000000000005</v>
+        <v>186.79999999999995</v>
       </c>
       <c r="N41" s="147">
-        <v>160.70000000000005</v>
+        <v>166.5</v>
       </c>
       <c r="O41" s="147">
-        <v>220.20000000000005</v>
+        <v>217.5</v>
       </c>
       <c r="P41" s="147">
-        <v>261.20000000000005</v>
+        <v>262</v>
       </c>
       <c r="Q41" s="147">
-        <v>268.79999999999995</v>
+        <v>271.39999999999986</v>
       </c>
       <c r="R41" s="147">
-        <v>277.5</v>
+        <v>272.80000000000018</v>
       </c>
       <c r="S41" s="147">
-        <v>334</v>
+        <v>254</v>
       </c>
       <c r="T41" s="147">
-        <v>303</v>
+        <v>235</v>
       </c>
       <c r="U41" s="147">
-        <v>91.400000000000091</v>
+        <v>205</v>
       </c>
       <c r="V41" s="147">
-        <v>5.3000000000001819</v>
+        <v>62</v>
       </c>
       <c r="X41" s="148"/>
     </row>
@@ -29622,55 +29632,55 @@
       </c>
       <c r="I43" s="69">
         <f t="shared" si="20"/>
-        <v>7.9119999999999981</v>
+        <v>6.0840000000000005</v>
       </c>
       <c r="J43" s="69">
         <f t="shared" si="20"/>
-        <v>8.1925925925925949</v>
+        <v>8.8222222222222193</v>
       </c>
       <c r="K43" s="69">
         <f t="shared" si="20"/>
-        <v>7.4480000000000022</v>
+        <v>7.8919999999999986</v>
       </c>
       <c r="L43" s="69">
         <f t="shared" si="20"/>
-        <v>9.5250000000000057</v>
+        <v>9.59375</v>
       </c>
       <c r="M43" s="69">
         <f t="shared" si="20"/>
-        <v>8.0916666666666686</v>
+        <v>7.7833333333333314</v>
       </c>
       <c r="N43" s="69">
         <f t="shared" si="20"/>
-        <v>6.6958333333333355</v>
+        <v>6.9375</v>
       </c>
       <c r="O43" s="69">
         <f t="shared" si="20"/>
-        <v>8.1555555555555568</v>
+        <v>8.0555555555555554</v>
       </c>
       <c r="P43" s="69">
         <f t="shared" si="20"/>
-        <v>10.046153846153848</v>
+        <v>10.076923076923077</v>
       </c>
       <c r="Q43" s="69">
         <f t="shared" si="20"/>
-        <v>10.338461538461537</v>
+        <v>10.438461538461533</v>
       </c>
       <c r="R43" s="69">
         <f t="shared" si="20"/>
-        <v>10.673076923076923</v>
+        <v>10.492307692307699</v>
       </c>
       <c r="S43" s="69">
         <f t="shared" si="20"/>
-        <v>12.37037037037037</v>
+        <v>9.4074074074074066</v>
       </c>
       <c r="T43" s="69">
         <f t="shared" si="20"/>
-        <v>11.653846153846153</v>
+        <v>9.0384615384615383</v>
       </c>
       <c r="U43" s="69">
         <f t="shared" si="20"/>
-        <v>3.5153846153846189</v>
+        <v>7.884615384615385</v>
       </c>
       <c r="V43" s="69">
         <v>0</v>
@@ -29997,7 +30007,7 @@
         <v>14588</v>
       </c>
       <c r="I49" s="68">
-        <v>6223.5999999999985</v>
+        <v>10264</v>
       </c>
       <c r="J49" s="68" t="s">
         <v>196</v>
@@ -30066,7 +30076,7 @@
         <v>21</v>
       </c>
       <c r="I50" s="69">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J50" s="69"/>
       <c r="K50" s="69"/>
@@ -30116,7 +30126,7 @@
       </c>
       <c r="I51" s="69">
         <f t="shared" si="22"/>
-        <v>1244.7199999999998</v>
+        <v>933.09090909090912</v>
       </c>
       <c r="J51" s="69"/>
       <c r="K51" s="69"/>
@@ -30164,43 +30174,43 @@
         <v>13688</v>
       </c>
       <c r="I52" s="147">
-        <v>15114.899999999994</v>
+        <v>18847.900000000001</v>
       </c>
       <c r="J52" s="147">
-        <v>26442</v>
+        <v>23951.700000000004</v>
       </c>
       <c r="K52" s="147">
-        <v>17275.800000000003</v>
+        <v>24122.800000000003</v>
       </c>
       <c r="L52" s="147">
-        <v>19112.099999999991</v>
+        <v>21545.400000000009</v>
       </c>
       <c r="M52" s="147">
-        <v>24128.100000000006</v>
+        <v>12896.200000000012</v>
       </c>
       <c r="N52" s="147">
-        <v>13797.700000000012</v>
+        <v>13308.299999999988</v>
       </c>
       <c r="O52" s="147">
-        <v>18083.700000000012</v>
+        <v>18192</v>
       </c>
       <c r="P52" s="147">
-        <v>22314.5</v>
+        <v>20671.799999999988</v>
       </c>
       <c r="Q52" s="147">
-        <v>22318.5</v>
+        <v>20778.100000000006</v>
       </c>
       <c r="R52" s="147">
-        <v>22525.299999999988</v>
+        <v>25066.299999999988</v>
       </c>
       <c r="S52" s="147">
-        <v>9452</v>
+        <v>19499</v>
       </c>
       <c r="T52" s="147">
-        <v>22008.399999999994</v>
+        <v>19063.299999999988</v>
       </c>
       <c r="U52" s="147">
-        <v>27246.600000000035</v>
+        <v>21876.799999999988</v>
       </c>
       <c r="V52" s="147">
         <v>0</v>
@@ -30316,55 +30326,55 @@
       </c>
       <c r="I54" s="69">
         <f t="shared" si="25"/>
-        <v>604.59599999999978</v>
+        <v>753.91600000000005</v>
       </c>
       <c r="J54" s="69">
         <f t="shared" si="25"/>
-        <v>979.33333333333337</v>
+        <v>887.10000000000014</v>
       </c>
       <c r="K54" s="69">
         <f t="shared" si="25"/>
-        <v>691.03200000000015</v>
+        <v>964.91200000000015</v>
       </c>
       <c r="L54" s="69">
         <f t="shared" si="25"/>
-        <v>1194.5062499999995</v>
+        <v>1346.5875000000005</v>
       </c>
       <c r="M54" s="69">
         <f t="shared" si="25"/>
-        <v>1005.3375000000002</v>
+        <v>537.34166666666715</v>
       </c>
       <c r="N54" s="69">
         <f t="shared" si="25"/>
-        <v>574.90416666666715</v>
+        <v>554.51249999999948</v>
       </c>
       <c r="O54" s="69">
         <f t="shared" si="25"/>
-        <v>669.76666666666711</v>
+        <v>673.77777777777783</v>
       </c>
       <c r="P54" s="69">
         <f t="shared" si="25"/>
-        <v>858.25</v>
+        <v>795.06923076923033</v>
       </c>
       <c r="Q54" s="69">
         <f t="shared" si="25"/>
-        <v>858.40384615384619</v>
+        <v>799.15769230769251</v>
       </c>
       <c r="R54" s="69">
         <f t="shared" si="25"/>
-        <v>866.35769230769188</v>
+        <v>964.08846153846105</v>
       </c>
       <c r="S54" s="69">
         <f t="shared" si="25"/>
-        <v>350.07407407407408</v>
+        <v>722.18518518518522</v>
       </c>
       <c r="T54" s="69">
         <f t="shared" si="25"/>
-        <v>846.47692307692284</v>
+        <v>733.20384615384569</v>
       </c>
       <c r="U54" s="69">
         <f t="shared" si="25"/>
-        <v>1047.9461538461551</v>
+        <v>841.41538461538414</v>
       </c>
       <c r="V54" s="69">
         <f t="shared" si="25"/>
@@ -30692,7 +30702,7 @@
         <v>22612</v>
       </c>
       <c r="I60" s="68">
-        <v>12159</v>
+        <v>21742</v>
       </c>
       <c r="J60" s="68" t="s">
         <v>196</v>
@@ -30761,7 +30771,7 @@
         <v>11</v>
       </c>
       <c r="I61" s="69">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="J61" s="69"/>
       <c r="K61" s="69"/>
@@ -30810,7 +30820,7 @@
       </c>
       <c r="I62" s="69">
         <f>I60/I61</f>
-        <v>2026.5</v>
+        <v>1976.5454545454545</v>
       </c>
       <c r="J62" s="69"/>
       <c r="K62" s="69"/>
@@ -30857,43 +30867,43 @@
         <v>20245</v>
       </c>
       <c r="I63" s="147">
-        <v>47080.2</v>
+        <v>44708.800000000003</v>
       </c>
       <c r="J63" s="147">
-        <v>46453.8</v>
+        <v>48824.900000000009</v>
       </c>
       <c r="K63" s="147">
         <v>49636.299999999988</v>
       </c>
       <c r="L63" s="147">
-        <v>38737.899999999994</v>
+        <v>39908.899999999994</v>
       </c>
       <c r="M63" s="147">
-        <v>35118.5</v>
+        <v>31812.200000000012</v>
       </c>
       <c r="N63" s="147">
-        <v>28270.999999999971</v>
+        <v>28190.300000000017</v>
       </c>
       <c r="O63" s="147">
-        <v>42923.299999999988</v>
+        <v>42949.299999999988</v>
       </c>
       <c r="P63" s="147">
-        <v>47202.099999999977</v>
+        <v>47310.700000000012</v>
       </c>
       <c r="Q63" s="147">
-        <v>48798.400000000023</v>
+        <v>49762.200000000012</v>
       </c>
       <c r="R63" s="147">
-        <v>49509.700000000012</v>
+        <v>50451</v>
       </c>
       <c r="S63" s="147">
-        <v>52988.799999999988</v>
+        <v>53003.400000000023</v>
       </c>
       <c r="T63" s="147">
-        <v>46277.700000000012</v>
+        <v>56170.799999999988</v>
       </c>
       <c r="U63" s="147">
-        <v>33802.599999999977</v>
+        <v>56190</v>
       </c>
       <c r="V63" s="147">
         <v>0</v>
@@ -31009,11 +31019,11 @@
       </c>
       <c r="I65" s="69">
         <f t="shared" si="29"/>
-        <v>1883.2079999999999</v>
+        <v>1788.3520000000001</v>
       </c>
       <c r="J65" s="69">
         <f t="shared" si="29"/>
-        <v>1720.5111111111112</v>
+        <v>1808.3296296296301</v>
       </c>
       <c r="K65" s="69">
         <f t="shared" si="29"/>
@@ -31021,43 +31031,43 @@
       </c>
       <c r="L65" s="69">
         <f t="shared" si="29"/>
-        <v>2421.1187499999996</v>
+        <v>2494.3062499999996</v>
       </c>
       <c r="M65" s="69">
         <f t="shared" si="29"/>
-        <v>1463.2708333333333</v>
+        <v>1325.5083333333339</v>
       </c>
       <c r="N65" s="69">
         <f t="shared" si="29"/>
-        <v>1177.9583333333321</v>
+        <v>1174.595833333334</v>
       </c>
       <c r="O65" s="69">
         <f t="shared" si="29"/>
-        <v>1589.7518518518514</v>
+        <v>1590.7148148148144</v>
       </c>
       <c r="P65" s="69">
         <f t="shared" si="29"/>
-        <v>1815.4653846153838</v>
+        <v>1819.6423076923081</v>
       </c>
       <c r="Q65" s="69">
         <f t="shared" si="29"/>
-        <v>1876.8615384615393</v>
+        <v>1913.9307692307698</v>
       </c>
       <c r="R65" s="69">
         <f t="shared" si="29"/>
-        <v>1904.2192307692312</v>
+        <v>1940.4230769230769</v>
       </c>
       <c r="S65" s="69">
         <f t="shared" si="29"/>
-        <v>1962.5481481481477</v>
+        <v>1963.0888888888896</v>
       </c>
       <c r="T65" s="69">
         <f t="shared" si="29"/>
-        <v>1779.9115384615388</v>
+        <v>2160.415384615384</v>
       </c>
       <c r="U65" s="69">
         <f t="shared" si="29"/>
-        <v>1300.099999999999</v>
+        <v>2161.1538461538462</v>
       </c>
       <c r="V65" s="69">
         <v>0</v>
@@ -31125,47 +31135,47 @@
       <c r="B2" s="46"/>
       <c r="C2" s="34">
         <f>SUM(C4:C733)</f>
-        <v>120801.14000000004</v>
+        <v>126598.56000000003</v>
       </c>
       <c r="D2" s="35">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>123001.82000000002</v>
+        <v>127301.54000000002</v>
       </c>
       <c r="E2" s="36">
         <f t="shared" si="0"/>
-        <v>29473.518461538464</v>
+        <v>24114.696923076925</v>
       </c>
       <c r="F2" s="34">
         <f t="shared" si="0"/>
-        <v>182246.36699999991</v>
+        <v>193353.07699999993</v>
       </c>
       <c r="G2" s="35">
         <f t="shared" si="0"/>
-        <v>183530.03999999995</v>
+        <v>193320.75999999995</v>
       </c>
       <c r="H2" s="36">
         <f t="shared" si="0"/>
-        <v>52760.916923076889</v>
+        <v>41455.00615384613</v>
       </c>
       <c r="I2" s="34">
         <f t="shared" si="0"/>
-        <v>2044.4</v>
+        <v>4381.3999999999996</v>
       </c>
       <c r="J2" s="35">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3078.0459809999998</v>
       </c>
       <c r="K2" s="36">
         <f t="shared" si="0"/>
-        <v>595000.00000000035</v>
+        <v>591000.00000000047</v>
       </c>
       <c r="L2" s="34">
         <f t="shared" si="0"/>
-        <v>287661.43249999994</v>
+        <v>318776.58249999984</v>
       </c>
       <c r="M2" s="36">
         <f t="shared" si="0"/>
-        <v>769950.58561538265</v>
+        <v>711087.49111538311</v>
       </c>
       <c r="N2" s="29"/>
     </row>
@@ -31365,7 +31375,7 @@
       </c>
       <c r="Y5" s="5">
         <f t="shared" si="2"/>
-        <v>26440.939999999995</v>
+        <v>43609.425980999993</v>
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
@@ -31452,7 +31462,7 @@
       </c>
       <c r="Y6" s="5">
         <f t="shared" si="4"/>
-        <v>51661.830769230757</v>
+        <v>30997.098461538462</v>
       </c>
       <c r="Z6" s="5">
         <f t="shared" si="4"/>
@@ -31579,7 +31589,7 @@
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="5"/>
-        <v>12311.949999999999</v>
+        <v>43427.1</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="5"/>
@@ -31666,7 +31676,7 @@
       </c>
       <c r="Y9" s="5">
         <f t="shared" si="6"/>
-        <v>99614.467615384623</v>
+        <v>40751.373115384602</v>
       </c>
       <c r="Z9" s="5">
         <f t="shared" si="6"/>
@@ -31793,19 +31803,19 @@
       </c>
       <c r="Y11" s="5">
         <f t="shared" si="7"/>
-        <v>358193.69076923071</v>
+        <v>354697.44444253843</v>
       </c>
       <c r="Z11" s="5">
         <f t="shared" si="7"/>
-        <v>433766.29538461531</v>
+        <v>430270.04905792302</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="7"/>
-        <v>483766.29538461531</v>
+        <v>480270.04905792302</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="7"/>
-        <v>533766.29538461531</v>
+        <v>530270.04905792302</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
@@ -31880,19 +31890,19 @@
       </c>
       <c r="Y12" s="5">
         <f t="shared" si="8"/>
-        <v>387275.90011538466</v>
+        <v>359527.95561538462</v>
       </c>
       <c r="Z12" s="5">
         <f t="shared" si="8"/>
-        <v>456724.05311538465</v>
+        <v>428976.10861538467</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="8"/>
-        <v>524029.9381153846</v>
+        <v>496281.99361538462</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="8"/>
-        <v>560276.27311538463</v>
+        <v>532528.32861538464</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -31967,19 +31977,19 @@
       </c>
       <c r="Y13" s="5">
         <f t="shared" si="9"/>
-        <v>-29082.209346153948</v>
+        <v>-4830.5111728461925</v>
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>-22957.757730769343</v>
+        <v>1293.9404425383545</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
-        <v>-40263.642730769294</v>
+        <v>-16011.944557461597</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>-26509.977730769315</v>
+        <v>-2258.2795574616175</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
@@ -41488,10 +41498,10 @@
       <c r="K251" s="5">
         <v>0</v>
       </c>
-      <c r="L251" s="157"/>
-      <c r="M251" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L251" s="157">
+        <v>2101.6799999999998</v>
+      </c>
+      <c r="M251" s="41"/>
       <c r="O251" s="29"/>
       <c r="P251" s="5"/>
       <c r="R251" s="5"/>
@@ -41527,9 +41537,7 @@
         <v>0</v>
       </c>
       <c r="L252" s="157"/>
-      <c r="M252" s="41">
-        <v>0</v>
-      </c>
+      <c r="M252" s="41"/>
       <c r="O252" s="29"/>
       <c r="P252" s="5"/>
       <c r="R252" s="5"/>
@@ -41564,10 +41572,10 @@
       <c r="K253" s="5">
         <v>0</v>
       </c>
-      <c r="L253" s="157"/>
-      <c r="M253" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L253" s="157">
+        <v>0</v>
+      </c>
+      <c r="M253" s="41"/>
       <c r="O253" s="29"/>
       <c r="P253" s="5"/>
       <c r="R253" s="5"/>
@@ -41602,10 +41610,10 @@
       <c r="K254" s="5">
         <v>0</v>
       </c>
-      <c r="L254" s="157"/>
-      <c r="M254" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L254" s="157">
+        <v>5359.8399999999992</v>
+      </c>
+      <c r="M254" s="41"/>
       <c r="O254" s="29"/>
       <c r="P254" s="5"/>
       <c r="R254" s="5"/>
@@ -41640,10 +41648,10 @@
       <c r="K255" s="5">
         <v>0</v>
       </c>
-      <c r="L255" s="157"/>
-      <c r="M255" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L255" s="157">
+        <v>467.03999999999996</v>
+      </c>
+      <c r="M255" s="41"/>
       <c r="O255" s="29"/>
       <c r="P255" s="5"/>
       <c r="R255" s="5"/>
@@ -41678,10 +41686,10 @@
       <c r="K256" s="5">
         <v>0</v>
       </c>
-      <c r="L256" s="157"/>
-      <c r="M256" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L256" s="157">
+        <v>2014.11</v>
+      </c>
+      <c r="M256" s="41"/>
       <c r="O256" s="29"/>
       <c r="P256" s="5"/>
       <c r="R256" s="5"/>
@@ -41716,10 +41724,10 @@
       <c r="K257" s="5">
         <v>0</v>
       </c>
-      <c r="L257" s="157"/>
-      <c r="M257" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L257" s="157">
+        <v>895.16</v>
+      </c>
+      <c r="M257" s="41"/>
       <c r="O257" s="29"/>
       <c r="P257" s="5"/>
       <c r="R257" s="5"/>
@@ -41754,10 +41762,10 @@
       <c r="K258" s="5">
         <v>0</v>
       </c>
-      <c r="L258" s="157"/>
-      <c r="M258" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+      <c r="L258" s="157">
+        <v>895.16</v>
+      </c>
+      <c r="M258" s="41"/>
       <c r="O258" s="29"/>
       <c r="P258" s="5"/>
       <c r="R258" s="5"/>
@@ -41793,9 +41801,7 @@
         <v>0</v>
       </c>
       <c r="L259" s="157"/>
-      <c r="M259" s="41">
-        <v>0</v>
-      </c>
+      <c r="M259" s="41"/>
       <c r="O259" s="29"/>
       <c r="P259" s="5"/>
       <c r="R259" s="5"/>
@@ -41811,31 +41817,33 @@
         <f t="shared" si="15"/>
         <v>set/26</v>
       </c>
-      <c r="C260" s="39"/>
+      <c r="C260" s="39">
+        <v>1488.4</v>
+      </c>
       <c r="D260" s="40">
         <v>1345.3200000000004</v>
       </c>
-      <c r="E260" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F260" s="39"/>
+      <c r="E260" s="42"/>
+      <c r="F260" s="39">
+        <v>2174.9</v>
+      </c>
       <c r="G260" s="40">
         <v>1986.8200000000004</v>
       </c>
-      <c r="H260" s="182">
-        <v>1884.3184615384612</v>
-      </c>
+      <c r="H260" s="42"/>
       <c r="I260" s="39">
         <v>1118</v>
       </c>
-      <c r="J260" s="40"/>
+      <c r="J260" s="40">
+        <v>0</v>
+      </c>
       <c r="K260" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L260" s="157"/>
-      <c r="M260" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L260" s="157">
+        <v>5176.3599999999997</v>
+      </c>
+      <c r="M260" s="41"/>
       <c r="O260" s="29"/>
       <c r="P260" s="5"/>
       <c r="R260" s="5"/>
@@ -41851,25 +41859,33 @@
         <f t="shared" ref="B261:B324" si="17">TEXT(A261,"MMM/AA")</f>
         <v>set/26</v>
       </c>
-      <c r="C261" s="39"/>
-      <c r="D261" s="40"/>
-      <c r="E261" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F261" s="39"/>
-      <c r="G261" s="40"/>
-      <c r="H261" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I261" s="39"/>
-      <c r="J261" s="40"/>
+      <c r="C261" s="39">
+        <v>896.61</v>
+      </c>
+      <c r="D261" s="40">
+        <v>1171.5799999999997</v>
+      </c>
+      <c r="E261" s="42"/>
+      <c r="F261" s="39">
+        <v>1620.7</v>
+      </c>
+      <c r="G261" s="40">
+        <v>2013.1200000000003</v>
+      </c>
+      <c r="H261" s="42"/>
+      <c r="I261" s="39">
+        <v>445</v>
+      </c>
+      <c r="J261" s="40">
+        <v>401.78</v>
+      </c>
       <c r="K261" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L261" s="157"/>
-      <c r="M261" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L261" s="157">
+        <v>758.93999999999994</v>
+      </c>
+      <c r="M261" s="41"/>
       <c r="O261" s="29"/>
       <c r="P261" s="5"/>
       <c r="R261" s="5"/>
@@ -41885,25 +41901,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C262" s="39"/>
-      <c r="D262" s="40"/>
-      <c r="E262" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F262" s="39"/>
-      <c r="G262" s="40"/>
-      <c r="H262" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I262" s="39"/>
-      <c r="J262" s="40"/>
+      <c r="C262" s="39">
+        <v>637.30999999999995</v>
+      </c>
+      <c r="D262" s="40">
+        <v>288.83999999999997</v>
+      </c>
+      <c r="E262" s="42"/>
+      <c r="F262" s="39">
+        <v>2073.8200000000002</v>
+      </c>
+      <c r="G262" s="40">
+        <v>2534.7800000000007</v>
+      </c>
+      <c r="H262" s="42"/>
+      <c r="I262" s="39">
+        <v>722</v>
+      </c>
+      <c r="J262" s="40">
+        <v>669.67598100000009</v>
+      </c>
       <c r="K262" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L262" s="157"/>
-      <c r="M262" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L262" s="157">
+        <v>5409.8799999999992</v>
+      </c>
+      <c r="M262" s="41"/>
       <c r="O262" s="29"/>
       <c r="P262" s="5"/>
       <c r="R262" s="5"/>
@@ -41919,25 +41943,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C263" s="39"/>
-      <c r="D263" s="40"/>
-      <c r="E263" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F263" s="39"/>
-      <c r="G263" s="40"/>
-      <c r="H263" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I263" s="39"/>
-      <c r="J263" s="40"/>
+      <c r="C263" s="39">
+        <v>1224.8900000000001</v>
+      </c>
+      <c r="D263" s="40">
+        <v>786.49999999999989</v>
+      </c>
+      <c r="E263" s="42"/>
+      <c r="F263" s="39">
+        <v>1905.64</v>
+      </c>
+      <c r="G263" s="40">
+        <v>2315.7399999999998</v>
+      </c>
+      <c r="H263" s="42"/>
+      <c r="I263" s="39">
+        <v>925</v>
+      </c>
+      <c r="J263" s="40">
+        <v>987.55999999999983</v>
+      </c>
       <c r="K263" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L263" s="157"/>
-      <c r="M263" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L263" s="157">
+        <v>914.61999999999989</v>
+      </c>
+      <c r="M263" s="41"/>
       <c r="O263" s="29"/>
       <c r="P263" s="5"/>
       <c r="R263" s="5"/>
@@ -41953,25 +41985,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C264" s="39"/>
-      <c r="D264" s="40"/>
-      <c r="E264" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F264" s="39"/>
-      <c r="G264" s="40"/>
-      <c r="H264" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I264" s="39"/>
-      <c r="J264" s="40"/>
+      <c r="C264" s="39">
+        <v>1223.3399999999999</v>
+      </c>
+      <c r="D264" s="40">
+        <v>1092.96</v>
+      </c>
+      <c r="E264" s="42"/>
+      <c r="F264" s="39">
+        <v>2147.21</v>
+      </c>
+      <c r="G264" s="40">
+        <v>1505.4199999999998</v>
+      </c>
+      <c r="H264" s="42"/>
+      <c r="I264" s="39">
+        <v>245</v>
+      </c>
+      <c r="J264" s="40">
+        <v>771.46999999999991</v>
+      </c>
       <c r="K264" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L264" s="157"/>
-      <c r="M264" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L264" s="157">
+        <v>3619.56</v>
+      </c>
+      <c r="M264" s="41"/>
       <c r="O264" s="29"/>
       <c r="P264" s="5"/>
       <c r="R264" s="5"/>
@@ -41987,25 +42027,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C265" s="39"/>
-      <c r="D265" s="40"/>
-      <c r="E265" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F265" s="39"/>
-      <c r="G265" s="40"/>
-      <c r="H265" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I265" s="39"/>
-      <c r="J265" s="40"/>
+      <c r="C265" s="39">
+        <v>326.87</v>
+      </c>
+      <c r="D265" s="40">
+        <v>959.83999999999992</v>
+      </c>
+      <c r="E265" s="42"/>
+      <c r="F265" s="39">
+        <v>1184.44</v>
+      </c>
+      <c r="G265" s="40">
+        <v>1421.6600000000005</v>
+      </c>
+      <c r="H265" s="42"/>
+      <c r="I265" s="39">
+        <v>0</v>
+      </c>
+      <c r="J265" s="40">
+        <v>247.56</v>
+      </c>
       <c r="K265" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L265" s="157"/>
-      <c r="M265" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L265" s="157">
+        <v>3502.7999999999997</v>
+      </c>
+      <c r="M265" s="41"/>
       <c r="O265" s="29"/>
       <c r="P265" s="5"/>
       <c r="R265" s="5"/>
@@ -58195,7 +58243,7 @@
         <v>20095.73</v>
       </c>
       <c r="N2" s="72">
-        <v>7778.88</v>
+        <v>81878.399999999994</v>
       </c>
       <c r="P2" s="29"/>
     </row>
@@ -58240,7 +58288,7 @@
         <v>285583</v>
       </c>
       <c r="N3" s="72">
-        <v>162068</v>
+        <v>167432</v>
       </c>
       <c r="O3" s="4"/>
       <c r="P3" s="29"/>
@@ -58735,7 +58783,7 @@
         <v>1592</v>
       </c>
       <c r="N14" s="72">
-        <v>459</v>
+        <v>483</v>
       </c>
       <c r="P14" s="29"/>
     </row>
@@ -58777,10 +58825,10 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <v>314543.35700000002</v>
+        <v>324336.21000000002</v>
       </c>
       <c r="N15" s="72">
-        <v>293604.81</v>
+        <v>309493.43</v>
       </c>
       <c r="P15" s="29"/>
     </row>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-29T14:35:42.625-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="441" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FC64A70-3345-4C47-94D2-65CC3B4648C3}"/>
+  <xr:revisionPtr revIDLastSave="555" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{598D903D-53BA-4F67-BFC9-0EBCDF09814A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="396">
   <si>
     <t>ACOMPANHAMENTO SUPERESTRUTURA — FOLHA DE ENTRADA</t>
   </si>
@@ -1467,7 +1467,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="30" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1656,6 +1659,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="24">
@@ -2592,15 +2600,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="211">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3157,14 +3166,17 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 10" xfId="4" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 10 10" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal 3" xfId="5" xr:uid="{7C80A04F-F605-4CCE-A63F-3076120C0650}"/>
     <cellStyle name="Normal_Licitadas" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Porcentagem" xfId="2" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Vírgula" xfId="6" builtinId="3"/>
   </cellStyles>
   <dxfs count="15">
     <dxf>
@@ -4131,7 +4143,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N61"/>
+  <dimension ref="B1:P61"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -4142,8 +4154,8 @@
     <col min="13" max="19" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:14" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="193" t="s">
         <v>0</v>
       </c>
@@ -4153,7 +4165,7 @@
       <c r="F2" s="194"/>
       <c r="G2" s="194"/>
     </row>
-    <row r="3" spans="2:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="195" t="s">
         <v>1</v>
       </c>
@@ -4163,7 +4175,7 @@
       <c r="F3" s="196"/>
       <c r="G3" s="197"/>
     </row>
-    <row r="4" spans="2:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="198"/>
       <c r="C4" s="194"/>
       <c r="D4" s="194"/>
@@ -4171,7 +4183,7 @@
       <c r="F4" s="194"/>
       <c r="G4" s="199"/>
     </row>
-    <row r="5" spans="2:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="198"/>
       <c r="C5" s="194"/>
       <c r="D5" s="194"/>
@@ -4179,7 +4191,7 @@
       <c r="F5" s="194"/>
       <c r="G5" s="199"/>
     </row>
-    <row r="6" spans="2:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="198"/>
       <c r="C6" s="194"/>
       <c r="D6" s="194"/>
@@ -4187,7 +4199,7 @@
       <c r="F6" s="194"/>
       <c r="G6" s="199"/>
     </row>
-    <row r="7" spans="2:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="200"/>
       <c r="C7" s="201"/>
       <c r="D7" s="201"/>
@@ -4195,26 +4207,26 @@
       <c r="F7" s="201"/>
       <c r="G7" s="202"/>
     </row>
-    <row r="8" spans="2:14" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="80">
-        <v>46284</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="73" t="s">
         <v>5</v>
       </c>
@@ -4254,8 +4266,14 @@
       <c r="N13" s="75" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O13" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="P13" s="75" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="77" t="s">
         <v>8</v>
       </c>
@@ -4289,10 +4307,16 @@
       <c r="L14" s="79">
         <v>100292</v>
       </c>
-      <c r="M14" s="78"/>
-      <c r="N14" s="79"/>
-    </row>
-    <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M14" s="78">
+        <v>105010</v>
+      </c>
+      <c r="N14" s="79">
+        <v>105184</v>
+      </c>
+      <c r="O14" s="78"/>
+      <c r="P14" s="79"/>
+    </row>
+    <row r="15" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="77" t="s">
         <v>9</v>
       </c>
@@ -4300,7 +4324,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="79">
-        <v>102500</v>
+        <v>105300</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79"/>
@@ -4312,8 +4336,10 @@
       <c r="L15" s="79"/>
       <c r="M15" s="78"/>
       <c r="N15" s="79"/>
-    </row>
-    <row r="16" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O15" s="78"/>
+      <c r="P15" s="79"/>
+    </row>
+    <row r="16" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="77" t="s">
         <v>10</v>
       </c>
@@ -4333,8 +4359,10 @@
       <c r="L16" s="79"/>
       <c r="M16" s="78"/>
       <c r="N16" s="79"/>
-    </row>
-    <row r="17" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O16" s="78"/>
+      <c r="P16" s="79"/>
+    </row>
+    <row r="17" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="77" t="s">
         <v>11</v>
       </c>
@@ -4354,8 +4382,10 @@
       <c r="L17" s="79"/>
       <c r="M17" s="78"/>
       <c r="N17" s="79"/>
-    </row>
-    <row r="18" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O17" s="78"/>
+      <c r="P17" s="79"/>
+    </row>
+    <row r="18" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="77" t="s">
         <v>12</v>
       </c>
@@ -4391,8 +4421,10 @@
       </c>
       <c r="M18" s="78"/>
       <c r="N18" s="79"/>
-    </row>
-    <row r="19" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O18" s="78"/>
+      <c r="P18" s="79"/>
+    </row>
+    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="77" t="s">
         <v>13</v>
       </c>
@@ -4400,7 +4432,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="79">
-        <v>47000</v>
+        <v>52000</v>
       </c>
       <c r="E19" s="78"/>
       <c r="F19" s="79"/>
@@ -4412,8 +4444,10 @@
       <c r="L19" s="79"/>
       <c r="M19" s="78"/>
       <c r="N19" s="79"/>
-    </row>
-    <row r="20" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O19" s="78"/>
+      <c r="P19" s="79"/>
+    </row>
+    <row r="20" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="77" t="s">
         <v>14</v>
       </c>
@@ -4427,26 +4461,28 @@
         <v>23000</v>
       </c>
       <c r="F20" s="79">
-        <v>51460</v>
+        <v>55400</v>
       </c>
       <c r="G20" s="78">
-        <v>60160</v>
+        <v>60000</v>
       </c>
       <c r="H20" s="79">
-        <v>64880</v>
+        <v>71000</v>
       </c>
       <c r="I20" s="78">
         <v>71775</v>
       </c>
       <c r="J20" s="79">
-        <v>71940</v>
+        <v>75100</v>
       </c>
       <c r="K20" s="78"/>
       <c r="L20" s="79"/>
       <c r="M20" s="78"/>
       <c r="N20" s="79"/>
-    </row>
-    <row r="21" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O20" s="78"/>
+      <c r="P20" s="79"/>
+    </row>
+    <row r="21" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="77" t="s">
         <v>15</v>
       </c>
@@ -4466,7 +4502,7 @@
         <v>35000</v>
       </c>
       <c r="H21" s="79">
-        <v>39000</v>
+        <v>40000</v>
       </c>
       <c r="I21" s="78">
         <v>40120</v>
@@ -4474,12 +4510,26 @@
       <c r="J21" s="79">
         <v>45680</v>
       </c>
-      <c r="K21" s="78"/>
-      <c r="L21" s="79"/>
-      <c r="M21" s="78"/>
-      <c r="N21" s="79"/>
-    </row>
-    <row r="22" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K21" s="78">
+        <v>71775</v>
+      </c>
+      <c r="L21" s="79">
+        <v>71940</v>
+      </c>
+      <c r="M21" s="78">
+        <v>47030</v>
+      </c>
+      <c r="N21" s="79">
+        <v>48180</v>
+      </c>
+      <c r="O21" s="78">
+        <v>61300</v>
+      </c>
+      <c r="P21" s="79">
+        <v>61700</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="77" t="s">
         <v>16</v>
       </c>
@@ -4487,7 +4537,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="79">
-        <v>45000</v>
+        <v>47000</v>
       </c>
       <c r="E22" s="78"/>
       <c r="F22" s="79"/>
@@ -4499,8 +4549,10 @@
       <c r="L22" s="79"/>
       <c r="M22" s="78"/>
       <c r="N22" s="79"/>
-    </row>
-    <row r="23" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O22" s="78"/>
+      <c r="P22" s="79"/>
+    </row>
+    <row r="23" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="77" t="s">
         <v>17</v>
       </c>
@@ -4527,7 +4579,7 @@
         <v>38340</v>
       </c>
       <c r="J23" s="79">
-        <v>39100</v>
+        <v>40060</v>
       </c>
       <c r="K23" s="78">
         <v>40100</v>
@@ -4539,10 +4591,12 @@
         <v>41500</v>
       </c>
       <c r="N23" s="79">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="24" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>47010</v>
+      </c>
+      <c r="O23" s="78"/>
+      <c r="P23" s="79"/>
+    </row>
+    <row r="24" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="77" t="s">
         <v>18</v>
       </c>
@@ -4556,7 +4610,7 @@
         <v>34600</v>
       </c>
       <c r="F24" s="79">
-        <v>34980</v>
+        <v>45000</v>
       </c>
       <c r="G24" s="78"/>
       <c r="H24" s="79"/>
@@ -4566,8 +4620,10 @@
       <c r="L24" s="79"/>
       <c r="M24" s="78"/>
       <c r="N24" s="79"/>
-    </row>
-    <row r="25" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O24" s="78"/>
+      <c r="P24" s="79"/>
+    </row>
+    <row r="25" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="77" t="s">
         <v>19</v>
       </c>
@@ -4603,8 +4659,10 @@
       </c>
       <c r="M25" s="78"/>
       <c r="N25" s="79"/>
-    </row>
-    <row r="26" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O25" s="78"/>
+      <c r="P25" s="79"/>
+    </row>
+    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="77" t="s">
         <v>20</v>
       </c>
@@ -4614,8 +4672,12 @@
       <c r="D26" s="79">
         <v>8700</v>
       </c>
-      <c r="E26" s="78"/>
-      <c r="F26" s="79"/>
+      <c r="E26" s="78">
+        <v>34400</v>
+      </c>
+      <c r="F26" s="79">
+        <v>35000</v>
+      </c>
       <c r="G26" s="78"/>
       <c r="H26" s="79"/>
       <c r="I26" s="78"/>
@@ -4624,8 +4686,10 @@
       <c r="L26" s="79"/>
       <c r="M26" s="78"/>
       <c r="N26" s="79"/>
-    </row>
-    <row r="27" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O26" s="78"/>
+      <c r="P26" s="79"/>
+    </row>
+    <row r="27" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="77" t="s">
         <v>21</v>
       </c>
@@ -4639,23 +4703,29 @@
         <v>11607</v>
       </c>
       <c r="F27" s="79">
-        <v>31464</v>
-      </c>
-      <c r="G27" s="78"/>
-      <c r="H27" s="79"/>
+        <v>21540</v>
+      </c>
+      <c r="G27" s="78">
+        <v>23020</v>
+      </c>
+      <c r="H27" s="79">
+        <v>37020</v>
+      </c>
       <c r="I27" s="78"/>
       <c r="J27" s="79"/>
       <c r="K27" s="78"/>
       <c r="L27" s="79"/>
       <c r="M27" s="78"/>
       <c r="N27" s="79"/>
-    </row>
-    <row r="29" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O27" s="78"/>
+      <c r="P27" s="79"/>
+    </row>
+    <row r="29" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
         <v>23</v>
       </c>
@@ -4663,12 +4733,12 @@
         <v>131260</v>
       </c>
     </row>
-    <row r="31" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="191" t="s">
         <v>25</v>
       </c>
@@ -4687,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="D33" s="81">
-        <v>103820</v>
+        <v>106160</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4695,10 +4765,10 @@
         <v>29</v>
       </c>
       <c r="C34" s="81">
-        <v>104000</v>
+        <v>107440</v>
       </c>
       <c r="D34" s="81">
-        <v>104980</v>
+        <v>108500</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4706,10 +4776,10 @@
         <v>30</v>
       </c>
       <c r="C35" s="81">
-        <v>105020</v>
+        <v>109200</v>
       </c>
       <c r="D35" s="81">
-        <v>105160</v>
+        <v>110700</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4717,33 +4787,25 @@
         <v>31</v>
       </c>
       <c r="C36" s="81">
-        <v>107440</v>
+        <v>112720</v>
       </c>
       <c r="D36" s="81">
-        <v>108500</v>
+        <v>114720</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="192" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="81">
-        <v>110100</v>
-      </c>
-      <c r="D37" s="81">
-        <v>110700</v>
-      </c>
+      <c r="C37" s="81"/>
+      <c r="D37" s="81"/>
     </row>
     <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="192" t="s">
         <v>33</v>
       </c>
-      <c r="C38" s="81">
-        <v>112720</v>
-      </c>
-      <c r="D38" s="81">
-        <v>114720</v>
-      </c>
+      <c r="C38" s="81"/>
+      <c r="D38" s="81"/>
     </row>
     <row r="39" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="192" t="s">
@@ -5042,9 +5104,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" style="7" customWidth="1"/>
-    <col min="2" max="10" width="0" style="7" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="11" width="9.140625" style="7" collapsed="1"/>
-    <col min="12" max="24" width="9.140625" style="7"/>
+    <col min="2" max="10" width="9.140625" style="7" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="24" width="9.140625" style="7"/>
     <col min="25" max="39" width="9.140625" style="83"/>
   </cols>
   <sheetData>
@@ -5341,43 +5402,56 @@
         <v>5.7221466803051929E-2</v>
       </c>
       <c r="L5" s="62">
-        <v>6.838534272852112E-2</v>
+        <f>L6-K6</f>
+        <v>7.1195414356986897E-2</v>
       </c>
       <c r="M5" s="62">
-        <v>5.4980898342331941E-2</v>
+        <f t="shared" ref="M5:X5" si="1">M6-L6</f>
+        <v>8.188176322115398E-2</v>
       </c>
       <c r="N5" s="62">
-        <v>4.9262025827937761E-2</v>
+        <f t="shared" si="1"/>
+        <v>4.8233907822541167E-2</v>
       </c>
       <c r="O5" s="62">
-        <v>7.9219165797931257E-2</v>
+        <f t="shared" si="1"/>
+        <v>5.7602435507203731E-2</v>
       </c>
       <c r="P5" s="62">
-        <v>6.3407609757920314E-2</v>
+        <f t="shared" si="1"/>
+        <v>5.9597632283525326E-2</v>
       </c>
       <c r="Q5" s="62">
-        <v>6.6420533761949452E-2</v>
+        <f t="shared" si="1"/>
+        <v>6.6399322145811235E-2</v>
       </c>
       <c r="R5" s="62">
-        <v>6.4862832753759814E-2</v>
+        <f t="shared" si="1"/>
+        <v>6.337337741019422E-2</v>
       </c>
       <c r="S5" s="62">
-        <v>6.8231813326713797E-2</v>
+        <f t="shared" si="1"/>
+        <v>6.5918181443970547E-2</v>
       </c>
       <c r="T5" s="62">
-        <v>7.3676056959709468E-2</v>
+        <f t="shared" si="1"/>
+        <v>7.6648971764140539E-2</v>
       </c>
       <c r="U5" s="62">
-        <v>5.5051669806670644E-2</v>
+        <f t="shared" si="1"/>
+        <v>5.8794301524071946E-2</v>
       </c>
       <c r="V5" s="62">
-        <v>5.6373363884686056E-2</v>
+        <f t="shared" si="1"/>
+        <v>5.350472654669014E-2</v>
       </c>
       <c r="W5" s="62">
-        <v>4.97874413665923E-2</v>
+        <f t="shared" si="1"/>
+        <v>5.3740477450843316E-2</v>
       </c>
       <c r="X5" s="62">
-        <v>7.4454204409100111E-3</v>
+        <f t="shared" si="1"/>
+        <v>4.4939541135864403E-3</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
@@ -5397,60 +5471,46 @@
         <v>0.18110000000000001</v>
       </c>
       <c r="K6" s="62">
-        <f>K5+J6</f>
-        <v>0.23832146680305194</v>
+        <v>0.23861553440928052</v>
       </c>
       <c r="L6" s="62">
-        <f t="shared" ref="L6:X6" si="1">L5+K6</f>
-        <v>0.30670680953157303</v>
+        <v>0.30981094876626741</v>
       </c>
       <c r="M6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.36168770787390497</v>
+        <v>0.39169271198742139</v>
       </c>
       <c r="N6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.41094973370184273</v>
+        <v>0.43992661980996256</v>
       </c>
       <c r="O6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.49016889949977399</v>
+        <v>0.49752905531716629</v>
       </c>
       <c r="P6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.5535765092576943</v>
+        <v>0.55712668760069162</v>
       </c>
       <c r="Q6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.61999704301964376</v>
+        <v>0.62352600974650285</v>
       </c>
       <c r="R6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.68485987577340357</v>
+        <v>0.68689938715669707</v>
       </c>
       <c r="S6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.75309168910011737</v>
+        <v>0.75281756860066762</v>
       </c>
       <c r="T6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.82676774605982684</v>
+        <v>0.82946654036480816</v>
       </c>
       <c r="U6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.88181941586649748</v>
+        <v>0.8882608418888801</v>
       </c>
       <c r="V6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.93819277975118354</v>
+        <v>0.94176556843557024</v>
       </c>
       <c r="W6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.98798022111777584</v>
+        <v>0.99550604588641356</v>
       </c>
       <c r="X6" s="62">
-        <f t="shared" si="1"/>
-        <v>0.99542564155868585</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -5485,7 +5545,7 @@
         <v>4.0500000000000008E-2</v>
       </c>
       <c r="K7" s="62">
-        <v>1.8600000000000005E-2</v>
+        <v>4.3200000000000016E-2</v>
       </c>
       <c r="L7" s="62"/>
       <c r="M7" s="62"/>
@@ -5543,7 +5603,7 @@
       </c>
       <c r="K8" s="62">
         <f t="shared" si="2"/>
-        <v>0.19970000000000002</v>
+        <v>0.22430000000000003</v>
       </c>
       <c r="L8" s="62"/>
       <c r="M8" s="62"/>
@@ -5828,44 +5888,42 @@
         <v>6.3208252221123126E-2</v>
       </c>
       <c r="L14" s="62">
-        <v>6.6670982606025331E-2</v>
+        <v>7.1195414356986897E-2</v>
       </c>
       <c r="M14" s="62">
-        <v>5.9593114964889331E-2</v>
+        <v>8.188176322115398E-2</v>
       </c>
       <c r="N14" s="62">
-        <v>5.6203080462458657E-2</v>
+        <v>4.8233907822541167E-2</v>
       </c>
       <c r="O14" s="62">
-        <v>7.1947067934844719E-2</v>
+        <v>5.7602435507203731E-2</v>
       </c>
       <c r="P14" s="62">
-        <v>6.4043364522890792E-2</v>
+        <v>5.9597632283525326E-2</v>
       </c>
       <c r="Q14" s="62">
-        <v>6.5451590728183809E-2</v>
+        <v>6.6399322145811235E-2</v>
       </c>
       <c r="R14" s="62">
-        <v>6.4690641558152739E-2</v>
+        <v>6.337337741019422E-2</v>
       </c>
       <c r="S14" s="62">
-        <v>6.5138507184757749E-2</v>
+        <v>6.5918181443970547E-2</v>
       </c>
       <c r="T14" s="62">
-        <v>7.1007960471492521E-2</v>
+        <v>7.6648971764140539E-2</v>
       </c>
       <c r="U14" s="62">
-        <v>5.1315395251485478E-2</v>
+        <v>5.8794301524071946E-2</v>
       </c>
       <c r="V14" s="62">
-        <v>4.5520343246704953E-2</v>
+        <v>5.350472654669014E-2</v>
       </c>
       <c r="W14" s="62">
-        <v>4.9492344068807148E-2</v>
-      </c>
-      <c r="X14" s="62">
-        <v>2.254641027713597E-2</v>
-      </c>
+        <v>5.3740477450843316E-2</v>
+      </c>
+      <c r="X14" s="62"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -5889,55 +5947,55 @@
       </c>
       <c r="L15" s="62">
         <f t="shared" si="3"/>
-        <v>0.3130501791141217</v>
+        <v>0.31757461086508326</v>
       </c>
       <c r="M15" s="62">
         <f t="shared" si="3"/>
-        <v>0.37264329407901103</v>
+        <v>0.39945637408623724</v>
       </c>
       <c r="N15" s="62">
         <f t="shared" si="3"/>
-        <v>0.42884637454146968</v>
+        <v>0.44769028190877841</v>
       </c>
       <c r="O15" s="62">
         <f t="shared" si="3"/>
-        <v>0.50079344247631441</v>
+        <v>0.50529271741598214</v>
       </c>
       <c r="P15" s="62">
         <f t="shared" si="3"/>
-        <v>0.56483680699920524</v>
+        <v>0.56489034969950747</v>
       </c>
       <c r="Q15" s="62">
         <f t="shared" si="3"/>
-        <v>0.63028839772738909</v>
+        <v>0.6312896718453187</v>
       </c>
       <c r="R15" s="62">
         <f t="shared" si="3"/>
-        <v>0.69497903928554183</v>
+        <v>0.69466304925551292</v>
       </c>
       <c r="S15" s="62">
         <f t="shared" si="3"/>
-        <v>0.76011754647029961</v>
+        <v>0.76058123069948347</v>
       </c>
       <c r="T15" s="62">
         <f t="shared" si="3"/>
-        <v>0.8311255069417921</v>
+        <v>0.83723020246362401</v>
       </c>
       <c r="U15" s="62">
         <f t="shared" si="3"/>
-        <v>0.88244090219327753</v>
+        <v>0.89602450398769595</v>
       </c>
       <c r="V15" s="62">
         <f t="shared" si="3"/>
-        <v>0.92796124543998249</v>
+        <v>0.94952923053438609</v>
       </c>
       <c r="W15" s="62">
         <f t="shared" si="3"/>
-        <v>0.97745358950878969</v>
+        <v>1.0032697079852295</v>
       </c>
       <c r="X15" s="62">
         <f t="shared" si="3"/>
-        <v>0.99999999978592569</v>
+        <v>1.0032697079852295</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.25">
@@ -6256,11 +6314,9 @@
         <v>239</v>
       </c>
       <c r="K22" s="86">
-        <v>241</v>
-      </c>
-      <c r="L22" s="86">
-        <v>237</v>
-      </c>
+        <v>229</v>
+      </c>
+      <c r="L22" s="86"/>
       <c r="M22" s="62"/>
       <c r="N22" s="62"/>
       <c r="O22" s="62"/>
@@ -6490,11 +6546,9 @@
         <v>109</v>
       </c>
       <c r="K27" s="87">
-        <v>113</v>
-      </c>
-      <c r="L27" s="86">
-        <v>1.1000000000000001</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="L27" s="86"/>
       <c r="M27" s="62"/>
       <c r="N27" s="62"/>
       <c r="O27" s="62"/>
@@ -6724,11 +6778,9 @@
         <v>46</v>
       </c>
       <c r="K32" s="86">
-        <v>46</v>
-      </c>
-      <c r="L32" s="86">
-        <v>46</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="L32" s="86"/>
       <c r="M32" s="62"/>
       <c r="N32" s="62"/>
       <c r="O32" s="62"/>
@@ -6958,11 +7010,9 @@
         <v>48</v>
       </c>
       <c r="K37" s="87">
-        <v>48</v>
-      </c>
-      <c r="L37" s="87">
-        <v>48</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="L37" s="87"/>
       <c r="M37" s="62"/>
       <c r="N37" s="62"/>
       <c r="O37" s="62"/>
@@ -7593,7 +7643,7 @@
         <v>96</v>
       </c>
       <c r="U4" s="103">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="V4" s="102">
         <v>96</v>
@@ -8894,7 +8944,9 @@
       <c r="T12" s="102">
         <v>3</v>
       </c>
-      <c r="U12" s="103"/>
+      <c r="U12" s="103">
+        <v>3</v>
+      </c>
       <c r="V12" s="102">
         <v>3</v>
       </c>
@@ -9057,7 +9109,7 @@
         <v>5</v>
       </c>
       <c r="U13" s="13">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V13" s="12">
         <v>5</v>
@@ -9384,9 +9436,7 @@
       <c r="T15" s="12">
         <v>4</v>
       </c>
-      <c r="U15" s="13">
-        <v>8</v>
-      </c>
+      <c r="U15" s="13"/>
       <c r="V15" s="12">
         <v>4</v>
       </c>
@@ -9713,7 +9763,7 @@
         <v>23</v>
       </c>
       <c r="U17" s="13">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="V17" s="12">
         <v>23</v>
@@ -9877,7 +9927,7 @@
         <v>2</v>
       </c>
       <c r="U18" s="103">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V18" s="102">
         <v>2</v>
@@ -10041,7 +10091,7 @@
         <v>22</v>
       </c>
       <c r="U19" s="13">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="V19" s="12">
         <v>22</v>
@@ -10205,7 +10255,7 @@
         <v>18</v>
       </c>
       <c r="U20" s="103">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="V20" s="102">
         <v>18</v>
@@ -10369,7 +10419,7 @@
         <v>3</v>
       </c>
       <c r="U21" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V21" s="12">
         <v>3</v>
@@ -10858,7 +10908,9 @@
       <c r="T24" s="102">
         <v>6</v>
       </c>
-      <c r="U24" s="103"/>
+      <c r="U24" s="103">
+        <v>4</v>
+      </c>
       <c r="V24" s="102">
         <v>6</v>
       </c>
@@ -11184,9 +11236,7 @@
       <c r="T26" s="102">
         <v>1</v>
       </c>
-      <c r="U26" s="103">
-        <v>4</v>
-      </c>
+      <c r="U26" s="103"/>
       <c r="V26" s="102">
         <v>1</v>
       </c>
@@ -11346,7 +11396,9 @@
       <c r="T27" s="12">
         <v>8</v>
       </c>
-      <c r="U27" s="13"/>
+      <c r="U27" s="13">
+        <v>4</v>
+      </c>
       <c r="V27" s="12">
         <v>8</v>
       </c>
@@ -12165,7 +12217,7 @@
         <v>3</v>
       </c>
       <c r="U32" s="108">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V32" s="107">
         <v>3</v>
@@ -12349,7 +12401,7 @@
       </c>
       <c r="U33" s="113">
         <f t="shared" si="8"/>
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="V33" s="113">
         <f t="shared" si="8"/>
@@ -14129,7 +14181,7 @@
         <v>16</v>
       </c>
       <c r="U44" s="103">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="V44" s="102">
         <v>16</v>
@@ -14290,7 +14342,9 @@
       <c r="T45" s="12">
         <v>2</v>
       </c>
-      <c r="U45" s="13"/>
+      <c r="U45" s="13">
+        <v>1</v>
+      </c>
       <c r="V45" s="12">
         <v>2</v>
       </c>
@@ -14453,7 +14507,7 @@
         <v>6</v>
       </c>
       <c r="U46" s="103">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V46" s="102">
         <v>6</v>
@@ -16910,7 +16964,9 @@
       <c r="T61" s="12">
         <v>2</v>
       </c>
-      <c r="U61" s="13"/>
+      <c r="U61" s="13">
+        <v>2</v>
+      </c>
       <c r="V61" s="12">
         <v>2</v>
       </c>
@@ -17070,7 +17126,9 @@
       <c r="T62" s="102">
         <v>2</v>
       </c>
-      <c r="U62" s="103"/>
+      <c r="U62" s="103">
+        <v>2</v>
+      </c>
       <c r="V62" s="102">
         <v>2</v>
       </c>
@@ -17233,7 +17291,7 @@
         <v>2</v>
       </c>
       <c r="U63" s="13">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V63" s="12">
         <v>2</v>
@@ -17561,7 +17619,7 @@
         <v>3</v>
       </c>
       <c r="U65" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V65" s="12">
         <v>3</v>
@@ -17725,7 +17783,7 @@
         <v>8</v>
       </c>
       <c r="U66" s="103">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="V66" s="102">
         <v>8</v>
@@ -17889,7 +17947,7 @@
         <v>8</v>
       </c>
       <c r="U67" s="13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V67" s="12">
         <v>8</v>
@@ -18053,7 +18111,7 @@
         <v>3</v>
       </c>
       <c r="U68" s="103">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V68" s="102">
         <v>3</v>
@@ -18214,7 +18272,9 @@
       <c r="T69" s="12">
         <v>1</v>
       </c>
-      <c r="U69" s="13"/>
+      <c r="U69" s="13">
+        <v>1</v>
+      </c>
       <c r="V69" s="12">
         <v>1</v>
       </c>
@@ -19193,7 +19253,7 @@
         <v>3</v>
       </c>
       <c r="U75" s="13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V75" s="12">
         <v>3</v>
@@ -19357,7 +19417,7 @@
         <v>6</v>
       </c>
       <c r="U76" s="103">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V76" s="102">
         <v>6</v>
@@ -19518,7 +19578,9 @@
       <c r="T77" s="12">
         <v>1</v>
       </c>
-      <c r="U77" s="13"/>
+      <c r="U77" s="13">
+        <v>1</v>
+      </c>
       <c r="V77" s="12">
         <v>1</v>
       </c>
@@ -19681,7 +19743,7 @@
         <v>1</v>
       </c>
       <c r="U78" s="108">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="V78" s="107">
         <v>1</v>
@@ -19865,7 +19927,7 @@
       </c>
       <c r="U79" s="112">
         <f t="shared" si="18"/>
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="V79" s="112">
         <f t="shared" si="18"/>
@@ -21321,7 +21383,7 @@
         <v>8</v>
       </c>
       <c r="U88" s="103">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V88" s="102">
         <v>8</v>
@@ -21669,7 +21731,7 @@
       </c>
       <c r="U90" s="112">
         <f t="shared" si="28"/>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="V90" s="112">
         <f t="shared" si="28"/>
@@ -27186,7 +27248,7 @@
         <v>1105</v>
       </c>
       <c r="I5" s="68">
-        <v>880</v>
+        <v>1155</v>
       </c>
       <c r="J5" s="68"/>
       <c r="K5" s="68"/>
@@ -27243,7 +27305,7 @@
         <v>21</v>
       </c>
       <c r="I6" s="69">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J6" s="69"/>
       <c r="K6" s="69"/>
@@ -27293,7 +27355,7 @@
       </c>
       <c r="I7" s="69">
         <f t="shared" si="2"/>
-        <v>51.764705882352942</v>
+        <v>50.217391304347828</v>
       </c>
       <c r="J7" s="69"/>
       <c r="K7" s="69"/>
@@ -27357,37 +27419,37 @@
         <v>1051</v>
       </c>
       <c r="I8" s="147">
-        <v>1402.1999999999998</v>
+        <v>1352.8999999999996</v>
       </c>
       <c r="J8" s="147">
-        <v>1370.6999999999998</v>
+        <v>1385.1000000000004</v>
       </c>
       <c r="K8" s="147">
-        <v>1240.1000000000004</v>
+        <v>1253.1999999999998</v>
       </c>
       <c r="L8" s="147">
-        <v>913.79999999999927</v>
+        <v>923.40000000000055</v>
       </c>
       <c r="M8" s="147">
-        <v>1240.1000000000004</v>
+        <v>1253.2000000000007</v>
       </c>
       <c r="N8" s="147">
-        <v>1305.3999999999996</v>
+        <v>1319.2000000000007</v>
       </c>
       <c r="O8" s="147">
-        <v>1501.2000000000007</v>
+        <v>1517.1000000000004</v>
       </c>
       <c r="P8" s="147">
-        <v>1435.8999999999996</v>
+        <v>1451.1000000000004</v>
       </c>
       <c r="Q8" s="147">
-        <v>1370.7000000000007</v>
+        <v>1385.1000000000004</v>
       </c>
       <c r="R8" s="147">
-        <v>1435.8999999999996</v>
+        <v>1451.0999999999985</v>
       </c>
       <c r="S8" s="147">
-        <v>1066.0999999999985</v>
+        <v>990.69999999999709</v>
       </c>
       <c r="T8" s="147">
         <v>0</v>
@@ -27530,47 +27592,47 @@
       </c>
       <c r="I10" s="69">
         <f t="shared" si="5"/>
-        <v>56.087999999999994</v>
+        <v>54.115999999999985</v>
       </c>
       <c r="J10" s="69">
         <f t="shared" si="5"/>
-        <v>50.766666666666659</v>
+        <v>51.300000000000011</v>
       </c>
       <c r="K10" s="69">
         <f t="shared" si="5"/>
-        <v>49.604000000000013</v>
+        <v>50.127999999999993</v>
       </c>
       <c r="L10" s="69">
         <f t="shared" si="5"/>
-        <v>57.112499999999955</v>
+        <v>57.712500000000034</v>
       </c>
       <c r="M10" s="69">
         <f t="shared" si="5"/>
-        <v>51.670833333333348</v>
+        <v>52.216666666666697</v>
       </c>
       <c r="N10" s="69">
         <f t="shared" si="5"/>
-        <v>54.391666666666652</v>
+        <v>54.966666666666697</v>
       </c>
       <c r="O10" s="69">
         <f t="shared" si="5"/>
-        <v>55.60000000000003</v>
+        <v>56.188888888888904</v>
       </c>
       <c r="P10" s="69">
         <f t="shared" si="5"/>
-        <v>55.226923076923065</v>
+        <v>55.811538461538476</v>
       </c>
       <c r="Q10" s="69">
         <f t="shared" si="5"/>
-        <v>52.719230769230798</v>
+        <v>53.273076923076935</v>
       </c>
       <c r="R10" s="69">
         <f t="shared" si="5"/>
-        <v>55.226923076923065</v>
+        <v>55.811538461538404</v>
       </c>
       <c r="S10" s="69">
         <f t="shared" si="5"/>
-        <v>39.485185185185131</v>
+        <v>36.692592592592483</v>
       </c>
       <c r="T10" s="69">
         <f t="shared" si="5"/>
@@ -27951,7 +28013,7 @@
         <v>20537</v>
       </c>
       <c r="I16" s="153">
-        <v>9855</v>
+        <v>13615</v>
       </c>
       <c r="J16" s="153"/>
       <c r="K16" s="153"/>
@@ -27994,7 +28056,7 @@
         <v>16</v>
       </c>
       <c r="I17" s="69">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J17" s="69"/>
       <c r="K17" s="69"/>
@@ -28044,7 +28106,7 @@
       </c>
       <c r="I18" s="69">
         <f t="shared" si="7"/>
-        <v>758.07692307692309</v>
+        <v>800.88235294117646</v>
       </c>
       <c r="J18" s="69"/>
       <c r="K18" s="69"/>
@@ -28092,19 +28154,19 @@
         <v>16832</v>
       </c>
       <c r="I19" s="147">
-        <v>19957.899999999994</v>
+        <v>19642.699999999997</v>
       </c>
       <c r="J19" s="147">
-        <v>19826</v>
+        <v>19828.5</v>
       </c>
       <c r="K19" s="147">
-        <v>16325.200000000012</v>
+        <v>16333.400000000009</v>
       </c>
       <c r="L19" s="147">
         <v>12810.299999999988</v>
       </c>
       <c r="M19" s="147">
-        <v>17729.700000000012</v>
+        <v>17724.5</v>
       </c>
       <c r="N19" s="147">
         <v>18617.200000000012</v>
@@ -28113,10 +28175,10 @@
         <v>21409.799999999988</v>
       </c>
       <c r="P19" s="147">
-        <v>20513.899999999994</v>
+        <v>20513.399999999994</v>
       </c>
       <c r="Q19" s="147">
-        <v>19843.299999999988</v>
+        <v>19843.799999999988</v>
       </c>
       <c r="R19" s="147">
         <v>20484.799999999988</v>
@@ -28125,7 +28187,7 @@
         <v>20484.799999999988</v>
       </c>
       <c r="T19" s="147">
-        <v>11236.599999999977</v>
+        <v>11546.299999999988</v>
       </c>
       <c r="U19" s="147">
         <v>0</v>
@@ -28244,15 +28306,15 @@
       </c>
       <c r="I21" s="69">
         <f t="shared" si="10"/>
-        <v>798.3159999999998</v>
+        <v>785.70799999999986</v>
       </c>
       <c r="J21" s="69">
         <f t="shared" si="10"/>
-        <v>734.2962962962963</v>
+        <v>734.38888888888891</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="10"/>
-        <v>653.00800000000049</v>
+        <v>653.33600000000035</v>
       </c>
       <c r="L21" s="69">
         <f t="shared" si="10"/>
@@ -28260,7 +28322,7 @@
       </c>
       <c r="M21" s="69">
         <f t="shared" si="10"/>
-        <v>738.73750000000052</v>
+        <v>738.52083333333337</v>
       </c>
       <c r="N21" s="69">
         <f t="shared" si="10"/>
@@ -28272,11 +28334,11 @@
       </c>
       <c r="P21" s="69">
         <f t="shared" si="10"/>
-        <v>788.99615384615367</v>
+        <v>788.97692307692284</v>
       </c>
       <c r="Q21" s="69">
         <f t="shared" si="10"/>
-        <v>763.20384615384569</v>
+        <v>763.22307692307652</v>
       </c>
       <c r="R21" s="69">
         <f t="shared" si="10"/>
@@ -28288,7 +28350,7 @@
       </c>
       <c r="T21" s="69">
         <f t="shared" si="10"/>
-        <v>432.17692307692221</v>
+        <v>444.0884615384611</v>
       </c>
       <c r="U21" s="69">
         <f t="shared" si="10"/>
@@ -28619,7 +28681,7 @@
         <v>41202</v>
       </c>
       <c r="I27" s="68">
-        <v>25071</v>
+        <v>34647</v>
       </c>
       <c r="J27" s="68" t="s">
         <v>196</v>
@@ -28688,7 +28750,7 @@
         <v>13</v>
       </c>
       <c r="I28" s="69">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J28" s="69"/>
       <c r="K28" s="69"/>
@@ -28738,7 +28800,7 @@
       </c>
       <c r="I29" s="69">
         <f t="shared" si="12"/>
-        <v>2279.181818181818</v>
+        <v>2665.1538461538462</v>
       </c>
       <c r="J29" s="69"/>
       <c r="K29" s="69"/>
@@ -28786,43 +28848,43 @@
         <v>41202</v>
       </c>
       <c r="I30" s="147">
-        <v>51643.799999999988</v>
+        <v>42976.200000000012</v>
       </c>
       <c r="J30" s="147">
-        <v>85090.700000000012</v>
+        <v>50286.200000000012</v>
       </c>
       <c r="K30" s="147">
-        <v>40690.900000000023</v>
+        <v>55255.166666666686</v>
       </c>
       <c r="L30" s="147">
-        <v>21151</v>
+        <v>37919.966666666674</v>
       </c>
       <c r="M30" s="147">
-        <v>34574</v>
+        <v>49715.066666666651</v>
       </c>
       <c r="N30" s="147">
-        <v>37784.700000000012</v>
+        <v>37907.700000000012</v>
       </c>
       <c r="O30" s="147">
         <v>50217.700000000012</v>
       </c>
       <c r="P30" s="147">
-        <v>45950.599999999977</v>
+        <v>45499.5</v>
       </c>
       <c r="Q30" s="147">
-        <v>51976.699999999953</v>
+        <v>51922.299999999988</v>
       </c>
       <c r="R30" s="147">
-        <v>45354</v>
+        <v>45895.599999999977</v>
       </c>
       <c r="S30" s="147">
-        <v>38685.5</v>
+        <v>36868.900000000023</v>
       </c>
       <c r="T30" s="147">
-        <v>50592.099999999977</v>
+        <v>688152.10000000009</v>
       </c>
       <c r="U30" s="147">
-        <v>0</v>
+        <v>40718.799999999814</v>
       </c>
       <c r="V30" s="147">
         <v>0</v>
@@ -28938,27 +29000,27 @@
       </c>
       <c r="I32" s="69">
         <f t="shared" si="15"/>
-        <v>2065.7519999999995</v>
+        <v>1719.0480000000005</v>
       </c>
       <c r="J32" s="69">
         <f t="shared" si="15"/>
-        <v>3151.5074074074078</v>
+        <v>1862.4518518518523</v>
       </c>
       <c r="K32" s="69">
         <f t="shared" si="15"/>
-        <v>1627.6360000000009</v>
+        <v>2210.2066666666674</v>
       </c>
       <c r="L32" s="69">
         <f t="shared" si="15"/>
-        <v>1321.9375</v>
+        <v>2369.9979166666672</v>
       </c>
       <c r="M32" s="69">
         <f t="shared" si="15"/>
-        <v>1440.5833333333333</v>
+        <v>2071.4611111111103</v>
       </c>
       <c r="N32" s="69">
         <f t="shared" si="15"/>
-        <v>1574.3625000000004</v>
+        <v>1579.4875000000004</v>
       </c>
       <c r="O32" s="69">
         <f t="shared" si="15"/>
@@ -28966,27 +29028,27 @@
       </c>
       <c r="P32" s="69">
         <f t="shared" si="15"/>
-        <v>1767.3307692307683</v>
+        <v>1749.9807692307693</v>
       </c>
       <c r="Q32" s="69">
         <f t="shared" si="15"/>
-        <v>1999.1038461538444</v>
+        <v>1997.0115384615381</v>
       </c>
       <c r="R32" s="69">
         <f t="shared" si="15"/>
-        <v>1744.3846153846155</v>
+        <v>1765.2153846153838</v>
       </c>
       <c r="S32" s="69">
         <f t="shared" si="15"/>
-        <v>1432.7962962962963</v>
+        <v>1365.5148148148157</v>
       </c>
       <c r="T32" s="69">
         <f t="shared" si="15"/>
-        <v>1945.849999999999</v>
+        <v>26467.388461538467</v>
       </c>
       <c r="U32" s="69">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>1566.1076923076851</v>
       </c>
       <c r="V32" s="69">
         <v>0</v>
@@ -29313,7 +29375,7 @@
         <v>57</v>
       </c>
       <c r="I38" s="68">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="J38" s="68" t="s">
         <v>196</v>
@@ -29431,8 +29493,7 @@
         <v>3.3529411764705883</v>
       </c>
       <c r="I40" s="69">
-        <f t="shared" si="17"/>
-        <v>3.625</v>
+        <v>22</v>
       </c>
       <c r="J40" s="69"/>
       <c r="K40" s="69"/>
@@ -29480,46 +29541,46 @@
         <v>57</v>
       </c>
       <c r="I41" s="147">
-        <v>152.10000000000002</v>
+        <v>132.20000000000005</v>
       </c>
       <c r="J41" s="147">
-        <v>238.19999999999993</v>
+        <v>262</v>
       </c>
       <c r="K41" s="147">
-        <v>197.29999999999995</v>
+        <v>196.70000000000005</v>
       </c>
       <c r="L41" s="147">
-        <v>153.5</v>
+        <v>187.40000000000009</v>
       </c>
       <c r="M41" s="147">
-        <v>186.79999999999995</v>
+        <v>214.29999999999995</v>
       </c>
       <c r="N41" s="147">
-        <v>166.5</v>
+        <v>157.29999999999995</v>
       </c>
       <c r="O41" s="147">
-        <v>217.5</v>
+        <v>226.20000000000005</v>
       </c>
       <c r="P41" s="147">
-        <v>262</v>
+        <v>261.79999999999995</v>
       </c>
       <c r="Q41" s="147">
-        <v>271.39999999999986</v>
+        <v>267.80000000000018</v>
       </c>
       <c r="R41" s="147">
-        <v>272.80000000000018</v>
+        <v>288.69999999999982</v>
       </c>
       <c r="S41" s="147">
-        <v>254</v>
+        <v>330.59999999999991</v>
       </c>
       <c r="T41" s="147">
-        <v>235</v>
+        <v>257.80000000000018</v>
       </c>
       <c r="U41" s="147">
-        <v>205</v>
+        <v>80.900000000000091</v>
       </c>
       <c r="V41" s="147">
-        <v>62</v>
+        <v>10.099999999999909</v>
       </c>
       <c r="X41" s="148"/>
     </row>
@@ -29632,55 +29693,55 @@
       </c>
       <c r="I43" s="69">
         <f t="shared" si="20"/>
-        <v>6.0840000000000005</v>
+        <v>5.288000000000002</v>
       </c>
       <c r="J43" s="69">
         <f t="shared" si="20"/>
-        <v>8.8222222222222193</v>
+        <v>9.7037037037037042</v>
       </c>
       <c r="K43" s="69">
         <f t="shared" si="20"/>
-        <v>7.8919999999999986</v>
+        <v>7.8680000000000021</v>
       </c>
       <c r="L43" s="69">
         <f t="shared" si="20"/>
-        <v>9.59375</v>
+        <v>11.712500000000006</v>
       </c>
       <c r="M43" s="69">
         <f t="shared" si="20"/>
-        <v>7.7833333333333314</v>
+        <v>8.9291666666666654</v>
       </c>
       <c r="N43" s="69">
         <f t="shared" si="20"/>
-        <v>6.9375</v>
+        <v>6.5541666666666645</v>
       </c>
       <c r="O43" s="69">
         <f t="shared" si="20"/>
-        <v>8.0555555555555554</v>
+        <v>8.37777777777778</v>
       </c>
       <c r="P43" s="69">
         <f t="shared" si="20"/>
-        <v>10.076923076923077</v>
+        <v>10.069230769230767</v>
       </c>
       <c r="Q43" s="69">
         <f t="shared" si="20"/>
-        <v>10.438461538461533</v>
+        <v>10.300000000000008</v>
       </c>
       <c r="R43" s="69">
         <f t="shared" si="20"/>
-        <v>10.492307692307699</v>
+        <v>11.103846153846147</v>
       </c>
       <c r="S43" s="69">
         <f t="shared" si="20"/>
-        <v>9.4074074074074066</v>
+        <v>12.244444444444442</v>
       </c>
       <c r="T43" s="69">
         <f t="shared" si="20"/>
-        <v>9.0384615384615383</v>
+        <v>9.9153846153846228</v>
       </c>
       <c r="U43" s="69">
         <f t="shared" si="20"/>
-        <v>7.884615384615385</v>
+        <v>3.1115384615384651</v>
       </c>
       <c r="V43" s="69">
         <v>0</v>
@@ -30007,7 +30068,7 @@
         <v>14588</v>
       </c>
       <c r="I49" s="68">
-        <v>10264</v>
+        <v>16920</v>
       </c>
       <c r="J49" s="68" t="s">
         <v>196</v>
@@ -30076,7 +30137,7 @@
         <v>21</v>
       </c>
       <c r="I50" s="69">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J50" s="69"/>
       <c r="K50" s="69"/>
@@ -30126,7 +30187,7 @@
       </c>
       <c r="I51" s="69">
         <f t="shared" si="22"/>
-        <v>933.09090909090912</v>
+        <v>995.29411764705878</v>
       </c>
       <c r="J51" s="69"/>
       <c r="K51" s="69"/>
@@ -30174,47 +30235,45 @@
         <v>13688</v>
       </c>
       <c r="I52" s="147">
-        <v>18847.900000000001</v>
+        <v>19854.100000000006</v>
       </c>
       <c r="J52" s="147">
-        <v>23951.700000000004</v>
+        <v>24090.600000000006</v>
       </c>
       <c r="K52" s="147">
-        <v>24122.800000000003</v>
+        <v>21931.899999999994</v>
       </c>
       <c r="L52" s="147">
-        <v>21545.400000000009</v>
+        <v>18763.100000000006</v>
       </c>
       <c r="M52" s="147">
-        <v>12896.200000000012</v>
+        <v>17120</v>
       </c>
       <c r="N52" s="147">
-        <v>13308.299999999988</v>
+        <v>13402</v>
       </c>
       <c r="O52" s="147">
-        <v>18192</v>
+        <v>18204.100000000006</v>
       </c>
       <c r="P52" s="147">
-        <v>20671.799999999988</v>
+        <v>20481.600000000006</v>
       </c>
       <c r="Q52" s="147">
-        <v>20778.100000000006</v>
+        <v>20755.299999999988</v>
       </c>
       <c r="R52" s="147">
-        <v>25066.299999999988</v>
+        <v>25178.899999999994</v>
       </c>
       <c r="S52" s="147">
-        <v>19499</v>
+        <v>29723.499999999971</v>
       </c>
       <c r="T52" s="147">
-        <v>19063.299999999988</v>
+        <v>20181.5</v>
       </c>
       <c r="U52" s="147">
-        <v>21876.799999999988</v>
-      </c>
-      <c r="V52" s="147">
-        <v>0</v>
-      </c>
+        <v>10132.599999999977</v>
+      </c>
+      <c r="V52" s="147"/>
       <c r="X52" s="148"/>
     </row>
     <row r="53" spans="1:24" s="144" customFormat="1" x14ac:dyDescent="0.25">
@@ -30326,55 +30385,55 @@
       </c>
       <c r="I54" s="69">
         <f t="shared" si="25"/>
-        <v>753.91600000000005</v>
+        <v>794.16400000000021</v>
       </c>
       <c r="J54" s="69">
         <f t="shared" si="25"/>
-        <v>887.10000000000014</v>
+        <v>892.24444444444464</v>
       </c>
       <c r="K54" s="69">
         <f t="shared" si="25"/>
-        <v>964.91200000000015</v>
+        <v>877.27599999999973</v>
       </c>
       <c r="L54" s="69">
         <f t="shared" si="25"/>
-        <v>1346.5875000000005</v>
+        <v>1172.6937500000004</v>
       </c>
       <c r="M54" s="69">
         <f t="shared" si="25"/>
-        <v>537.34166666666715</v>
+        <v>713.33333333333337</v>
       </c>
       <c r="N54" s="69">
         <f t="shared" si="25"/>
-        <v>554.51249999999948</v>
+        <v>558.41666666666663</v>
       </c>
       <c r="O54" s="69">
         <f t="shared" si="25"/>
-        <v>673.77777777777783</v>
+        <v>674.22592592592616</v>
       </c>
       <c r="P54" s="69">
         <f t="shared" si="25"/>
-        <v>795.06923076923033</v>
+        <v>787.75384615384633</v>
       </c>
       <c r="Q54" s="69">
         <f t="shared" si="25"/>
-        <v>799.15769230769251</v>
+        <v>798.28076923076878</v>
       </c>
       <c r="R54" s="69">
         <f t="shared" si="25"/>
-        <v>964.08846153846105</v>
+        <v>968.41923076923058</v>
       </c>
       <c r="S54" s="69">
         <f t="shared" si="25"/>
-        <v>722.18518518518522</v>
+        <v>1100.8703703703693</v>
       </c>
       <c r="T54" s="69">
         <f t="shared" si="25"/>
-        <v>733.20384615384569</v>
+        <v>776.21153846153845</v>
       </c>
       <c r="U54" s="69">
         <f t="shared" si="25"/>
-        <v>841.41538461538414</v>
+        <v>389.7153846153837</v>
       </c>
       <c r="V54" s="69">
         <f t="shared" si="25"/>
@@ -30702,7 +30761,7 @@
         <v>22612</v>
       </c>
       <c r="I60" s="68">
-        <v>21742</v>
+        <v>28922</v>
       </c>
       <c r="J60" s="68" t="s">
         <v>196</v>
@@ -30771,7 +30830,7 @@
         <v>11</v>
       </c>
       <c r="I61" s="69">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J61" s="69"/>
       <c r="K61" s="69"/>
@@ -30820,7 +30879,7 @@
       </c>
       <c r="I62" s="69">
         <f>I60/I61</f>
-        <v>1976.5454545454545</v>
+        <v>1928.1333333333334</v>
       </c>
       <c r="J62" s="69"/>
       <c r="K62" s="69"/>
@@ -30867,46 +30926,46 @@
         <v>20245</v>
       </c>
       <c r="I63" s="147">
-        <v>44708.800000000003</v>
+        <v>35224.199999999997</v>
       </c>
       <c r="J63" s="147">
-        <v>48824.900000000009</v>
+        <v>46993.830769230772</v>
       </c>
       <c r="K63" s="147">
-        <v>49636.299999999988</v>
+        <v>41887.830769230757</v>
       </c>
       <c r="L63" s="147">
-        <v>39908.899999999994</v>
+        <v>40917.930769230763</v>
       </c>
       <c r="M63" s="147">
-        <v>31812.200000000012</v>
+        <v>45112.430769230763</v>
       </c>
       <c r="N63" s="147">
-        <v>28190.300000000017</v>
+        <v>35209.430769230763</v>
       </c>
       <c r="O63" s="147">
-        <v>42949.299999999988</v>
+        <v>44397.03076923074</v>
       </c>
       <c r="P63" s="147">
-        <v>47310.700000000012</v>
+        <v>47746.730769230751</v>
       </c>
       <c r="Q63" s="147">
-        <v>49762.200000000012</v>
+        <v>50767.930769230763</v>
       </c>
       <c r="R63" s="147">
-        <v>50451</v>
+        <v>51729.130769230775</v>
       </c>
       <c r="S63" s="147">
-        <v>53003.400000000023</v>
+        <v>52981.03076923074</v>
       </c>
       <c r="T63" s="147">
-        <v>56170.799999999988</v>
+        <v>33930.730769230751</v>
       </c>
       <c r="U63" s="147">
-        <v>56190</v>
+        <v>50032.330769230728</v>
       </c>
       <c r="V63" s="147">
-        <v>0</v>
+        <v>31989.430769230938</v>
       </c>
       <c r="X63" s="148"/>
     </row>
@@ -31019,55 +31078,55 @@
       </c>
       <c r="I65" s="69">
         <f t="shared" si="29"/>
-        <v>1788.3520000000001</v>
+        <v>1408.9679999999998</v>
       </c>
       <c r="J65" s="69">
         <f t="shared" si="29"/>
-        <v>1808.3296296296301</v>
+        <v>1740.5122507122508</v>
       </c>
       <c r="K65" s="69">
         <f t="shared" si="29"/>
-        <v>1985.4519999999995</v>
+        <v>1675.5132307692302</v>
       </c>
       <c r="L65" s="69">
         <f t="shared" si="29"/>
-        <v>2494.3062499999996</v>
+        <v>2557.3706730769227</v>
       </c>
       <c r="M65" s="69">
         <f t="shared" si="29"/>
-        <v>1325.5083333333339</v>
+        <v>1879.6846153846152</v>
       </c>
       <c r="N65" s="69">
         <f t="shared" si="29"/>
-        <v>1174.595833333334</v>
+        <v>1467.0596153846152</v>
       </c>
       <c r="O65" s="69">
         <f t="shared" si="29"/>
-        <v>1590.7148148148144</v>
+        <v>1644.3344729344719</v>
       </c>
       <c r="P65" s="69">
         <f t="shared" si="29"/>
-        <v>1819.6423076923081</v>
+        <v>1836.4127218934905</v>
       </c>
       <c r="Q65" s="69">
         <f t="shared" si="29"/>
-        <v>1913.9307692307698</v>
+        <v>1952.612721893491</v>
       </c>
       <c r="R65" s="69">
         <f t="shared" si="29"/>
-        <v>1940.4230769230769</v>
+        <v>1989.5819526627222</v>
       </c>
       <c r="S65" s="69">
         <f t="shared" si="29"/>
-        <v>1963.0888888888896</v>
+        <v>1962.2603988603978</v>
       </c>
       <c r="T65" s="69">
         <f t="shared" si="29"/>
-        <v>2160.415384615384</v>
+        <v>1305.028106508875</v>
       </c>
       <c r="U65" s="69">
         <f t="shared" si="29"/>
-        <v>2161.1538461538462</v>
+        <v>1924.3204142011818</v>
       </c>
       <c r="V65" s="69">
         <v>0</v>
@@ -31135,47 +31194,47 @@
       <c r="B2" s="46"/>
       <c r="C2" s="34">
         <f>SUM(C4:C733)</f>
-        <v>126598.56000000003</v>
+        <v>134099.62000000002</v>
       </c>
       <c r="D2" s="35">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>127301.54000000002</v>
+        <v>135150.58000000005</v>
       </c>
       <c r="E2" s="36">
         <f t="shared" si="0"/>
-        <v>24114.696923076925</v>
+        <v>18755.875384615385</v>
       </c>
       <c r="F2" s="34">
         <f t="shared" si="0"/>
-        <v>193353.07699999993</v>
+        <v>199210.08699999994</v>
       </c>
       <c r="G2" s="35">
         <f t="shared" si="0"/>
-        <v>193320.75999999995</v>
+        <v>200023.69999999995</v>
       </c>
       <c r="H2" s="36">
         <f t="shared" si="0"/>
-        <v>41455.00615384613</v>
+        <v>30149.095384615372</v>
       </c>
       <c r="I2" s="34">
         <f t="shared" si="0"/>
-        <v>4381.3999999999996</v>
+        <v>7914.5999999999995</v>
       </c>
       <c r="J2" s="35">
         <f t="shared" si="0"/>
-        <v>3078.0459809999998</v>
+        <v>8744.0259809999989</v>
       </c>
       <c r="K2" s="36">
         <f t="shared" si="0"/>
-        <v>591000.00000000047</v>
+        <v>587000.00000000058</v>
       </c>
       <c r="L2" s="34">
         <f t="shared" si="0"/>
-        <v>318776.58249999984</v>
+        <v>327338.98249999981</v>
       </c>
       <c r="M2" s="36">
         <f t="shared" si="0"/>
-        <v>711087.49111538311</v>
+        <v>683919.90903846011</v>
       </c>
       <c r="N2" s="29"/>
     </row>
@@ -31375,7 +31434,7 @@
       </c>
       <c r="Y5" s="5">
         <f t="shared" si="2"/>
-        <v>43609.425980999993</v>
+        <v>63827.385980999999</v>
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
@@ -31462,7 +31521,7 @@
       </c>
       <c r="Y6" s="5">
         <f t="shared" si="4"/>
-        <v>30997.098461538462</v>
+        <v>10332.366153846153</v>
       </c>
       <c r="Z6" s="5">
         <f t="shared" si="4"/>
@@ -31589,7 +31648,7 @@
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="5"/>
-        <v>43427.1</v>
+        <v>51989.5</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="5"/>
@@ -31676,7 +31735,7 @@
       </c>
       <c r="Y9" s="5">
         <f t="shared" si="6"/>
-        <v>40751.373115384602</v>
+        <v>13583.791038461537</v>
       </c>
       <c r="Z9" s="5">
         <f t="shared" si="6"/>
@@ -31803,19 +31862,19 @@
       </c>
       <c r="Y11" s="5">
         <f t="shared" si="7"/>
-        <v>354697.44444253843</v>
+        <v>354250.6721348461</v>
       </c>
       <c r="Z11" s="5">
         <f t="shared" si="7"/>
-        <v>430270.04905792302</v>
+        <v>429823.2767502307</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="7"/>
-        <v>480270.04905792302</v>
+        <v>479823.2767502307</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="7"/>
-        <v>530270.04905792302</v>
+        <v>529823.2767502307</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
@@ -31890,19 +31949,19 @@
       </c>
       <c r="Y12" s="5">
         <f t="shared" si="8"/>
-        <v>359527.95561538462</v>
+        <v>340922.7735384616</v>
       </c>
       <c r="Z12" s="5">
         <f t="shared" si="8"/>
-        <v>428976.10861538467</v>
+        <v>410370.92653846159</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="8"/>
-        <v>496281.99361538462</v>
+        <v>477676.81153846154</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="8"/>
-        <v>532528.32861538464</v>
+        <v>513923.1465384615</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -31977,19 +32036,19 @@
       </c>
       <c r="Y13" s="5">
         <f t="shared" si="9"/>
-        <v>-4830.5111728461925</v>
+        <v>13327.898596384504</v>
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>1293.9404425383545</v>
+        <v>19452.35021176911</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
-        <v>-16011.944557461597</v>
+        <v>2146.4652117691585</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>-2258.2795574616175</v>
+        <v>15900.130211769196</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
@@ -42031,21 +42090,21 @@
         <v>326.87</v>
       </c>
       <c r="D265" s="40">
-        <v>959.83999999999992</v>
+        <v>1257.7800000000002</v>
       </c>
       <c r="E265" s="42"/>
       <c r="F265" s="39">
         <v>1184.44</v>
       </c>
       <c r="G265" s="40">
-        <v>1421.6600000000005</v>
+        <v>1739.9200000000003</v>
       </c>
       <c r="H265" s="42"/>
       <c r="I265" s="39">
         <v>0</v>
       </c>
       <c r="J265" s="40">
-        <v>247.56</v>
+        <v>386.03999999999996</v>
       </c>
       <c r="K265" s="5">
         <v>0</v>
@@ -42069,25 +42128,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C266" s="39"/>
-      <c r="D266" s="40"/>
-      <c r="E266" s="182">
-        <v>0</v>
-      </c>
-      <c r="F266" s="39"/>
-      <c r="G266" s="40"/>
-      <c r="H266" s="182">
-        <v>0</v>
-      </c>
-      <c r="I266" s="39"/>
-      <c r="J266" s="40"/>
+      <c r="C266" s="39">
+        <v>579.52</v>
+      </c>
+      <c r="D266" s="40">
+        <v>0</v>
+      </c>
+      <c r="E266" s="42"/>
+      <c r="F266" s="39">
+        <v>371.83</v>
+      </c>
+      <c r="G266" s="40">
+        <v>0</v>
+      </c>
+      <c r="H266" s="42"/>
+      <c r="I266" s="39">
+        <v>0</v>
+      </c>
+      <c r="J266" s="40">
+        <v>0</v>
+      </c>
       <c r="K266" s="5">
         <v>0</v>
       </c>
-      <c r="L266" s="157"/>
-      <c r="M266" s="41">
-        <v>0</v>
-      </c>
+      <c r="L266" s="157">
+        <v>0</v>
+      </c>
+      <c r="M266" s="41"/>
       <c r="O266" s="29"/>
       <c r="P266" s="5"/>
       <c r="R266" s="5"/>
@@ -42103,25 +42170,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C267" s="39"/>
-      <c r="D267" s="40"/>
-      <c r="E267" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F267" s="39"/>
-      <c r="G267" s="40"/>
-      <c r="H267" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I267" s="39"/>
-      <c r="J267" s="40"/>
+      <c r="C267" s="39">
+        <v>1302.97</v>
+      </c>
+      <c r="D267" s="40">
+        <v>1182</v>
+      </c>
+      <c r="E267" s="42"/>
+      <c r="F267" s="39">
+        <v>1303.3800000000001</v>
+      </c>
+      <c r="G267" s="40">
+        <v>1587.7200000000003</v>
+      </c>
+      <c r="H267" s="42"/>
+      <c r="I267" s="39">
+        <v>701</v>
+      </c>
+      <c r="J267" s="40">
+        <v>229.29000000000002</v>
+      </c>
       <c r="K267" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L267" s="157"/>
-      <c r="M267" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L267" s="157">
+        <v>0</v>
+      </c>
+      <c r="M267" s="41"/>
       <c r="O267" s="29"/>
       <c r="P267" s="5"/>
       <c r="R267" s="5"/>
@@ -42137,25 +42212,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C268" s="39"/>
-      <c r="D268" s="40"/>
-      <c r="E268" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F268" s="39"/>
-      <c r="G268" s="40"/>
-      <c r="H268" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I268" s="39"/>
-      <c r="J268" s="40"/>
+      <c r="C268" s="39">
+        <v>1342.58</v>
+      </c>
+      <c r="D268" s="40">
+        <v>1513.9599999999998</v>
+      </c>
+      <c r="E268" s="42"/>
+      <c r="F268" s="39">
+        <v>1002.13</v>
+      </c>
+      <c r="G268" s="40">
+        <v>1205.3000000000002</v>
+      </c>
+      <c r="H268" s="42"/>
+      <c r="I268" s="39">
+        <v>329</v>
+      </c>
+      <c r="J268" s="40">
+        <v>833.75000000000023</v>
+      </c>
       <c r="K268" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L268" s="157"/>
-      <c r="M268" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L268" s="157">
+        <v>3502.7999999999997</v>
+      </c>
+      <c r="M268" s="41"/>
       <c r="O268" s="29"/>
       <c r="P268" s="5"/>
       <c r="R268" s="5"/>
@@ -42171,25 +42254,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C269" s="39"/>
-      <c r="D269" s="40"/>
-      <c r="E269" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F269" s="39"/>
-      <c r="G269" s="40"/>
-      <c r="H269" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I269" s="39"/>
-      <c r="J269" s="40"/>
+      <c r="C269" s="39">
+        <v>1259.99</v>
+      </c>
+      <c r="D269" s="40">
+        <v>1340.1999999999996</v>
+      </c>
+      <c r="E269" s="42"/>
+      <c r="F269" s="39">
+        <v>1046.97</v>
+      </c>
+      <c r="G269" s="40">
+        <v>933.30000000000007</v>
+      </c>
+      <c r="H269" s="42"/>
+      <c r="I269" s="39">
+        <v>974</v>
+      </c>
+      <c r="J269" s="40">
+        <v>910.9699999999998</v>
+      </c>
       <c r="K269" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L269" s="157"/>
-      <c r="M269" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L269" s="157">
+        <v>0</v>
+      </c>
+      <c r="M269" s="41"/>
       <c r="O269" s="29"/>
       <c r="P269" s="5"/>
       <c r="R269" s="5"/>
@@ -42205,25 +42296,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C270" s="39"/>
-      <c r="D270" s="40"/>
-      <c r="E270" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F270" s="39"/>
-      <c r="G270" s="40"/>
-      <c r="H270" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I270" s="39"/>
-      <c r="J270" s="40"/>
+      <c r="C270" s="39">
+        <v>1408.16</v>
+      </c>
+      <c r="D270" s="40">
+        <v>1520.3400000000001</v>
+      </c>
+      <c r="E270" s="42"/>
+      <c r="F270" s="39">
+        <v>1481.03</v>
+      </c>
+      <c r="G270" s="40">
+        <v>1491.66</v>
+      </c>
+      <c r="H270" s="42"/>
+      <c r="I270" s="39">
+        <v>455</v>
+      </c>
+      <c r="J270" s="40">
+        <v>1356.5700000000004</v>
+      </c>
       <c r="K270" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L270" s="157"/>
-      <c r="M270" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L270" s="157">
+        <v>5059.5999999999995</v>
+      </c>
+      <c r="M270" s="41"/>
       <c r="O270" s="29"/>
       <c r="P270" s="5"/>
       <c r="R270" s="5"/>
@@ -42239,25 +42338,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C271" s="39"/>
-      <c r="D271" s="40"/>
-      <c r="E271" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F271" s="39"/>
-      <c r="G271" s="40"/>
-      <c r="H271" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I271" s="39"/>
-      <c r="J271" s="40"/>
+      <c r="C271" s="39">
+        <v>1289.48</v>
+      </c>
+      <c r="D271" s="40">
+        <v>855.98000000000025</v>
+      </c>
+      <c r="E271" s="42"/>
+      <c r="F271" s="39">
+        <v>651.66999999999996</v>
+      </c>
+      <c r="G271" s="40">
+        <v>924.04</v>
+      </c>
+      <c r="H271" s="42"/>
+      <c r="I271" s="39">
+        <v>567.20000000000005</v>
+      </c>
+      <c r="J271" s="40">
+        <v>1490.87</v>
+      </c>
       <c r="K271" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L271" s="157"/>
-      <c r="M271" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L271" s="157">
+        <v>0</v>
+      </c>
+      <c r="M271" s="41"/>
       <c r="O271" s="29"/>
       <c r="P271" s="5"/>
       <c r="R271" s="5"/>
@@ -42273,25 +42380,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C272" s="39"/>
-      <c r="D272" s="40"/>
-      <c r="E272" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F272" s="39"/>
-      <c r="G272" s="40"/>
-      <c r="H272" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I272" s="39"/>
-      <c r="J272" s="40"/>
+      <c r="C272" s="39">
+        <v>318.36</v>
+      </c>
+      <c r="D272" s="40">
+        <v>1138.6199999999997</v>
+      </c>
+      <c r="E272" s="42"/>
+      <c r="F272" s="39">
+        <v>0</v>
+      </c>
+      <c r="G272" s="40">
+        <v>242.66</v>
+      </c>
+      <c r="H272" s="42"/>
+      <c r="I272" s="39">
+        <v>507</v>
+      </c>
+      <c r="J272" s="40">
+        <v>706.05</v>
+      </c>
       <c r="K272" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L272" s="157"/>
-      <c r="M272" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L272" s="157">
+        <v>0</v>
+      </c>
+      <c r="M272" s="41"/>
       <c r="O272" s="29"/>
       <c r="P272" s="5"/>
       <c r="R272" s="5"/>
@@ -58147,7 +58262,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
@@ -58156,9 +58271,11 @@
     <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="164" t="s">
         <v>217</v>
       </c>
@@ -58202,7 +58319,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="166" t="s">
         <v>231</v>
       </c>
@@ -58240,14 +58357,28 @@
         <v>37087.89</v>
       </c>
       <c r="M2" s="72">
-        <v>20095.73</v>
+        <v>38572.915000000001</v>
       </c>
       <c r="N2" s="72">
-        <v>81878.399999999994</v>
+        <v>8562.24</v>
+      </c>
+      <c r="O2" s="29">
+        <f>M2-N2</f>
+        <v>30010.675000000003</v>
       </c>
       <c r="P2" s="29"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="S2">
+        <v>60</v>
+      </c>
+      <c r="T2">
+        <v>24</v>
+      </c>
+      <c r="U2">
+        <f>T2*S2</f>
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="166" t="s">
         <v>233</v>
       </c>
@@ -58285,15 +58416,21 @@
         <v>509033</v>
       </c>
       <c r="M3" s="72">
-        <v>285583</v>
+        <v>292226</v>
       </c>
       <c r="N3" s="72">
-        <v>167432</v>
-      </c>
-      <c r="O3" s="4"/>
+        <v>177188</v>
+      </c>
+      <c r="O3" s="29">
+        <f t="shared" ref="O3:O15" si="0">M3-N3</f>
+        <v>115038</v>
+      </c>
       <c r="P3" s="29"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="R3">
+        <v>5946</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="166" t="s">
         <v>235</v>
       </c>
@@ -58331,15 +58468,30 @@
         <v>2036132</v>
       </c>
       <c r="M4" s="72">
-        <v>1150458</v>
+        <v>1287858</v>
       </c>
       <c r="N4" s="72">
         <f>M3*4</f>
-        <v>1142332</v>
+        <v>1168904</v>
+      </c>
+      <c r="O4" s="29">
+        <f t="shared" si="0"/>
+        <v>118954</v>
       </c>
       <c r="P4" s="29"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="R4">
+        <v>9659</v>
+      </c>
+      <c r="V4" s="209">
+        <f>U2*R3</f>
+        <v>8562240</v>
+      </c>
+      <c r="W4" s="210">
+        <f>V4/1000</f>
+        <v>8562.24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="166" t="s">
         <v>236</v>
       </c>
@@ -58382,9 +58534,17 @@
       <c r="N5" s="72">
         <v>319386</v>
       </c>
+      <c r="O5" s="29">
+        <f t="shared" si="0"/>
+        <v>78289</v>
+      </c>
       <c r="P5" s="29"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="V5" s="209">
+        <f>U2*R4</f>
+        <v>13908960</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="166" t="s">
         <v>237</v>
       </c>
@@ -58427,9 +58587,13 @@
       <c r="N6" s="72">
         <v>642561</v>
       </c>
+      <c r="O6" s="29">
+        <f t="shared" si="0"/>
+        <v>153416</v>
+      </c>
       <c r="P6" s="29"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="166" t="s">
         <v>238</v>
       </c>
@@ -58472,9 +58636,13 @@
       <c r="N7" s="72">
         <v>557904</v>
       </c>
+      <c r="O7" s="29">
+        <f t="shared" si="0"/>
+        <v>192096</v>
+      </c>
       <c r="P7" s="29"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="166" t="s">
         <v>239</v>
       </c>
@@ -58515,9 +58683,13 @@
       <c r="N8" s="72">
         <v>962</v>
       </c>
+      <c r="O8" s="29">
+        <f t="shared" si="0"/>
+        <v>732</v>
+      </c>
       <c r="P8" s="29"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="166" t="s">
         <v>240</v>
       </c>
@@ -58560,9 +58732,13 @@
       <c r="N9" s="72">
         <v>3432</v>
       </c>
+      <c r="O9" s="29">
+        <f t="shared" si="0"/>
+        <v>3719</v>
+      </c>
       <c r="P9" s="29"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="166" t="s">
         <v>242</v>
       </c>
@@ -58605,9 +58781,13 @@
       <c r="N10" s="72">
         <v>7</v>
       </c>
+      <c r="O10" s="29">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
       <c r="P10" s="29"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="166" t="s">
         <v>243</v>
       </c>
@@ -58650,9 +58830,13 @@
       <c r="N11" s="72">
         <v>0</v>
       </c>
+      <c r="O11" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="P11" s="29"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="166" t="s">
         <v>244</v>
       </c>
@@ -58695,9 +58879,13 @@
       <c r="N12" s="72">
         <v>6</v>
       </c>
+      <c r="O12" s="29">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
       <c r="P12" s="29"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="166" t="s">
         <v>246</v>
       </c>
@@ -58740,9 +58928,13 @@
       <c r="N13" s="72">
         <v>0</v>
       </c>
+      <c r="O13" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="P13" s="29"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="166" t="s">
         <v>247</v>
       </c>
@@ -58785,9 +58977,13 @@
       <c r="N14" s="72">
         <v>483</v>
       </c>
+      <c r="O14" s="29">
+        <f t="shared" si="0"/>
+        <v>1109</v>
+      </c>
       <c r="P14" s="29"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="166" t="s">
         <v>249</v>
       </c>
@@ -58829,6 +59025,10 @@
       </c>
       <c r="N15" s="72">
         <v>309493.43</v>
+      </c>
+      <c r="O15" s="29">
+        <f t="shared" si="0"/>
+        <v>14842.780000000028</v>
       </c>
       <c r="P15" s="29"/>
     </row>
@@ -59024,7 +59224,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="173" t="s">
         <v>21</v>
       </c>
@@ -59047,7 +59247,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" s="173" t="s">
         <v>282</v>
       </c>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-29T14:36:54.654-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -3134,6 +3134,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3166,8 +3168,6 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4156,56 +4156,56 @@
   <sheetData>
     <row r="1" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="193" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="F2" s="194"/>
-      <c r="G2" s="194"/>
+      <c r="B2" s="195" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="196"/>
+      <c r="D2" s="196"/>
+      <c r="E2" s="196"/>
+      <c r="F2" s="196"/>
+      <c r="G2" s="196"/>
     </row>
     <row r="3" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="195" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="196"/>
-      <c r="D3" s="196"/>
-      <c r="E3" s="196"/>
-      <c r="F3" s="196"/>
-      <c r="G3" s="197"/>
+      <c r="B3" s="197" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="198"/>
+      <c r="D3" s="198"/>
+      <c r="E3" s="198"/>
+      <c r="F3" s="198"/>
+      <c r="G3" s="199"/>
     </row>
     <row r="4" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="198"/>
-      <c r="C4" s="194"/>
-      <c r="D4" s="194"/>
-      <c r="E4" s="194"/>
-      <c r="F4" s="194"/>
-      <c r="G4" s="199"/>
+      <c r="B4" s="200"/>
+      <c r="C4" s="196"/>
+      <c r="D4" s="196"/>
+      <c r="E4" s="196"/>
+      <c r="F4" s="196"/>
+      <c r="G4" s="201"/>
     </row>
     <row r="5" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="198"/>
-      <c r="C5" s="194"/>
-      <c r="D5" s="194"/>
-      <c r="E5" s="194"/>
-      <c r="F5" s="194"/>
-      <c r="G5" s="199"/>
+      <c r="B5" s="200"/>
+      <c r="C5" s="196"/>
+      <c r="D5" s="196"/>
+      <c r="E5" s="196"/>
+      <c r="F5" s="196"/>
+      <c r="G5" s="201"/>
     </row>
     <row r="6" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="198"/>
-      <c r="C6" s="194"/>
-      <c r="D6" s="194"/>
-      <c r="E6" s="194"/>
-      <c r="F6" s="194"/>
-      <c r="G6" s="199"/>
+      <c r="B6" s="200"/>
+      <c r="C6" s="196"/>
+      <c r="D6" s="196"/>
+      <c r="E6" s="196"/>
+      <c r="F6" s="196"/>
+      <c r="G6" s="201"/>
     </row>
     <row r="7" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="200"/>
-      <c r="C7" s="201"/>
-      <c r="D7" s="201"/>
-      <c r="E7" s="201"/>
-      <c r="F7" s="201"/>
-      <c r="G7" s="202"/>
+      <c r="B7" s="202"/>
+      <c r="C7" s="203"/>
+      <c r="D7" s="203"/>
+      <c r="E7" s="203"/>
+      <c r="F7" s="203"/>
+      <c r="G7" s="204"/>
     </row>
     <row r="8" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -12604,7 +12604,7 @@
       <c r="O34" s="15"/>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A35" s="203" t="s">
+      <c r="A35" s="205" t="s">
         <v>97</v>
       </c>
       <c r="B35" s="89">
@@ -12770,7 +12770,7 @@
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A36" s="204"/>
+      <c r="A36" s="206"/>
       <c r="B36" s="96" t="s">
         <v>63</v>
       </c>
@@ -20130,7 +20130,7 @@
       <c r="O80" s="15"/>
     </row>
     <row r="81" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A81" s="203" t="s">
+      <c r="A81" s="205" t="s">
         <v>140</v>
       </c>
       <c r="B81" s="89">
@@ -20296,7 +20296,7 @@
       </c>
     </row>
     <row r="82" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A82" s="205"/>
+      <c r="A82" s="207"/>
       <c r="B82" s="96" t="s">
         <v>63</v>
       </c>
@@ -21934,7 +21934,7 @@
       <c r="O91" s="15"/>
     </row>
     <row r="92" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A92" s="203" t="s">
+      <c r="A92" s="205" t="s">
         <v>145</v>
       </c>
       <c r="B92" s="89">
@@ -22100,7 +22100,7 @@
       </c>
     </row>
     <row r="93" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A93" s="204"/>
+      <c r="A93" s="206"/>
       <c r="B93" s="96" t="s">
         <v>63</v>
       </c>
@@ -29469,7 +29469,7 @@
         <v>0</v>
       </c>
       <c r="C40" s="69">
-        <f t="shared" ref="C40:I40" si="17">IFERROR(C38/C39,0)</f>
+        <f t="shared" ref="C40:H40" si="17">IFERROR(C38/C39,0)</f>
         <v>0</v>
       </c>
       <c r="D40" s="69">
@@ -58482,11 +58482,11 @@
       <c r="R4">
         <v>9659</v>
       </c>
-      <c r="V4" s="209">
+      <c r="V4" s="193">
         <f>U2*R3</f>
         <v>8562240</v>
       </c>
-      <c r="W4" s="210">
+      <c r="W4" s="194">
         <f>V4/1000</f>
         <v>8562.24</v>
       </c>
@@ -58539,7 +58539,7 @@
         <v>78289</v>
       </c>
       <c r="P5" s="29"/>
-      <c r="V5" s="209">
+      <c r="V5" s="193">
         <f>U2*R4</f>
         <v>13908960</v>
       </c>
@@ -59056,25 +59056,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="206" t="s">
+      <c r="A1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="206" t="s">
+      <c r="B1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="206" t="s">
+      <c r="C1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="206" t="s">
+      <c r="D1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="206" t="s">
+      <c r="E1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="F1" s="206" t="s">
+      <c r="F1" s="208" t="s">
         <v>251</v>
       </c>
-      <c r="G1" s="206" t="s">
+      <c r="G1" s="208" t="s">
         <v>251</v>
       </c>
     </row>
@@ -59609,43 +59609,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="207" t="s">
+      <c r="A1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="B1" s="207" t="s">
+      <c r="B1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="C1" s="207" t="s">
+      <c r="C1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="D1" s="207" t="s">
+      <c r="D1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="E1" s="207" t="s">
+      <c r="E1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="F1" s="207" t="s">
+      <c r="F1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="G1" s="207" t="s">
+      <c r="G1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="H1" s="207" t="s">
+      <c r="H1" s="209" t="s">
         <v>319</v>
       </c>
-      <c r="J1" s="208" t="s">
+      <c r="J1" s="210" t="s">
         <v>320</v>
       </c>
-      <c r="K1" s="208" t="s">
+      <c r="K1" s="210" t="s">
         <v>320</v>
       </c>
-      <c r="L1" s="208" t="s">
+      <c r="L1" s="210" t="s">
         <v>320</v>
       </c>
-      <c r="M1" s="208" t="s">
+      <c r="M1" s="210" t="s">
         <v>320</v>
       </c>
-      <c r="N1" s="208" t="s">
+      <c r="N1" s="210" t="s">
         <v>320</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-10-06T11:16:04.841-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="555" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{598D903D-53BA-4F67-BFC9-0EBCDF09814A}"/>
+  <xr:revisionPtr revIDLastSave="627" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{398F1562-B18C-4C03-900E-1425C63AF87C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
   </externalReferences>
-  <calcPr calcId="191028" iterate="1"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="396">
   <si>
     <t>ACOMPANHAMENTO SUPERESTRUTURA — FOLHA DE ENTRADA</t>
   </si>
@@ -4143,7 +4143,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:P61"/>
+  <dimension ref="B1:R61"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -4154,8 +4154,8 @@
     <col min="13" max="19" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:18" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="195" t="s">
         <v>0</v>
       </c>
@@ -4165,7 +4165,7 @@
       <c r="F2" s="196"/>
       <c r="G2" s="196"/>
     </row>
-    <row r="3" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="197" t="s">
         <v>1</v>
       </c>
@@ -4175,7 +4175,7 @@
       <c r="F3" s="198"/>
       <c r="G3" s="199"/>
     </row>
-    <row r="4" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="200"/>
       <c r="C4" s="196"/>
       <c r="D4" s="196"/>
@@ -4183,7 +4183,7 @@
       <c r="F4" s="196"/>
       <c r="G4" s="201"/>
     </row>
-    <row r="5" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="200"/>
       <c r="C5" s="196"/>
       <c r="D5" s="196"/>
@@ -4191,7 +4191,7 @@
       <c r="F5" s="196"/>
       <c r="G5" s="201"/>
     </row>
-    <row r="6" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="200"/>
       <c r="C6" s="196"/>
       <c r="D6" s="196"/>
@@ -4199,7 +4199,7 @@
       <c r="F6" s="196"/>
       <c r="G6" s="201"/>
     </row>
-    <row r="7" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="202"/>
       <c r="C7" s="203"/>
       <c r="D7" s="203"/>
@@ -4207,13 +4207,13 @@
       <c r="F7" s="203"/>
       <c r="G7" s="204"/>
     </row>
-    <row r="8" spans="2:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
@@ -4221,12 +4221,12 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="73" t="s">
         <v>5</v>
       </c>
@@ -4272,8 +4272,14 @@
       <c r="P13" s="75" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q13" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="R13" s="75" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="77" t="s">
         <v>8</v>
       </c>
@@ -4313,10 +4319,16 @@
       <c r="N14" s="79">
         <v>105184</v>
       </c>
-      <c r="O14" s="78"/>
-      <c r="P14" s="79"/>
-    </row>
-    <row r="15" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O14" s="78">
+        <v>108670</v>
+      </c>
+      <c r="P14" s="79">
+        <v>108940</v>
+      </c>
+      <c r="Q14" s="78"/>
+      <c r="R14" s="79"/>
+    </row>
+    <row r="15" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="77" t="s">
         <v>9</v>
       </c>
@@ -4338,8 +4350,10 @@
       <c r="N15" s="79"/>
       <c r="O15" s="78"/>
       <c r="P15" s="79"/>
-    </row>
-    <row r="16" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q15" s="78"/>
+      <c r="R15" s="79"/>
+    </row>
+    <row r="16" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="77" t="s">
         <v>10</v>
       </c>
@@ -4347,7 +4361,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="79">
-        <v>85240</v>
+        <v>91360</v>
       </c>
       <c r="E16" s="78"/>
       <c r="F16" s="79"/>
@@ -4361,8 +4375,10 @@
       <c r="N16" s="79"/>
       <c r="O16" s="78"/>
       <c r="P16" s="79"/>
-    </row>
-    <row r="17" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q16" s="78"/>
+      <c r="R16" s="79"/>
+    </row>
+    <row r="17" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="77" t="s">
         <v>11</v>
       </c>
@@ -4370,7 +4386,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="79">
-        <v>85220</v>
+        <v>91360</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79"/>
@@ -4384,8 +4400,10 @@
       <c r="N17" s="79"/>
       <c r="O17" s="78"/>
       <c r="P17" s="79"/>
-    </row>
-    <row r="18" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q17" s="78"/>
+      <c r="R17" s="79"/>
+    </row>
+    <row r="18" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="77" t="s">
         <v>12</v>
       </c>
@@ -4419,12 +4437,18 @@
       <c r="L18" s="79">
         <v>82860</v>
       </c>
-      <c r="M18" s="78"/>
-      <c r="N18" s="79"/>
+      <c r="M18" s="78">
+        <v>85400</v>
+      </c>
+      <c r="N18" s="79">
+        <v>86970</v>
+      </c>
       <c r="O18" s="78"/>
       <c r="P18" s="79"/>
-    </row>
-    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q18" s="78"/>
+      <c r="R18" s="79"/>
+    </row>
+    <row r="19" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="77" t="s">
         <v>13</v>
       </c>
@@ -4446,8 +4470,10 @@
       <c r="N19" s="79"/>
       <c r="O19" s="78"/>
       <c r="P19" s="79"/>
-    </row>
-    <row r="20" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q19" s="78"/>
+      <c r="R19" s="79"/>
+    </row>
+    <row r="20" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="77" t="s">
         <v>14</v>
       </c>
@@ -4475,14 +4501,20 @@
       <c r="J20" s="79">
         <v>75100</v>
       </c>
-      <c r="K20" s="78"/>
-      <c r="L20" s="79"/>
+      <c r="K20" s="78">
+        <v>77000</v>
+      </c>
+      <c r="L20" s="79">
+        <v>77400</v>
+      </c>
       <c r="M20" s="78"/>
       <c r="N20" s="79"/>
       <c r="O20" s="78"/>
       <c r="P20" s="79"/>
-    </row>
-    <row r="21" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q20" s="78"/>
+      <c r="R20" s="79"/>
+    </row>
+    <row r="21" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="77" t="s">
         <v>15</v>
       </c>
@@ -4496,7 +4528,7 @@
         <v>23000</v>
       </c>
       <c r="F21" s="79">
-        <v>32840</v>
+        <v>33700</v>
       </c>
       <c r="G21" s="78">
         <v>35000</v>
@@ -4520,7 +4552,7 @@
         <v>47030</v>
       </c>
       <c r="N21" s="79">
-        <v>48180</v>
+        <v>50000</v>
       </c>
       <c r="O21" s="78">
         <v>61300</v>
@@ -4528,8 +4560,14 @@
       <c r="P21" s="79">
         <v>61700</v>
       </c>
-    </row>
-    <row r="22" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q21" s="78">
+        <v>50040</v>
+      </c>
+      <c r="R21" s="79">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="77" t="s">
         <v>16</v>
       </c>
@@ -4551,8 +4589,10 @@
       <c r="N22" s="79"/>
       <c r="O22" s="78"/>
       <c r="P22" s="79"/>
-    </row>
-    <row r="23" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q22" s="78"/>
+      <c r="R22" s="79"/>
+    </row>
+    <row r="23" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="77" t="s">
         <v>17</v>
       </c>
@@ -4595,8 +4635,10 @@
       </c>
       <c r="O23" s="78"/>
       <c r="P23" s="79"/>
-    </row>
-    <row r="24" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q23" s="78"/>
+      <c r="R23" s="79"/>
+    </row>
+    <row r="24" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="77" t="s">
         <v>18</v>
       </c>
@@ -4622,8 +4664,10 @@
       <c r="N24" s="79"/>
       <c r="O24" s="78"/>
       <c r="P24" s="79"/>
-    </row>
-    <row r="25" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q24" s="78"/>
+      <c r="R24" s="79"/>
+    </row>
+    <row r="25" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="77" t="s">
         <v>19</v>
       </c>
@@ -4661,8 +4705,10 @@
       <c r="N25" s="79"/>
       <c r="O25" s="78"/>
       <c r="P25" s="79"/>
-    </row>
-    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q25" s="78"/>
+      <c r="R25" s="79"/>
+    </row>
+    <row r="26" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="77" t="s">
         <v>20</v>
       </c>
@@ -4688,8 +4734,10 @@
       <c r="N26" s="79"/>
       <c r="O26" s="78"/>
       <c r="P26" s="79"/>
-    </row>
-    <row r="27" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q26" s="78"/>
+      <c r="R26" s="79"/>
+    </row>
+    <row r="27" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="77" t="s">
         <v>21</v>
       </c>
@@ -4709,7 +4757,7 @@
         <v>23020</v>
       </c>
       <c r="H27" s="79">
-        <v>37020</v>
+        <v>40086</v>
       </c>
       <c r="I27" s="78"/>
       <c r="J27" s="79"/>
@@ -4719,13 +4767,15 @@
       <c r="N27" s="79"/>
       <c r="O27" s="78"/>
       <c r="P27" s="79"/>
-    </row>
-    <row r="29" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q27" s="78"/>
+      <c r="R27" s="79"/>
+    </row>
+    <row r="29" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
         <v>23</v>
       </c>
@@ -4733,12 +4783,12 @@
         <v>131260</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="191" t="s">
         <v>25</v>
       </c>
@@ -5109,7 +5159,7 @@
     <col min="25" max="39" width="9.140625" style="83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="82" t="s">
         <v>49</v>
       </c>
@@ -5137,7 +5187,7 @@
       <c r="W1" s="82"/>
       <c r="X1" s="82"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" s="84" t="s">
         <v>50</v>
       </c>
@@ -5211,7 +5261,7 @@
         <v>46661</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>51</v>
       </c>
@@ -5285,7 +5335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>52</v>
       </c>
@@ -5382,7 +5432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>53</v>
       </c>
@@ -5394,67 +5444,61 @@
       <c r="G5" s="61"/>
       <c r="H5" s="61"/>
       <c r="I5" s="61"/>
-      <c r="J5" s="62">
-        <f>J7</f>
-        <v>4.0500000000000008E-2</v>
-      </c>
-      <c r="K5" s="62">
-        <v>5.7221466803051929E-2</v>
-      </c>
+      <c r="J5" s="61"/>
+      <c r="K5" s="61"/>
       <c r="L5" s="62">
-        <f>L6-K6</f>
-        <v>7.1195414356986897E-2</v>
+        <v>6.781286847493076E-2</v>
       </c>
       <c r="M5" s="62">
         <f t="shared" ref="M5:X5" si="1">M6-L6</f>
-        <v>8.188176322115398E-2</v>
+        <v>8.2269783378556061E-2</v>
       </c>
       <c r="N5" s="62">
         <f t="shared" si="1"/>
-        <v>4.8233907822541167E-2</v>
+        <v>5.3316920765678344E-2</v>
       </c>
       <c r="O5" s="62">
         <f t="shared" si="1"/>
-        <v>5.7602435507203731E-2</v>
+        <v>5.6864394668070473E-2</v>
       </c>
       <c r="P5" s="62">
         <f t="shared" si="1"/>
-        <v>5.9597632283525326E-2</v>
+        <v>5.7008471646305681E-2</v>
       </c>
       <c r="Q5" s="62">
         <f t="shared" si="1"/>
-        <v>6.6399322145811235E-2</v>
+        <v>6.6847314390614532E-2</v>
       </c>
       <c r="R5" s="62">
         <f t="shared" si="1"/>
-        <v>6.337337741019422E-2</v>
+        <v>6.5773175848752863E-2</v>
       </c>
       <c r="S5" s="62">
         <f t="shared" si="1"/>
-        <v>6.5918181443970547E-2</v>
+        <v>6.5830462848880944E-2</v>
       </c>
       <c r="T5" s="62">
         <f t="shared" si="1"/>
-        <v>7.6648971764140539E-2</v>
+        <v>7.5938391684603368E-2</v>
       </c>
       <c r="U5" s="62">
         <f t="shared" si="1"/>
-        <v>5.8794301524071946E-2</v>
+        <v>5.9193922251732256E-2</v>
       </c>
       <c r="V5" s="62">
         <f t="shared" si="1"/>
-        <v>5.350472654669014E-2</v>
+        <v>5.5645243385036958E-2</v>
       </c>
       <c r="W5" s="62">
         <f t="shared" si="1"/>
-        <v>5.3740477450843316E-2</v>
+        <v>5.5815010446328528E-2</v>
       </c>
       <c r="X5" s="62">
         <f t="shared" si="1"/>
-        <v>4.4939541135864403E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+        <v>4.743998030764196E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>54</v>
       </c>
@@ -5466,54 +5510,52 @@
       <c r="G6" s="61"/>
       <c r="H6" s="61"/>
       <c r="I6" s="61"/>
-      <c r="J6" s="62">
-        <f>J8</f>
-        <v>0.18110000000000001</v>
-      </c>
-      <c r="K6" s="62">
-        <v>0.23861553440928052</v>
-      </c>
+      <c r="J6" s="61"/>
+      <c r="K6" s="61"/>
       <c r="L6" s="62">
-        <v>0.30981094876626741</v>
+        <v>0.30051286847493075</v>
       </c>
       <c r="M6" s="62">
-        <v>0.39169271198742139</v>
+        <v>0.38278265185348681</v>
       </c>
       <c r="N6" s="62">
-        <v>0.43992661980996256</v>
+        <v>0.43609957261916515</v>
       </c>
       <c r="O6" s="62">
-        <v>0.49752905531716629</v>
+        <v>0.49296396728723563</v>
       </c>
       <c r="P6" s="62">
-        <v>0.55712668760069162</v>
+        <v>0.54997243893354131</v>
       </c>
       <c r="Q6" s="62">
-        <v>0.62352600974650285</v>
+        <v>0.61681975332415584</v>
       </c>
       <c r="R6" s="62">
-        <v>0.68689938715669707</v>
+        <v>0.6825929291729087</v>
       </c>
       <c r="S6" s="62">
-        <v>0.75281756860066762</v>
+        <v>0.74842339202178965</v>
       </c>
       <c r="T6" s="62">
-        <v>0.82946654036480816</v>
+        <v>0.82436178370639301</v>
       </c>
       <c r="U6" s="62">
-        <v>0.8882608418888801</v>
+        <v>0.88355570595812527</v>
       </c>
       <c r="V6" s="62">
-        <v>0.94176556843557024</v>
+        <v>0.93920094934316223</v>
       </c>
       <c r="W6" s="62">
-        <v>0.99550604588641356</v>
+        <v>0.99501595978949076</v>
       </c>
       <c r="X6" s="62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+        <v>0.99975995782025495</v>
+      </c>
+      <c r="Y6" s="83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>55</v>
       </c>
@@ -5541,13 +5583,15 @@
       <c r="I7" s="61">
         <v>5.6300000000000003E-2</v>
       </c>
-      <c r="J7" s="62">
-        <v>4.0500000000000008E-2</v>
-      </c>
-      <c r="K7" s="62">
-        <v>4.3200000000000016E-2</v>
-      </c>
-      <c r="L7" s="62"/>
+      <c r="J7" s="61">
+        <v>4.4499999999999984E-2</v>
+      </c>
+      <c r="K7" s="61">
+        <v>4.7600000000000003E-2</v>
+      </c>
+      <c r="L7" s="62">
+        <v>3.2000000000000084E-3</v>
+      </c>
       <c r="M7" s="62"/>
       <c r="N7" s="62"/>
       <c r="O7" s="62"/>
@@ -5561,7 +5605,7 @@
       <c r="W7" s="62"/>
       <c r="X7" s="62"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>56</v>
       </c>
@@ -5574,7 +5618,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="61">
-        <f t="shared" ref="D8:K8" si="2">D7+C8</f>
+        <f t="shared" ref="D8:L8" si="2">D7+C8</f>
         <v>1.1000000000000001E-3</v>
       </c>
       <c r="E8" s="61">
@@ -5597,15 +5641,18 @@
         <f t="shared" si="2"/>
         <v>0.1406</v>
       </c>
-      <c r="J8" s="62">
+      <c r="J8" s="61">
         <f t="shared" si="2"/>
-        <v>0.18110000000000001</v>
-      </c>
-      <c r="K8" s="62">
+        <v>0.18509999999999999</v>
+      </c>
+      <c r="K8" s="61">
         <f t="shared" si="2"/>
-        <v>0.22430000000000003</v>
-      </c>
-      <c r="L8" s="62"/>
+        <v>0.23269999999999999</v>
+      </c>
+      <c r="L8" s="62">
+        <f t="shared" si="2"/>
+        <v>0.2359</v>
+      </c>
       <c r="M8" s="62"/>
       <c r="N8" s="62"/>
       <c r="O8" s="62"/>
@@ -5619,7 +5666,7 @@
       <c r="W8" s="62"/>
       <c r="X8" s="62"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="82" t="s">
         <v>57</v>
       </c>
@@ -5647,7 +5694,7 @@
       <c r="W10" s="82"/>
       <c r="X10" s="82"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="84" t="s">
         <v>50</v>
       </c>
@@ -5721,7 +5768,7 @@
         <v>46661</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>51</v>
       </c>
@@ -5795,7 +5842,7 @@
         <v>7.7828947696293024E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>52</v>
       </c>
@@ -5869,7 +5916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>53</v>
       </c>
@@ -5925,7 +5972,7 @@
       </c>
       <c r="X14" s="62"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>54</v>
       </c>
@@ -5998,7 +6045,7 @@
         <v>1.0032697079852295</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>55</v>
       </c>
@@ -7484,7 +7531,9 @@
       <c r="V3" s="9">
         <v>5</v>
       </c>
-      <c r="W3" s="10"/>
+      <c r="W3" s="10">
+        <v>1</v>
+      </c>
       <c r="X3" s="9">
         <v>5</v>
       </c>
@@ -7648,7 +7697,9 @@
       <c r="V4" s="102">
         <v>96</v>
       </c>
-      <c r="W4" s="103"/>
+      <c r="W4" s="103">
+        <v>48</v>
+      </c>
       <c r="X4" s="102">
         <v>96</v>
       </c>
@@ -7972,7 +8023,9 @@
       <c r="V6" s="102">
         <v>3</v>
       </c>
-      <c r="W6" s="103"/>
+      <c r="W6" s="103">
+        <v>2</v>
+      </c>
       <c r="X6" s="102">
         <v>2</v>
       </c>
@@ -8136,7 +8189,9 @@
       <c r="V7" s="12">
         <v>8</v>
       </c>
-      <c r="W7" s="13"/>
+      <c r="W7" s="13">
+        <v>6</v>
+      </c>
       <c r="X7" s="12">
         <v>8</v>
       </c>
@@ -8300,7 +8355,9 @@
       <c r="V8" s="102">
         <v>4</v>
       </c>
-      <c r="W8" s="103"/>
+      <c r="W8" s="103">
+        <v>5</v>
+      </c>
       <c r="X8" s="102">
         <v>4</v>
       </c>
@@ -8464,7 +8521,9 @@
       <c r="V9" s="12">
         <v>5</v>
       </c>
-      <c r="W9" s="13"/>
+      <c r="W9" s="13">
+        <v>4</v>
+      </c>
       <c r="X9" s="12">
         <v>5</v>
       </c>
@@ -8628,7 +8687,9 @@
       <c r="V10" s="102">
         <v>1</v>
       </c>
-      <c r="W10" s="103"/>
+      <c r="W10" s="103">
+        <v>1</v>
+      </c>
       <c r="X10" s="102">
         <v>1</v>
       </c>
@@ -8950,7 +9011,9 @@
       <c r="V12" s="102">
         <v>3</v>
       </c>
-      <c r="W12" s="103"/>
+      <c r="W12" s="103">
+        <v>3</v>
+      </c>
       <c r="X12" s="102">
         <v>3</v>
       </c>
@@ -9114,7 +9177,9 @@
       <c r="V13" s="12">
         <v>5</v>
       </c>
-      <c r="W13" s="13"/>
+      <c r="W13" s="13">
+        <v>5</v>
+      </c>
       <c r="X13" s="12">
         <v>5</v>
       </c>
@@ -9278,7 +9343,9 @@
       <c r="V14" s="102">
         <v>2</v>
       </c>
-      <c r="W14" s="103"/>
+      <c r="W14" s="103">
+        <v>1</v>
+      </c>
       <c r="X14" s="102">
         <v>2</v>
       </c>
@@ -9604,7 +9671,9 @@
       <c r="V16" s="102">
         <v>8</v>
       </c>
-      <c r="W16" s="103"/>
+      <c r="W16" s="103">
+        <v>8</v>
+      </c>
       <c r="X16" s="102">
         <v>8</v>
       </c>
@@ -9768,7 +9837,9 @@
       <c r="V17" s="12">
         <v>23</v>
       </c>
-      <c r="W17" s="13"/>
+      <c r="W17" s="13">
+        <v>63</v>
+      </c>
       <c r="X17" s="12">
         <v>23</v>
       </c>
@@ -9932,7 +10003,9 @@
       <c r="V18" s="102">
         <v>2</v>
       </c>
-      <c r="W18" s="103"/>
+      <c r="W18" s="103">
+        <v>3</v>
+      </c>
       <c r="X18" s="102">
         <v>2</v>
       </c>
@@ -10096,7 +10169,9 @@
       <c r="V19" s="12">
         <v>22</v>
       </c>
-      <c r="W19" s="13"/>
+      <c r="W19" s="13">
+        <v>23</v>
+      </c>
       <c r="X19" s="12">
         <v>22</v>
       </c>
@@ -10260,7 +10335,9 @@
       <c r="V20" s="102">
         <v>18</v>
       </c>
-      <c r="W20" s="103"/>
+      <c r="W20" s="103">
+        <v>18</v>
+      </c>
       <c r="X20" s="102">
         <v>18</v>
       </c>
@@ -10424,7 +10501,9 @@
       <c r="V21" s="12">
         <v>3</v>
       </c>
-      <c r="W21" s="13"/>
+      <c r="W21" s="13">
+        <v>3</v>
+      </c>
       <c r="X21" s="12">
         <v>2</v>
       </c>
@@ -10588,7 +10667,9 @@
       <c r="V22" s="102">
         <v>3</v>
       </c>
-      <c r="W22" s="103"/>
+      <c r="W22" s="103">
+        <v>10</v>
+      </c>
       <c r="X22" s="102">
         <v>2</v>
       </c>
@@ -10752,7 +10833,9 @@
       <c r="V23" s="12">
         <v>4</v>
       </c>
-      <c r="W23" s="13"/>
+      <c r="W23" s="13">
+        <v>2</v>
+      </c>
       <c r="X23" s="12">
         <v>4</v>
       </c>
@@ -10914,7 +10997,9 @@
       <c r="V24" s="102">
         <v>6</v>
       </c>
-      <c r="W24" s="103"/>
+      <c r="W24" s="103">
+        <v>4</v>
+      </c>
       <c r="X24" s="102">
         <v>6</v>
       </c>
@@ -11078,7 +11163,9 @@
       <c r="V25" s="12">
         <v>8</v>
       </c>
-      <c r="W25" s="13"/>
+      <c r="W25" s="13">
+        <v>1</v>
+      </c>
       <c r="X25" s="12">
         <v>8</v>
       </c>
@@ -11402,7 +11489,9 @@
       <c r="V27" s="12">
         <v>8</v>
       </c>
-      <c r="W27" s="13"/>
+      <c r="W27" s="13">
+        <v>4</v>
+      </c>
       <c r="X27" s="12">
         <v>8</v>
       </c>
@@ -11566,7 +11655,9 @@
       <c r="V28" s="102">
         <v>2</v>
       </c>
-      <c r="W28" s="103"/>
+      <c r="W28" s="103">
+        <v>4</v>
+      </c>
       <c r="X28" s="102">
         <v>2</v>
       </c>
@@ -11730,7 +11821,9 @@
       <c r="V29" s="12">
         <v>1</v>
       </c>
-      <c r="W29" s="13"/>
+      <c r="W29" s="13">
+        <v>1</v>
+      </c>
       <c r="X29" s="12">
         <v>1</v>
       </c>
@@ -11894,7 +11987,9 @@
       <c r="V30" s="102">
         <v>1</v>
       </c>
-      <c r="W30" s="103"/>
+      <c r="W30" s="103">
+        <v>1</v>
+      </c>
       <c r="X30" s="102">
         <v>1</v>
       </c>
@@ -12058,7 +12153,9 @@
       <c r="V31" s="12">
         <v>2</v>
       </c>
-      <c r="W31" s="13"/>
+      <c r="W31" s="13">
+        <v>2</v>
+      </c>
       <c r="X31" s="12">
         <v>2</v>
       </c>
@@ -12222,7 +12319,9 @@
       <c r="V32" s="107">
         <v>3</v>
       </c>
-      <c r="W32" s="108"/>
+      <c r="W32" s="108">
+        <v>4</v>
+      </c>
       <c r="X32" s="107">
         <v>3</v>
       </c>
@@ -12409,7 +12508,7 @@
       </c>
       <c r="W33" s="113">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>227</v>
       </c>
       <c r="X33" s="113">
         <f t="shared" si="8"/>
@@ -13046,7 +13145,9 @@
       <c r="V37" s="9">
         <v>3</v>
       </c>
-      <c r="W37" s="10"/>
+      <c r="W37" s="10">
+        <v>6</v>
+      </c>
       <c r="X37" s="9">
         <v>3</v>
       </c>
@@ -13210,7 +13311,9 @@
       <c r="V38" s="102">
         <v>1</v>
       </c>
-      <c r="W38" s="103"/>
+      <c r="W38" s="103">
+        <v>1</v>
+      </c>
       <c r="X38" s="102">
         <v>1</v>
       </c>
@@ -13374,7 +13477,9 @@
       <c r="V39" s="12">
         <v>2</v>
       </c>
-      <c r="W39" s="13"/>
+      <c r="W39" s="13">
+        <v>1</v>
+      </c>
       <c r="X39" s="12">
         <v>2</v>
       </c>
@@ -13698,7 +13803,9 @@
       <c r="V41" s="12">
         <v>3</v>
       </c>
-      <c r="W41" s="13"/>
+      <c r="W41" s="13">
+        <v>3</v>
+      </c>
       <c r="X41" s="12">
         <v>3</v>
       </c>
@@ -14022,7 +14129,9 @@
       <c r="V43" s="12">
         <v>4</v>
       </c>
-      <c r="W43" s="13"/>
+      <c r="W43" s="13">
+        <v>2</v>
+      </c>
       <c r="X43" s="12">
         <v>4</v>
       </c>
@@ -14186,7 +14295,9 @@
       <c r="V44" s="102">
         <v>16</v>
       </c>
-      <c r="W44" s="103"/>
+      <c r="W44" s="103">
+        <v>11</v>
+      </c>
       <c r="X44" s="102">
         <v>15</v>
       </c>
@@ -14348,7 +14459,9 @@
       <c r="V45" s="12">
         <v>2</v>
       </c>
-      <c r="W45" s="13"/>
+      <c r="W45" s="13">
+        <v>1</v>
+      </c>
       <c r="X45" s="12">
         <v>2</v>
       </c>
@@ -14512,7 +14625,9 @@
       <c r="V46" s="102">
         <v>6</v>
       </c>
-      <c r="W46" s="103"/>
+      <c r="W46" s="103">
+        <v>5</v>
+      </c>
       <c r="X46" s="102">
         <v>5</v>
       </c>
@@ -14676,7 +14791,9 @@
       <c r="V47" s="12">
         <v>1</v>
       </c>
-      <c r="W47" s="13"/>
+      <c r="W47" s="13">
+        <v>2</v>
+      </c>
       <c r="X47" s="12">
         <v>1</v>
       </c>
@@ -14840,7 +14957,9 @@
       <c r="V48" s="102">
         <v>2</v>
       </c>
-      <c r="W48" s="103"/>
+      <c r="W48" s="103">
+        <v>2</v>
+      </c>
       <c r="X48" s="102">
         <v>2</v>
       </c>
@@ -15004,7 +15123,9 @@
       <c r="V49" s="12">
         <v>1</v>
       </c>
-      <c r="W49" s="13"/>
+      <c r="W49" s="13">
+        <v>2</v>
+      </c>
       <c r="X49" s="12">
         <v>1</v>
       </c>
@@ -15168,7 +15289,9 @@
       <c r="V50" s="102">
         <v>2</v>
       </c>
-      <c r="W50" s="103"/>
+      <c r="W50" s="103">
+        <v>1</v>
+      </c>
       <c r="X50" s="102">
         <v>2</v>
       </c>
@@ -15332,7 +15455,9 @@
       <c r="V51" s="12">
         <v>1</v>
       </c>
-      <c r="W51" s="13"/>
+      <c r="W51" s="13">
+        <v>1</v>
+      </c>
       <c r="X51" s="12">
         <v>1</v>
       </c>
@@ -15496,7 +15621,9 @@
       <c r="V52" s="102">
         <v>1</v>
       </c>
-      <c r="W52" s="103"/>
+      <c r="W52" s="103">
+        <v>1</v>
+      </c>
       <c r="X52" s="102">
         <v>1</v>
       </c>
@@ -15660,7 +15787,9 @@
       <c r="V53" s="12">
         <v>1</v>
       </c>
-      <c r="W53" s="13"/>
+      <c r="W53" s="13">
+        <v>1</v>
+      </c>
       <c r="X53" s="12">
         <v>1</v>
       </c>
@@ -15824,7 +15953,9 @@
       <c r="V54" s="102">
         <v>2</v>
       </c>
-      <c r="W54" s="103"/>
+      <c r="W54" s="103">
+        <v>5</v>
+      </c>
       <c r="X54" s="102">
         <v>2</v>
       </c>
@@ -15988,7 +16119,9 @@
       <c r="V55" s="12">
         <v>1</v>
       </c>
-      <c r="W55" s="13"/>
+      <c r="W55" s="13">
+        <v>1</v>
+      </c>
       <c r="X55" s="12">
         <v>1</v>
       </c>
@@ -16152,7 +16285,9 @@
       <c r="V56" s="102">
         <v>1</v>
       </c>
-      <c r="W56" s="103"/>
+      <c r="W56" s="103">
+        <v>1</v>
+      </c>
       <c r="X56" s="102">
         <v>1</v>
       </c>
@@ -16316,7 +16451,9 @@
       <c r="V57" s="12">
         <v>1</v>
       </c>
-      <c r="W57" s="13"/>
+      <c r="W57" s="13">
+        <v>2</v>
+      </c>
       <c r="X57" s="12">
         <v>1</v>
       </c>
@@ -16480,7 +16617,9 @@
       <c r="V58" s="102">
         <v>1</v>
       </c>
-      <c r="W58" s="103"/>
+      <c r="W58" s="103">
+        <v>1</v>
+      </c>
       <c r="X58" s="102">
         <v>1</v>
       </c>
@@ -16644,7 +16783,9 @@
       <c r="V59" s="12">
         <v>2</v>
       </c>
-      <c r="W59" s="13"/>
+      <c r="W59" s="13">
+        <v>2</v>
+      </c>
       <c r="X59" s="12">
         <v>2</v>
       </c>
@@ -16808,7 +16949,9 @@
       <c r="V60" s="102">
         <v>3</v>
       </c>
-      <c r="W60" s="103"/>
+      <c r="W60" s="103">
+        <v>4</v>
+      </c>
       <c r="X60" s="102">
         <v>3</v>
       </c>
@@ -16970,7 +17113,9 @@
       <c r="V61" s="12">
         <v>2</v>
       </c>
-      <c r="W61" s="13"/>
+      <c r="W61" s="13">
+        <v>2</v>
+      </c>
       <c r="X61" s="12">
         <v>2</v>
       </c>
@@ -17132,7 +17277,9 @@
       <c r="V62" s="102">
         <v>2</v>
       </c>
-      <c r="W62" s="103"/>
+      <c r="W62" s="103">
+        <v>2</v>
+      </c>
       <c r="X62" s="102">
         <v>2</v>
       </c>
@@ -17296,7 +17443,9 @@
       <c r="V63" s="12">
         <v>2</v>
       </c>
-      <c r="W63" s="13"/>
+      <c r="W63" s="13">
+        <v>9</v>
+      </c>
       <c r="X63" s="12">
         <v>2</v>
       </c>
@@ -17460,7 +17609,9 @@
       <c r="V64" s="102">
         <v>1</v>
       </c>
-      <c r="W64" s="103"/>
+      <c r="W64" s="103">
+        <v>1</v>
+      </c>
       <c r="X64" s="102">
         <v>1</v>
       </c>
@@ -17624,7 +17775,9 @@
       <c r="V65" s="12">
         <v>3</v>
       </c>
-      <c r="W65" s="13"/>
+      <c r="W65" s="13">
+        <v>3</v>
+      </c>
       <c r="X65" s="12">
         <v>3</v>
       </c>
@@ -17788,7 +17941,9 @@
       <c r="V66" s="102">
         <v>8</v>
       </c>
-      <c r="W66" s="103"/>
+      <c r="W66" s="103">
+        <v>12</v>
+      </c>
       <c r="X66" s="102">
         <v>8</v>
       </c>
@@ -17952,7 +18107,9 @@
       <c r="V67" s="12">
         <v>8</v>
       </c>
-      <c r="W67" s="13"/>
+      <c r="W67" s="13">
+        <v>12</v>
+      </c>
       <c r="X67" s="12">
         <v>8</v>
       </c>
@@ -18116,7 +18273,9 @@
       <c r="V68" s="102">
         <v>3</v>
       </c>
-      <c r="W68" s="103"/>
+      <c r="W68" s="103">
+        <v>3</v>
+      </c>
       <c r="X68" s="102">
         <v>2</v>
       </c>
@@ -18278,7 +18437,9 @@
       <c r="V69" s="12">
         <v>1</v>
       </c>
-      <c r="W69" s="13"/>
+      <c r="W69" s="13">
+        <v>1</v>
+      </c>
       <c r="X69" s="12">
         <v>1</v>
       </c>
@@ -18602,7 +18763,9 @@
       <c r="V71" s="12">
         <v>2</v>
       </c>
-      <c r="W71" s="13"/>
+      <c r="W71" s="13">
+        <v>1</v>
+      </c>
       <c r="X71" s="12">
         <v>2</v>
       </c>
@@ -18766,7 +18929,9 @@
       <c r="V72" s="102">
         <v>1</v>
       </c>
-      <c r="W72" s="103"/>
+      <c r="W72" s="103">
+        <v>1</v>
+      </c>
       <c r="X72" s="102">
         <v>1</v>
       </c>
@@ -18930,7 +19095,9 @@
       <c r="V73" s="12">
         <v>1</v>
       </c>
-      <c r="W73" s="13"/>
+      <c r="W73" s="13">
+        <v>1</v>
+      </c>
       <c r="X73" s="12">
         <v>1</v>
       </c>
@@ -19094,7 +19261,9 @@
       <c r="V74" s="102">
         <v>1</v>
       </c>
-      <c r="W74" s="103"/>
+      <c r="W74" s="103">
+        <v>2</v>
+      </c>
       <c r="X74" s="102">
         <v>1</v>
       </c>
@@ -19258,7 +19427,9 @@
       <c r="V75" s="12">
         <v>3</v>
       </c>
-      <c r="W75" s="13"/>
+      <c r="W75" s="13">
+        <v>3</v>
+      </c>
       <c r="X75" s="12">
         <v>3</v>
       </c>
@@ -19422,7 +19593,9 @@
       <c r="V76" s="102">
         <v>6</v>
       </c>
-      <c r="W76" s="103"/>
+      <c r="W76" s="103">
+        <v>7</v>
+      </c>
       <c r="X76" s="102">
         <v>6</v>
       </c>
@@ -19584,7 +19757,9 @@
       <c r="V77" s="12">
         <v>1</v>
       </c>
-      <c r="W77" s="13"/>
+      <c r="W77" s="13">
+        <v>1</v>
+      </c>
       <c r="X77" s="12">
         <v>1</v>
       </c>
@@ -19748,7 +19923,9 @@
       <c r="V78" s="107">
         <v>1</v>
       </c>
-      <c r="W78" s="108"/>
+      <c r="W78" s="108">
+        <v>1</v>
+      </c>
       <c r="X78" s="107">
         <v>1</v>
       </c>
@@ -19935,7 +20112,7 @@
       </c>
       <c r="W79" s="112">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="X79" s="112">
         <f t="shared" si="18"/>
@@ -20572,7 +20749,9 @@
       <c r="V83" s="9">
         <v>2</v>
       </c>
-      <c r="W83" s="10"/>
+      <c r="W83" s="10">
+        <v>27</v>
+      </c>
       <c r="X83" s="9">
         <v>2</v>
       </c>
@@ -20736,7 +20915,9 @@
       <c r="V84" s="102">
         <v>12</v>
       </c>
-      <c r="W84" s="103"/>
+      <c r="W84" s="103">
+        <v>5</v>
+      </c>
       <c r="X84" s="102">
         <v>12</v>
       </c>
@@ -21060,7 +21241,9 @@
       <c r="V86" s="102">
         <v>1</v>
       </c>
-      <c r="W86" s="103"/>
+      <c r="W86" s="103">
+        <v>2</v>
+      </c>
       <c r="X86" s="102">
         <v>1</v>
       </c>
@@ -21224,7 +21407,9 @@
       <c r="V87" s="12">
         <v>1</v>
       </c>
-      <c r="W87" s="13"/>
+      <c r="W87" s="13">
+        <v>1</v>
+      </c>
       <c r="X87" s="12">
         <v>1</v>
       </c>
@@ -21388,7 +21573,9 @@
       <c r="V88" s="102">
         <v>8</v>
       </c>
-      <c r="W88" s="103"/>
+      <c r="W88" s="103">
+        <v>11</v>
+      </c>
       <c r="X88" s="102">
         <v>8</v>
       </c>
@@ -21552,7 +21739,9 @@
       <c r="V89" s="17">
         <v>3</v>
       </c>
-      <c r="W89" s="18"/>
+      <c r="W89" s="18">
+        <v>3</v>
+      </c>
       <c r="X89" s="17">
         <v>3</v>
       </c>
@@ -21739,7 +21928,7 @@
       </c>
       <c r="W90" s="112">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="X90" s="112">
         <f t="shared" si="28"/>
@@ -22376,7 +22565,9 @@
       <c r="V94" s="122">
         <v>3</v>
       </c>
-      <c r="W94" s="123"/>
+      <c r="W94" s="123">
+        <v>7</v>
+      </c>
       <c r="X94" s="122">
         <v>3</v>
       </c>
@@ -22540,7 +22731,9 @@
       <c r="V95" s="12">
         <v>5</v>
       </c>
-      <c r="W95" s="13"/>
+      <c r="W95" s="13">
+        <v>5</v>
+      </c>
       <c r="X95" s="12">
         <v>5</v>
       </c>
@@ -22704,7 +22897,9 @@
       <c r="V96" s="102">
         <v>5</v>
       </c>
-      <c r="W96" s="103"/>
+      <c r="W96" s="103">
+        <v>6</v>
+      </c>
       <c r="X96" s="102">
         <v>5</v>
       </c>
@@ -22868,7 +23063,9 @@
       <c r="V97" s="12">
         <v>2</v>
       </c>
-      <c r="W97" s="13"/>
+      <c r="W97" s="13">
+        <v>1</v>
+      </c>
       <c r="X97" s="12">
         <v>2</v>
       </c>
@@ -23032,7 +23229,9 @@
       <c r="V98" s="102">
         <v>1</v>
       </c>
-      <c r="W98" s="103"/>
+      <c r="W98" s="103">
+        <v>1</v>
+      </c>
       <c r="X98" s="102">
         <v>1</v>
       </c>
@@ -23196,7 +23395,9 @@
       <c r="V99" s="12">
         <v>1</v>
       </c>
-      <c r="W99" s="13"/>
+      <c r="W99" s="13">
+        <v>2</v>
+      </c>
       <c r="X99" s="12">
         <v>1</v>
       </c>
@@ -23360,7 +23561,9 @@
       <c r="V100" s="127">
         <v>0</v>
       </c>
-      <c r="W100" s="66"/>
+      <c r="W100" s="66">
+        <v>7</v>
+      </c>
       <c r="X100" s="127">
         <v>0</v>
       </c>
@@ -23524,7 +23727,9 @@
       <c r="V101" s="12">
         <v>1</v>
       </c>
-      <c r="W101" s="13"/>
+      <c r="W101" s="13">
+        <v>1</v>
+      </c>
       <c r="X101" s="12">
         <v>1</v>
       </c>
@@ -23688,7 +23893,9 @@
       <c r="V102" s="102">
         <v>2</v>
       </c>
-      <c r="W102" s="103"/>
+      <c r="W102" s="103">
+        <v>2</v>
+      </c>
       <c r="X102" s="102">
         <v>2</v>
       </c>
@@ -23852,7 +24059,9 @@
       <c r="V103" s="127">
         <v>0</v>
       </c>
-      <c r="W103" s="66"/>
+      <c r="W103" s="66">
+        <v>1</v>
+      </c>
       <c r="X103" s="127">
         <v>0</v>
       </c>
@@ -24016,7 +24225,9 @@
       <c r="V104" s="102">
         <v>3</v>
       </c>
-      <c r="W104" s="103"/>
+      <c r="W104" s="103">
+        <v>2</v>
+      </c>
       <c r="X104" s="102">
         <v>3</v>
       </c>
@@ -24180,7 +24391,9 @@
       <c r="V105" s="12">
         <v>3</v>
       </c>
-      <c r="W105" s="13"/>
+      <c r="W105" s="13">
+        <v>5</v>
+      </c>
       <c r="X105" s="12">
         <v>3</v>
       </c>
@@ -24344,7 +24557,9 @@
       <c r="V106" s="102">
         <v>3</v>
       </c>
-      <c r="W106" s="103"/>
+      <c r="W106" s="103">
+        <v>4</v>
+      </c>
       <c r="X106" s="102">
         <v>3</v>
       </c>
@@ -24508,7 +24723,9 @@
       <c r="V107" s="12">
         <v>1</v>
       </c>
-      <c r="W107" s="13"/>
+      <c r="W107" s="13">
+        <v>2</v>
+      </c>
       <c r="X107" s="12">
         <v>1</v>
       </c>
@@ -24832,7 +25049,9 @@
       <c r="V109" s="12">
         <v>2</v>
       </c>
-      <c r="W109" s="13"/>
+      <c r="W109" s="13">
+        <v>1</v>
+      </c>
       <c r="X109" s="12">
         <v>2</v>
       </c>
@@ -24996,7 +25215,9 @@
       <c r="V110" s="102">
         <v>1</v>
       </c>
-      <c r="W110" s="103"/>
+      <c r="W110" s="103">
+        <v>1</v>
+      </c>
       <c r="X110" s="102">
         <v>1</v>
       </c>
@@ -25160,7 +25381,9 @@
       <c r="V111" s="12">
         <v>1</v>
       </c>
-      <c r="W111" s="13"/>
+      <c r="W111" s="13">
+        <v>1</v>
+      </c>
       <c r="X111" s="12">
         <v>1</v>
       </c>
@@ -25324,7 +25547,9 @@
       <c r="V112" s="102">
         <v>2</v>
       </c>
-      <c r="W112" s="103"/>
+      <c r="W112" s="103">
+        <v>2</v>
+      </c>
       <c r="X112" s="102">
         <v>1</v>
       </c>
@@ -25488,7 +25713,9 @@
       <c r="V113" s="12">
         <v>0</v>
       </c>
-      <c r="W113" s="13"/>
+      <c r="W113" s="13">
+        <v>1</v>
+      </c>
       <c r="X113" s="12">
         <v>0</v>
       </c>
@@ -25652,7 +25879,9 @@
       <c r="V114" s="127">
         <v>0</v>
       </c>
-      <c r="W114" s="66"/>
+      <c r="W114" s="66">
+        <v>112</v>
+      </c>
       <c r="X114" s="127">
         <v>0</v>
       </c>
@@ -25816,7 +26045,9 @@
       <c r="V115" s="17">
         <v>1</v>
       </c>
-      <c r="W115" s="18"/>
+      <c r="W115" s="18">
+        <v>2</v>
+      </c>
       <c r="X115" s="17">
         <v>1</v>
       </c>
@@ -26003,7 +26234,7 @@
       </c>
       <c r="W116" s="112">
         <f t="shared" si="38"/>
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="X116" s="112">
         <f t="shared" si="38"/>
@@ -27248,9 +27479,11 @@
         <v>1105</v>
       </c>
       <c r="I5" s="68">
-        <v>1155</v>
-      </c>
-      <c r="J5" s="68"/>
+        <v>1265</v>
+      </c>
+      <c r="J5" s="68">
+        <v>147</v>
+      </c>
       <c r="K5" s="68"/>
       <c r="L5" s="68"/>
       <c r="M5" s="68"/>
@@ -27307,7 +27540,9 @@
       <c r="I6" s="69">
         <v>23</v>
       </c>
-      <c r="J6" s="69"/>
+      <c r="J6" s="69">
+        <v>3</v>
+      </c>
       <c r="K6" s="69"/>
       <c r="L6" s="69"/>
       <c r="M6" s="69"/>
@@ -27330,7 +27565,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="69">
-        <f t="shared" ref="C7:I7" si="2">IFERROR(C5/C6,0)</f>
+        <f t="shared" ref="C7:J7" si="2">IFERROR(C5/C6,0)</f>
         <v>6</v>
       </c>
       <c r="D7" s="69">
@@ -27355,9 +27590,12 @@
       </c>
       <c r="I7" s="69">
         <f t="shared" si="2"/>
-        <v>50.217391304347828</v>
-      </c>
-      <c r="J7" s="69"/>
+        <v>55</v>
+      </c>
+      <c r="J7" s="69">
+        <f t="shared" si="2"/>
+        <v>49</v>
+      </c>
       <c r="K7" s="69"/>
       <c r="L7" s="69"/>
       <c r="M7" s="69"/>
@@ -27422,34 +27660,34 @@
         <v>1352.8999999999996</v>
       </c>
       <c r="J8" s="147">
-        <v>1385.1000000000004</v>
+        <v>1406.5</v>
       </c>
       <c r="K8" s="147">
-        <v>1253.1999999999998</v>
+        <v>1259.5</v>
       </c>
       <c r="L8" s="147">
-        <v>923.40000000000055</v>
+        <v>928.10000000000036</v>
       </c>
       <c r="M8" s="147">
-        <v>1253.2000000000007</v>
+        <v>1259.5</v>
       </c>
       <c r="N8" s="147">
-        <v>1319.2000000000007</v>
+        <v>1325.7999999999993</v>
       </c>
       <c r="O8" s="147">
-        <v>1517.1000000000004</v>
+        <v>1524.7000000000007</v>
       </c>
       <c r="P8" s="147">
-        <v>1451.1000000000004</v>
+        <v>1458.3999999999996</v>
       </c>
       <c r="Q8" s="147">
-        <v>1385.1000000000004</v>
+        <v>1392.1000000000004</v>
       </c>
       <c r="R8" s="147">
-        <v>1451.0999999999985</v>
+        <v>1458.3999999999996</v>
       </c>
       <c r="S8" s="147">
-        <v>990.69999999999709</v>
+        <v>1004.0999999999985</v>
       </c>
       <c r="T8" s="147">
         <v>0</v>
@@ -27596,43 +27834,43 @@
       </c>
       <c r="J10" s="69">
         <f t="shared" si="5"/>
-        <v>51.300000000000011</v>
+        <v>52.092592592592595</v>
       </c>
       <c r="K10" s="69">
         <f t="shared" si="5"/>
-        <v>50.127999999999993</v>
+        <v>50.38</v>
       </c>
       <c r="L10" s="69">
         <f t="shared" si="5"/>
-        <v>57.712500000000034</v>
+        <v>58.006250000000023</v>
       </c>
       <c r="M10" s="69">
         <f t="shared" si="5"/>
-        <v>52.216666666666697</v>
+        <v>52.479166666666664</v>
       </c>
       <c r="N10" s="69">
         <f t="shared" si="5"/>
-        <v>54.966666666666697</v>
+        <v>55.241666666666639</v>
       </c>
       <c r="O10" s="69">
         <f t="shared" si="5"/>
-        <v>56.188888888888904</v>
+        <v>56.470370370370397</v>
       </c>
       <c r="P10" s="69">
         <f t="shared" si="5"/>
-        <v>55.811538461538476</v>
+        <v>56.092307692307678</v>
       </c>
       <c r="Q10" s="69">
         <f t="shared" si="5"/>
-        <v>53.273076923076935</v>
+        <v>53.542307692307709</v>
       </c>
       <c r="R10" s="69">
         <f t="shared" si="5"/>
-        <v>55.811538461538404</v>
+        <v>56.092307692307678</v>
       </c>
       <c r="S10" s="69">
         <f t="shared" si="5"/>
-        <v>36.692592592592483</v>
+        <v>37.188888888888833</v>
       </c>
       <c r="T10" s="69">
         <f t="shared" si="5"/>
@@ -28154,31 +28392,31 @@
         <v>16832</v>
       </c>
       <c r="I19" s="147">
-        <v>19642.699999999997</v>
+        <v>13615</v>
       </c>
       <c r="J19" s="147">
-        <v>19828.5</v>
+        <v>22273.800000000003</v>
       </c>
       <c r="K19" s="147">
-        <v>16333.400000000009</v>
+        <v>17983.499999999985</v>
       </c>
       <c r="L19" s="147">
-        <v>12810.299999999988</v>
+        <v>12729.600000000006</v>
       </c>
       <c r="M19" s="147">
-        <v>17724.5</v>
+        <v>17684.899999999994</v>
       </c>
       <c r="N19" s="147">
-        <v>18617.200000000012</v>
+        <v>18621.899999999994</v>
       </c>
       <c r="O19" s="147">
         <v>21409.799999999988</v>
       </c>
       <c r="P19" s="147">
-        <v>20513.399999999994</v>
+        <v>20509.700000000012</v>
       </c>
       <c r="Q19" s="147">
-        <v>19843.799999999988</v>
+        <v>19846.899999999994</v>
       </c>
       <c r="R19" s="147">
         <v>20484.799999999988</v>
@@ -28187,7 +28425,7 @@
         <v>20484.799999999988</v>
       </c>
       <c r="T19" s="147">
-        <v>11546.299999999988</v>
+        <v>13594.799999999988</v>
       </c>
       <c r="U19" s="147">
         <v>0</v>
@@ -28306,27 +28544,27 @@
       </c>
       <c r="I21" s="69">
         <f t="shared" si="10"/>
-        <v>785.70799999999986</v>
+        <v>544.6</v>
       </c>
       <c r="J21" s="69">
         <f t="shared" si="10"/>
-        <v>734.38888888888891</v>
+        <v>824.95555555555563</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="10"/>
-        <v>653.33600000000035</v>
+        <v>719.33999999999946</v>
       </c>
       <c r="L21" s="69">
         <f t="shared" si="10"/>
-        <v>800.64374999999927</v>
+        <v>795.60000000000036</v>
       </c>
       <c r="M21" s="69">
         <f t="shared" si="10"/>
-        <v>738.52083333333337</v>
+        <v>736.87083333333305</v>
       </c>
       <c r="N21" s="69">
         <f t="shared" si="10"/>
-        <v>775.71666666666715</v>
+        <v>775.9124999999998</v>
       </c>
       <c r="O21" s="69">
         <f t="shared" si="10"/>
@@ -28334,11 +28572,11 @@
       </c>
       <c r="P21" s="69">
         <f t="shared" si="10"/>
-        <v>788.97692307692284</v>
+        <v>788.83461538461586</v>
       </c>
       <c r="Q21" s="69">
         <f t="shared" si="10"/>
-        <v>763.22307692307652</v>
+        <v>763.34230769230749</v>
       </c>
       <c r="R21" s="69">
         <f t="shared" si="10"/>
@@ -28350,7 +28588,7 @@
       </c>
       <c r="T21" s="69">
         <f t="shared" si="10"/>
-        <v>444.0884615384611</v>
+        <v>522.87692307692259</v>
       </c>
       <c r="U21" s="69">
         <f t="shared" si="10"/>
@@ -28681,10 +28919,10 @@
         <v>41202</v>
       </c>
       <c r="I27" s="68">
-        <v>34647</v>
-      </c>
-      <c r="J27" s="68" t="s">
-        <v>196</v>
+        <v>36285</v>
+      </c>
+      <c r="J27" s="68">
+        <v>7348</v>
       </c>
       <c r="K27" s="68" t="s">
         <v>196</v>
@@ -28752,7 +28990,9 @@
       <c r="I28" s="69">
         <v>13</v>
       </c>
-      <c r="J28" s="69"/>
+      <c r="J28" s="69">
+        <v>2</v>
+      </c>
       <c r="K28" s="69"/>
       <c r="L28" s="69"/>
       <c r="M28" s="69"/>
@@ -28775,7 +29015,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="69">
-        <f t="shared" ref="C29:I29" si="12">IFERROR(C27/C28,0)</f>
+        <f t="shared" ref="C29:J29" si="12">IFERROR(C27/C28,0)</f>
         <v>1045.75</v>
       </c>
       <c r="D29" s="69">
@@ -28800,9 +29040,12 @@
       </c>
       <c r="I29" s="69">
         <f t="shared" si="12"/>
-        <v>2665.1538461538462</v>
-      </c>
-      <c r="J29" s="69"/>
+        <v>2791.1538461538462</v>
+      </c>
+      <c r="J29" s="69">
+        <f t="shared" si="12"/>
+        <v>3674</v>
+      </c>
       <c r="K29" s="69"/>
       <c r="L29" s="69"/>
       <c r="M29" s="69"/>
@@ -28848,43 +29091,43 @@
         <v>41202</v>
       </c>
       <c r="I30" s="147">
-        <v>42976.200000000012</v>
+        <v>36285</v>
       </c>
       <c r="J30" s="147">
-        <v>50286.200000000012</v>
+        <v>55457.799999999988</v>
       </c>
       <c r="K30" s="147">
-        <v>55255.166666666686</v>
+        <v>45223.200000000012</v>
       </c>
       <c r="L30" s="147">
-        <v>37919.966666666674</v>
+        <v>36609.5</v>
       </c>
       <c r="M30" s="147">
-        <v>49715.066666666651</v>
+        <v>38266.299999999988</v>
       </c>
       <c r="N30" s="147">
-        <v>37907.700000000012</v>
+        <v>49823.700000000012</v>
       </c>
       <c r="O30" s="147">
         <v>50217.700000000012</v>
       </c>
       <c r="P30" s="147">
-        <v>45499.5</v>
+        <v>47717.900000000023</v>
       </c>
       <c r="Q30" s="147">
-        <v>51922.299999999988</v>
+        <v>52575.700000000012</v>
       </c>
       <c r="R30" s="147">
-        <v>45895.599999999977</v>
+        <v>48370.599999999977</v>
       </c>
       <c r="S30" s="147">
-        <v>36868.900000000023</v>
+        <v>36785.800000000047</v>
       </c>
       <c r="T30" s="147">
-        <v>688152.10000000009</v>
+        <v>49910.900000000023</v>
       </c>
       <c r="U30" s="147">
-        <v>40718.799999999814</v>
+        <v>47310.799999999814</v>
       </c>
       <c r="V30" s="147">
         <v>0</v>
@@ -29000,27 +29243,27 @@
       </c>
       <c r="I32" s="69">
         <f t="shared" si="15"/>
-        <v>1719.0480000000005</v>
+        <v>1451.4</v>
       </c>
       <c r="J32" s="69">
         <f t="shared" si="15"/>
-        <v>1862.4518518518523</v>
+        <v>2053.9925925925922</v>
       </c>
       <c r="K32" s="69">
         <f t="shared" si="15"/>
-        <v>2210.2066666666674</v>
+        <v>1808.9280000000006</v>
       </c>
       <c r="L32" s="69">
         <f t="shared" si="15"/>
-        <v>2369.9979166666672</v>
+        <v>2288.09375</v>
       </c>
       <c r="M32" s="69">
         <f t="shared" si="15"/>
-        <v>2071.4611111111103</v>
+        <v>1594.4291666666661</v>
       </c>
       <c r="N32" s="69">
         <f t="shared" si="15"/>
-        <v>1579.4875000000004</v>
+        <v>2075.9875000000006</v>
       </c>
       <c r="O32" s="69">
         <f t="shared" si="15"/>
@@ -29028,27 +29271,27 @@
       </c>
       <c r="P32" s="69">
         <f t="shared" si="15"/>
-        <v>1749.9807692307693</v>
+        <v>1835.303846153847</v>
       </c>
       <c r="Q32" s="69">
         <f t="shared" si="15"/>
-        <v>1997.0115384615381</v>
+        <v>2022.1423076923081</v>
       </c>
       <c r="R32" s="69">
         <f t="shared" si="15"/>
-        <v>1765.2153846153838</v>
+        <v>1860.4076923076914</v>
       </c>
       <c r="S32" s="69">
         <f t="shared" si="15"/>
-        <v>1365.5148148148157</v>
+        <v>1362.4370370370389</v>
       </c>
       <c r="T32" s="69">
         <f t="shared" si="15"/>
-        <v>26467.388461538467</v>
+        <v>1919.650000000001</v>
       </c>
       <c r="U32" s="69">
         <f t="shared" si="15"/>
-        <v>1566.1076923076851</v>
+        <v>1819.6461538461467</v>
       </c>
       <c r="V32" s="69">
         <v>0</v>
@@ -29375,10 +29618,10 @@
         <v>57</v>
       </c>
       <c r="I38" s="68">
-        <v>101</v>
-      </c>
-      <c r="J38" s="68" t="s">
-        <v>196</v>
+        <v>119</v>
+      </c>
+      <c r="J38" s="68">
+        <v>9</v>
       </c>
       <c r="K38" s="68" t="s">
         <v>196</v>
@@ -29444,9 +29687,11 @@
         <v>17</v>
       </c>
       <c r="I39" s="69">
-        <v>16</v>
-      </c>
-      <c r="J39" s="69"/>
+        <v>22</v>
+      </c>
+      <c r="J39" s="69">
+        <v>1</v>
+      </c>
       <c r="K39" s="69"/>
       <c r="L39" s="69"/>
       <c r="M39" s="69"/>
@@ -29495,7 +29740,9 @@
       <c r="I40" s="69">
         <v>22</v>
       </c>
-      <c r="J40" s="69"/>
+      <c r="J40" s="69">
+        <v>22</v>
+      </c>
       <c r="K40" s="69"/>
       <c r="L40" s="69"/>
       <c r="M40" s="69"/>
@@ -29544,43 +29791,43 @@
         <v>132.20000000000005</v>
       </c>
       <c r="J41" s="147">
-        <v>262</v>
+        <v>272.79999999999995</v>
       </c>
       <c r="K41" s="147">
-        <v>196.70000000000005</v>
+        <v>196.39999999999998</v>
       </c>
       <c r="L41" s="147">
-        <v>187.40000000000009</v>
+        <v>186.99999999999989</v>
       </c>
       <c r="M41" s="147">
-        <v>214.29999999999995</v>
+        <v>213.5</v>
       </c>
       <c r="N41" s="147">
-        <v>157.29999999999995</v>
+        <v>158.09999999999991</v>
       </c>
       <c r="O41" s="147">
-        <v>226.20000000000005</v>
+        <v>226.90000000000009</v>
       </c>
       <c r="P41" s="147">
-        <v>261.79999999999995</v>
+        <v>261.69999999999982</v>
       </c>
       <c r="Q41" s="147">
         <v>267.80000000000018</v>
       </c>
       <c r="R41" s="147">
-        <v>288.69999999999982</v>
+        <v>288.09999999999991</v>
       </c>
       <c r="S41" s="147">
-        <v>330.59999999999991</v>
+        <v>330.90000000000009</v>
       </c>
       <c r="T41" s="147">
-        <v>257.80000000000018</v>
+        <v>261.40000000000009</v>
       </c>
       <c r="U41" s="147">
         <v>80.900000000000091</v>
       </c>
       <c r="V41" s="147">
-        <v>10.099999999999909</v>
+        <v>9.3000000000001819</v>
       </c>
       <c r="X41" s="148"/>
     </row>
@@ -29697,31 +29944,31 @@
       </c>
       <c r="J43" s="69">
         <f t="shared" si="20"/>
-        <v>9.7037037037037042</v>
+        <v>10.103703703703703</v>
       </c>
       <c r="K43" s="69">
         <f t="shared" si="20"/>
-        <v>7.8680000000000021</v>
+        <v>7.855999999999999</v>
       </c>
       <c r="L43" s="69">
         <f t="shared" si="20"/>
-        <v>11.712500000000006</v>
+        <v>11.687499999999993</v>
       </c>
       <c r="M43" s="69">
         <f t="shared" si="20"/>
-        <v>8.9291666666666654</v>
+        <v>8.8958333333333339</v>
       </c>
       <c r="N43" s="69">
         <f t="shared" si="20"/>
-        <v>6.5541666666666645</v>
+        <v>6.5874999999999959</v>
       </c>
       <c r="O43" s="69">
         <f t="shared" si="20"/>
-        <v>8.37777777777778</v>
+        <v>8.403703703703707</v>
       </c>
       <c r="P43" s="69">
         <f t="shared" si="20"/>
-        <v>10.069230769230767</v>
+        <v>10.065384615384609</v>
       </c>
       <c r="Q43" s="69">
         <f t="shared" si="20"/>
@@ -29729,15 +29976,15 @@
       </c>
       <c r="R43" s="69">
         <f t="shared" si="20"/>
-        <v>11.103846153846147</v>
+        <v>11.080769230769228</v>
       </c>
       <c r="S43" s="69">
         <f t="shared" si="20"/>
-        <v>12.244444444444442</v>
+        <v>12.255555555555558</v>
       </c>
       <c r="T43" s="69">
         <f t="shared" si="20"/>
-        <v>9.9153846153846228</v>
+        <v>10.053846153846157</v>
       </c>
       <c r="U43" s="69">
         <f t="shared" si="20"/>
@@ -30068,10 +30315,10 @@
         <v>14588</v>
       </c>
       <c r="I49" s="68">
-        <v>16920</v>
-      </c>
-      <c r="J49" s="68" t="s">
-        <v>196</v>
+        <v>18166</v>
+      </c>
+      <c r="J49" s="68">
+        <v>1450</v>
       </c>
       <c r="K49" s="68" t="s">
         <v>196</v>
@@ -30139,7 +30386,9 @@
       <c r="I50" s="69">
         <v>17</v>
       </c>
-      <c r="J50" s="69"/>
+      <c r="J50" s="69">
+        <v>3</v>
+      </c>
       <c r="K50" s="69"/>
       <c r="L50" s="69"/>
       <c r="M50" s="69"/>
@@ -30162,7 +30411,7 @@
         <v>0</v>
       </c>
       <c r="C51" s="69">
-        <f t="shared" ref="C51:I51" si="22">IFERROR(C49/C50,0)</f>
+        <f t="shared" ref="C51:J51" si="22">IFERROR(C49/C50,0)</f>
         <v>0</v>
       </c>
       <c r="D51" s="69">
@@ -30187,9 +30436,12 @@
       </c>
       <c r="I51" s="69">
         <f t="shared" si="22"/>
-        <v>995.29411764705878</v>
-      </c>
-      <c r="J51" s="69"/>
+        <v>1068.5882352941176</v>
+      </c>
+      <c r="J51" s="69">
+        <f t="shared" si="22"/>
+        <v>483.33333333333331</v>
+      </c>
       <c r="K51" s="69"/>
       <c r="L51" s="69"/>
       <c r="M51" s="69"/>
@@ -30238,40 +30490,40 @@
         <v>19854.100000000006</v>
       </c>
       <c r="J52" s="147">
-        <v>24090.600000000006</v>
+        <v>21512.800000000003</v>
       </c>
       <c r="K52" s="147">
-        <v>21931.899999999994</v>
+        <v>33846.800000000003</v>
       </c>
       <c r="L52" s="147">
-        <v>18763.100000000006</v>
+        <v>17470.700000000012</v>
       </c>
       <c r="M52" s="147">
-        <v>17120</v>
+        <v>10765.700000000012</v>
       </c>
       <c r="N52" s="147">
-        <v>13402</v>
+        <v>12574.5</v>
       </c>
       <c r="O52" s="147">
-        <v>18204.100000000006</v>
+        <v>18857.700000000012</v>
       </c>
       <c r="P52" s="147">
-        <v>20481.600000000006</v>
+        <v>19841.200000000012</v>
       </c>
       <c r="Q52" s="147">
-        <v>20755.299999999988</v>
+        <v>21669.899999999994</v>
       </c>
       <c r="R52" s="147">
-        <v>25178.899999999994</v>
+        <v>23715.899999999994</v>
       </c>
       <c r="S52" s="147">
-        <v>29723.499999999971</v>
+        <v>10968.200000000012</v>
       </c>
       <c r="T52" s="147">
-        <v>20181.5</v>
+        <v>19240.699999999983</v>
       </c>
       <c r="U52" s="147">
-        <v>10132.599999999977</v>
+        <v>31189.099999999919</v>
       </c>
       <c r="V52" s="147"/>
       <c r="X52" s="148"/>
@@ -30389,51 +30641,51 @@
       </c>
       <c r="J54" s="69">
         <f t="shared" si="25"/>
-        <v>892.24444444444464</v>
+        <v>796.77037037037053</v>
       </c>
       <c r="K54" s="69">
         <f t="shared" si="25"/>
-        <v>877.27599999999973</v>
+        <v>1353.8720000000001</v>
       </c>
       <c r="L54" s="69">
         <f t="shared" si="25"/>
-        <v>1172.6937500000004</v>
+        <v>1091.9187500000007</v>
       </c>
       <c r="M54" s="69">
         <f t="shared" si="25"/>
-        <v>713.33333333333337</v>
+        <v>448.57083333333384</v>
       </c>
       <c r="N54" s="69">
         <f t="shared" si="25"/>
-        <v>558.41666666666663</v>
+        <v>523.9375</v>
       </c>
       <c r="O54" s="69">
         <f t="shared" si="25"/>
-        <v>674.22592592592616</v>
+        <v>698.43333333333374</v>
       </c>
       <c r="P54" s="69">
         <f t="shared" si="25"/>
-        <v>787.75384615384633</v>
+        <v>763.12307692307741</v>
       </c>
       <c r="Q54" s="69">
         <f t="shared" si="25"/>
-        <v>798.28076923076878</v>
+        <v>833.45769230769213</v>
       </c>
       <c r="R54" s="69">
         <f t="shared" si="25"/>
-        <v>968.41923076923058</v>
+        <v>912.14999999999975</v>
       </c>
       <c r="S54" s="69">
         <f t="shared" si="25"/>
-        <v>1100.8703703703693</v>
+        <v>406.22962962963004</v>
       </c>
       <c r="T54" s="69">
         <f t="shared" si="25"/>
-        <v>776.21153846153845</v>
+        <v>740.02692307692246</v>
       </c>
       <c r="U54" s="69">
         <f t="shared" si="25"/>
-        <v>389.7153846153837</v>
+        <v>1199.580769230766</v>
       </c>
       <c r="V54" s="69">
         <f t="shared" si="25"/>
@@ -30761,10 +31013,10 @@
         <v>22612</v>
       </c>
       <c r="I60" s="68">
-        <v>28922</v>
-      </c>
-      <c r="J60" s="68" t="s">
-        <v>196</v>
+        <v>32756</v>
+      </c>
+      <c r="J60" s="68">
+        <v>2299</v>
       </c>
       <c r="K60" s="68" t="s">
         <v>196</v>
@@ -30832,7 +31084,9 @@
       <c r="I61" s="69">
         <v>15</v>
       </c>
-      <c r="J61" s="69"/>
+      <c r="J61" s="69">
+        <v>1</v>
+      </c>
       <c r="K61" s="69"/>
       <c r="L61" s="69"/>
       <c r="M61" s="69"/>
@@ -30879,9 +31133,12 @@
       </c>
       <c r="I62" s="69">
         <f>I60/I61</f>
-        <v>1928.1333333333334</v>
-      </c>
-      <c r="J62" s="69"/>
+        <v>2183.7333333333331</v>
+      </c>
+      <c r="J62" s="69">
+        <f>J60/J61</f>
+        <v>2299</v>
+      </c>
       <c r="K62" s="69"/>
       <c r="L62" s="69"/>
       <c r="M62" s="69"/>
@@ -30929,43 +31186,43 @@
         <v>35224.199999999997</v>
       </c>
       <c r="J63" s="147">
-        <v>46993.830769230772</v>
+        <v>45728.5</v>
       </c>
       <c r="K63" s="147">
-        <v>41887.830769230757</v>
+        <v>50769.200000000012</v>
       </c>
       <c r="L63" s="147">
-        <v>40917.930769230763</v>
+        <v>39510.100000000006</v>
       </c>
       <c r="M63" s="147">
-        <v>45112.430769230763</v>
+        <v>44845.800000000017</v>
       </c>
       <c r="N63" s="147">
-        <v>35209.430769230763</v>
+        <v>34939.299999999988</v>
       </c>
       <c r="O63" s="147">
-        <v>44397.03076923074</v>
+        <v>44051.200000000012</v>
       </c>
       <c r="P63" s="147">
-        <v>47746.730769230751</v>
+        <v>47004.400000000023</v>
       </c>
       <c r="Q63" s="147">
-        <v>50767.930769230763</v>
+        <v>49998.700000000012</v>
       </c>
       <c r="R63" s="147">
-        <v>51729.130769230775</v>
+        <v>50818.5</v>
       </c>
       <c r="S63" s="147">
-        <v>52981.03076923074</v>
+        <v>52431.700000000012</v>
       </c>
       <c r="T63" s="147">
-        <v>33930.730769230751</v>
+        <v>36387.700000000012</v>
       </c>
       <c r="U63" s="147">
-        <v>50032.330769230728</v>
+        <v>47263.099999999977</v>
       </c>
       <c r="V63" s="147">
-        <v>31989.430769230938</v>
+        <v>32415.79999999993</v>
       </c>
       <c r="X63" s="148"/>
     </row>
@@ -31082,51 +31339,51 @@
       </c>
       <c r="J65" s="69">
         <f t="shared" si="29"/>
-        <v>1740.5122507122508</v>
+        <v>1693.648148148148</v>
       </c>
       <c r="K65" s="69">
         <f t="shared" si="29"/>
-        <v>1675.5132307692302</v>
+        <v>2030.7680000000005</v>
       </c>
       <c r="L65" s="69">
         <f t="shared" si="29"/>
-        <v>2557.3706730769227</v>
+        <v>2469.3812500000004</v>
       </c>
       <c r="M65" s="69">
         <f t="shared" si="29"/>
-        <v>1879.6846153846152</v>
+        <v>1868.5750000000007</v>
       </c>
       <c r="N65" s="69">
         <f t="shared" si="29"/>
-        <v>1467.0596153846152</v>
+        <v>1455.8041666666661</v>
       </c>
       <c r="O65" s="69">
         <f t="shared" si="29"/>
-        <v>1644.3344729344719</v>
+        <v>1631.5259259259265</v>
       </c>
       <c r="P65" s="69">
         <f t="shared" si="29"/>
-        <v>1836.4127218934905</v>
+        <v>1807.8615384615393</v>
       </c>
       <c r="Q65" s="69">
         <f t="shared" si="29"/>
-        <v>1952.612721893491</v>
+        <v>1923.0269230769236</v>
       </c>
       <c r="R65" s="69">
         <f t="shared" si="29"/>
-        <v>1989.5819526627222</v>
+        <v>1954.5576923076924</v>
       </c>
       <c r="S65" s="69">
         <f t="shared" si="29"/>
-        <v>1962.2603988603978</v>
+        <v>1941.9148148148151</v>
       </c>
       <c r="T65" s="69">
         <f t="shared" si="29"/>
-        <v>1305.028106508875</v>
+        <v>1399.5269230769236</v>
       </c>
       <c r="U65" s="69">
         <f t="shared" si="29"/>
-        <v>1924.3204142011818</v>
+        <v>1817.8115384615376</v>
       </c>
       <c r="V65" s="69">
         <v>0</v>
@@ -31194,47 +31451,47 @@
       <c r="B2" s="46"/>
       <c r="C2" s="34">
         <f>SUM(C4:C733)</f>
-        <v>134099.62000000002</v>
+        <v>140861.58000000002</v>
       </c>
       <c r="D2" s="35">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>135150.58000000005</v>
+        <v>140757.66000000006</v>
       </c>
       <c r="E2" s="36">
         <f t="shared" si="0"/>
-        <v>18755.875384615385</v>
+        <v>12503.916923076924</v>
       </c>
       <c r="F2" s="34">
         <f t="shared" si="0"/>
-        <v>199210.08699999994</v>
+        <v>205357.03699999992</v>
       </c>
       <c r="G2" s="35">
         <f t="shared" si="0"/>
-        <v>200023.69999999995</v>
+        <v>203362.47999999998</v>
       </c>
       <c r="H2" s="36">
         <f t="shared" si="0"/>
-        <v>30149.095384615372</v>
+        <v>16958.866153846153</v>
       </c>
       <c r="I2" s="34">
         <f t="shared" si="0"/>
-        <v>7914.5999999999995</v>
+        <v>11968.449999999999</v>
       </c>
       <c r="J2" s="35">
         <f t="shared" si="0"/>
-        <v>8744.0259809999989</v>
+        <v>16608.355980999997</v>
       </c>
       <c r="K2" s="36">
         <f t="shared" si="0"/>
-        <v>587000.00000000058</v>
+        <v>579814.81481481565</v>
       </c>
       <c r="L2" s="34">
         <f t="shared" si="0"/>
-        <v>327338.98249999981</v>
+        <v>345297.78222199978</v>
       </c>
       <c r="M2" s="36">
         <f t="shared" si="0"/>
-        <v>683919.90903846011</v>
+        <v>662619.65655555553</v>
       </c>
       <c r="N2" s="29"/>
     </row>
@@ -31434,11 +31691,11 @@
       </c>
       <c r="Y5" s="5">
         <f t="shared" si="2"/>
-        <v>63827.385980999999</v>
+        <v>73069.385980999999</v>
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>7568.1900000000005</v>
       </c>
       <c r="AA5" s="5">
         <f t="shared" si="2"/>
@@ -31521,11 +31778,11 @@
       </c>
       <c r="Y6" s="5">
         <f t="shared" si="4"/>
-        <v>10332.366153846153</v>
+        <v>0</v>
       </c>
       <c r="Z6" s="5">
         <f t="shared" si="4"/>
-        <v>75572.604615384596</v>
+        <v>59277.597891737882</v>
       </c>
       <c r="AA6" s="5">
         <f t="shared" si="4"/>
@@ -31648,11 +31905,11 @@
       </c>
       <c r="Y8" s="5">
         <f t="shared" si="5"/>
-        <v>51989.5</v>
+        <v>59170.239721999998</v>
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>10778.059999999998</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="5"/>
@@ -31735,11 +31992,11 @@
       </c>
       <c r="Y9" s="5">
         <f t="shared" si="6"/>
-        <v>13583.791038461537</v>
+        <v>0</v>
       </c>
       <c r="Z9" s="5">
         <f t="shared" si="6"/>
-        <v>69448.15300000002</v>
+        <v>61731.691555555582</v>
       </c>
       <c r="AA9" s="5">
         <f t="shared" si="6"/>
@@ -31862,19 +32119,19 @@
       </c>
       <c r="Y11" s="5">
         <f t="shared" si="7"/>
-        <v>354250.6721348461</v>
+        <v>353160.30598099995</v>
       </c>
       <c r="Z11" s="5">
         <f t="shared" si="7"/>
-        <v>429823.2767502307</v>
+        <v>420006.09387273784</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="7"/>
-        <v>479823.2767502307</v>
+        <v>470006.09387273784</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="7"/>
-        <v>529823.2767502307</v>
+        <v>520006.09387273784</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
@@ -31949,19 +32206,19 @@
       </c>
       <c r="Y12" s="5">
         <f t="shared" si="8"/>
-        <v>340922.7735384616</v>
+        <v>334519.72222200001</v>
       </c>
       <c r="Z12" s="5">
         <f t="shared" si="8"/>
-        <v>410370.92653846159</v>
+        <v>407029.47377755563</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="8"/>
-        <v>477676.81153846154</v>
+        <v>474335.35877755558</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="8"/>
-        <v>513923.1465384615</v>
+        <v>510581.69377755554</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -32036,19 +32293,19 @@
       </c>
       <c r="Y13" s="5">
         <f t="shared" si="9"/>
-        <v>13327.898596384504</v>
+        <v>18640.583758999943</v>
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>19452.35021176911</v>
+        <v>12976.62009518221</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
-        <v>2146.4652117691585</v>
+        <v>-4329.2649048177409</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>15900.130211769196</v>
+        <v>9424.4000951822964</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
@@ -42422,25 +42679,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C273" s="39"/>
-      <c r="D273" s="40"/>
-      <c r="E273" s="182">
-        <v>0</v>
-      </c>
-      <c r="F273" s="39"/>
-      <c r="G273" s="40"/>
-      <c r="H273" s="182">
-        <v>0</v>
-      </c>
-      <c r="I273" s="39"/>
-      <c r="J273" s="40"/>
+      <c r="C273" s="39">
+        <v>236.09</v>
+      </c>
+      <c r="D273" s="40">
+        <v>0</v>
+      </c>
+      <c r="E273" s="42"/>
+      <c r="F273" s="39">
+        <v>0</v>
+      </c>
+      <c r="G273" s="40">
+        <v>0</v>
+      </c>
+      <c r="H273" s="42"/>
+      <c r="I273" s="39">
+        <v>0</v>
+      </c>
+      <c r="J273" s="40">
+        <v>0</v>
+      </c>
       <c r="K273" s="5">
         <v>0</v>
       </c>
-      <c r="L273" s="157"/>
-      <c r="M273" s="41">
-        <v>0</v>
-      </c>
+      <c r="L273" s="157">
+        <v>0</v>
+      </c>
+      <c r="M273" s="41"/>
       <c r="O273" s="29"/>
       <c r="P273" s="5"/>
       <c r="R273" s="5"/>
@@ -42456,25 +42721,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C274" s="39"/>
-      <c r="D274" s="40"/>
-      <c r="E274" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F274" s="39"/>
-      <c r="G274" s="40"/>
-      <c r="H274" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I274" s="39"/>
-      <c r="J274" s="40"/>
+      <c r="C274" s="39">
+        <v>1220.27</v>
+      </c>
+      <c r="D274" s="40">
+        <v>1035.1200000000001</v>
+      </c>
+      <c r="E274" s="42"/>
+      <c r="F274" s="39">
+        <v>0</v>
+      </c>
+      <c r="G274" s="40">
+        <v>0</v>
+      </c>
+      <c r="H274" s="42"/>
+      <c r="I274" s="39">
+        <v>782</v>
+      </c>
+      <c r="J274" s="40">
+        <v>2330.4899999999993</v>
+      </c>
       <c r="K274" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L274" s="157"/>
-      <c r="M274" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L274" s="157">
+        <v>4903.92</v>
+      </c>
+      <c r="M274" s="41"/>
       <c r="O274" s="29"/>
       <c r="P274" s="5"/>
       <c r="R274" s="5"/>
@@ -42490,25 +42763,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C275" s="39"/>
-      <c r="D275" s="40"/>
-      <c r="E275" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F275" s="39"/>
-      <c r="G275" s="40"/>
-      <c r="H275" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I275" s="39"/>
-      <c r="J275" s="40"/>
+      <c r="C275" s="39">
+        <v>285.36</v>
+      </c>
+      <c r="D275" s="40">
+        <v>719.68</v>
+      </c>
+      <c r="E275" s="42"/>
+      <c r="F275" s="39">
+        <v>625.83000000000004</v>
+      </c>
+      <c r="G275" s="40">
+        <v>153.63999999999999</v>
+      </c>
+      <c r="H275" s="42"/>
+      <c r="I275" s="39">
+        <v>1344.9</v>
+      </c>
+      <c r="J275" s="40">
+        <v>1529.65</v>
+      </c>
       <c r="K275" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L275" s="157"/>
-      <c r="M275" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L275" s="157">
+        <v>0</v>
+      </c>
+      <c r="M275" s="41"/>
       <c r="O275" s="29"/>
       <c r="P275" s="5"/>
       <c r="R275" s="5"/>
@@ -42524,25 +42805,33 @@
         <f t="shared" si="17"/>
         <v>set/26</v>
       </c>
-      <c r="C276" s="39"/>
-      <c r="D276" s="40"/>
-      <c r="E276" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F276" s="39"/>
-      <c r="G276" s="40"/>
-      <c r="H276" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I276" s="39"/>
-      <c r="J276" s="40"/>
+      <c r="C276" s="39">
+        <v>921.29</v>
+      </c>
+      <c r="D276" s="40">
+        <v>451</v>
+      </c>
+      <c r="E276" s="42"/>
+      <c r="F276" s="39">
+        <v>1358.18</v>
+      </c>
+      <c r="G276" s="40">
+        <v>958.82000000000016</v>
+      </c>
+      <c r="H276" s="42"/>
+      <c r="I276" s="39">
+        <v>922.7</v>
+      </c>
+      <c r="J276" s="40">
+        <v>2063.6</v>
+      </c>
       <c r="K276" s="5">
-        <v>666.66666666666663</v>
-      </c>
-      <c r="L276" s="157"/>
-      <c r="M276" s="41">
-        <v>4527.9303461538457</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L276" s="157">
+        <v>2276.8197219999997</v>
+      </c>
+      <c r="M276" s="41"/>
       <c r="O276" s="29"/>
       <c r="P276" s="5"/>
       <c r="R276" s="5"/>
@@ -42558,25 +42847,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C277" s="39"/>
-      <c r="D277" s="40"/>
-      <c r="E277" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F277" s="39"/>
-      <c r="G277" s="40"/>
-      <c r="H277" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I277" s="39"/>
-      <c r="J277" s="40"/>
+      <c r="C277" s="39">
+        <v>1622.16</v>
+      </c>
+      <c r="D277" s="40">
+        <v>1536.76</v>
+      </c>
+      <c r="E277" s="42"/>
+      <c r="F277" s="39">
+        <v>930.69</v>
+      </c>
+      <c r="G277" s="40">
+        <v>1144.4999999999998</v>
+      </c>
+      <c r="H277" s="42"/>
+      <c r="I277" s="39">
+        <v>934.25</v>
+      </c>
+      <c r="J277" s="40">
+        <v>1286.47</v>
+      </c>
       <c r="K277" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L277" s="157"/>
-      <c r="M277" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L277" s="157">
+        <v>4349.3099999999995</v>
+      </c>
+      <c r="M277" s="41"/>
       <c r="O277" s="29"/>
       <c r="P277" s="5"/>
       <c r="R277" s="5"/>
@@ -42592,25 +42889,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C278" s="39"/>
-      <c r="D278" s="40"/>
-      <c r="E278" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F278" s="39"/>
-      <c r="G278" s="40"/>
-      <c r="H278" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I278" s="39"/>
-      <c r="J278" s="40"/>
+      <c r="C278" s="39">
+        <v>1317.09</v>
+      </c>
+      <c r="D278" s="40">
+        <v>1161.92</v>
+      </c>
+      <c r="E278" s="42"/>
+      <c r="F278" s="39">
+        <v>1437.93</v>
+      </c>
+      <c r="G278" s="40">
+        <v>251.6</v>
+      </c>
+      <c r="H278" s="42"/>
+      <c r="I278" s="39">
+        <v>70</v>
+      </c>
+      <c r="J278" s="40">
+        <v>654.12</v>
+      </c>
       <c r="K278" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L278" s="157"/>
-      <c r="M278" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L278" s="157">
+        <v>330.82</v>
+      </c>
+      <c r="M278" s="41"/>
       <c r="O278" s="29"/>
       <c r="P278" s="5"/>
       <c r="R278" s="5"/>
@@ -42626,25 +42931,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C279" s="39"/>
-      <c r="D279" s="40"/>
-      <c r="E279" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F279" s="39"/>
-      <c r="G279" s="40"/>
-      <c r="H279" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I279" s="39"/>
-      <c r="J279" s="40"/>
+      <c r="C279" s="39">
+        <v>643.05999999999995</v>
+      </c>
+      <c r="D279" s="40">
+        <v>702.59999999999991</v>
+      </c>
+      <c r="E279" s="42"/>
+      <c r="F279" s="39">
+        <v>688.12</v>
+      </c>
+      <c r="G279" s="40">
+        <v>830.22</v>
+      </c>
+      <c r="H279" s="42"/>
+      <c r="I279" s="39">
+        <v>0</v>
+      </c>
+      <c r="J279" s="40">
+        <v>0</v>
+      </c>
       <c r="K279" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L279" s="157"/>
-      <c r="M279" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L279" s="157">
+        <v>6097.9299999999994</v>
+      </c>
+      <c r="M279" s="41"/>
       <c r="O279" s="29"/>
       <c r="P279" s="5"/>
       <c r="R279" s="5"/>
@@ -42660,18 +42973,26 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C280" s="39"/>
-      <c r="D280" s="40"/>
-      <c r="E280" s="182">
-        <v>0</v>
-      </c>
-      <c r="F280" s="39"/>
-      <c r="G280" s="40"/>
-      <c r="H280" s="182">
-        <v>0</v>
-      </c>
-      <c r="I280" s="39"/>
-      <c r="J280" s="40"/>
+      <c r="C280" s="39">
+        <v>0</v>
+      </c>
+      <c r="D280" s="40">
+        <v>0</v>
+      </c>
+      <c r="E280" s="42"/>
+      <c r="F280" s="39">
+        <v>0</v>
+      </c>
+      <c r="G280" s="40">
+        <v>0</v>
+      </c>
+      <c r="H280" s="42"/>
+      <c r="I280" s="39">
+        <v>0</v>
+      </c>
+      <c r="J280" s="40">
+        <v>0</v>
+      </c>
       <c r="K280" s="5">
         <v>0</v>
       </c>
@@ -42694,20 +43015,28 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C281" s="39"/>
-      <c r="D281" s="40"/>
-      <c r="E281" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F281" s="39"/>
-      <c r="G281" s="40"/>
-      <c r="H281" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I281" s="39"/>
-      <c r="J281" s="40"/>
+      <c r="C281" s="39">
+        <v>516.64</v>
+      </c>
+      <c r="D281" s="40">
+        <v>0</v>
+      </c>
+      <c r="E281" s="42"/>
+      <c r="F281" s="39">
+        <v>1106.2</v>
+      </c>
+      <c r="G281" s="40">
+        <v>0</v>
+      </c>
+      <c r="H281" s="42"/>
+      <c r="I281" s="39">
+        <v>0</v>
+      </c>
+      <c r="J281" s="40">
+        <v>0</v>
+      </c>
       <c r="K281" s="5">
-        <v>1296.2962962962963</v>
+        <v>0</v>
       </c>
       <c r="L281" s="157"/>
       <c r="M281" s="41">
@@ -58360,11 +58689,11 @@
         <v>38572.915000000001</v>
       </c>
       <c r="N2" s="72">
-        <v>8562.24</v>
+        <v>9061.92</v>
       </c>
       <c r="O2" s="29">
         <f>M2-N2</f>
-        <v>30010.675000000003</v>
+        <v>29510.995000000003</v>
       </c>
       <c r="P2" s="29"/>
       <c r="S2">
@@ -58419,15 +58748,15 @@
         <v>292226</v>
       </c>
       <c r="N3" s="72">
-        <v>177188</v>
+        <v>178376</v>
       </c>
       <c r="O3" s="29">
         <f t="shared" ref="O3:O15" si="0">M3-N3</f>
-        <v>115038</v>
+        <v>113850</v>
       </c>
       <c r="P3" s="29"/>
       <c r="R3">
-        <v>5946</v>
+        <v>6293</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -58484,11 +58813,11 @@
       </c>
       <c r="V4" s="193">
         <f>U2*R3</f>
-        <v>8562240</v>
+        <v>9061920</v>
       </c>
       <c r="W4" s="194">
         <f>V4/1000</f>
-        <v>8562.24</v>
+        <v>9061.92</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -59224,7 +59553,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="120" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A10" s="173" t="s">
         <v>21</v>
       </c>
@@ -59247,7 +59576,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="173" t="s">
         <v>282</v>
       </c>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-10-14T08:03:09.372-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="627" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{398F1562-B18C-4C03-900E-1425C63AF87C}"/>
+  <xr:revisionPtr revIDLastSave="705" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CA3825A-27A6-4FBC-8C10-9D42E986BEAC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="398">
   <si>
     <t>ACOMPANHAMENTO SUPERESTRUTURA — FOLHA DE ENTRADA</t>
   </si>
@@ -1462,6 +1462,12 @@
     <t xml:space="preserve">1. Essas locomotivas deverão ser emprestadas pela EFC visto que não há CAPEX previsto e nem locomotivas disponíveis para locação em mercado. 
 17/08: Iniciar tratativas com a EFC. Elaboração de apresentação para reunião nesta semana na EFC - na apresentação deve constar as locomotivas disponíveis na FICO e suas respectivas capacidades de carga. </t>
   </si>
+  <si>
+    <t>Trilho 24m  consumida Barras</t>
+  </si>
+  <si>
+    <t>Trilho 24m  consumida Ton</t>
+  </si>
 </sst>
 </file>
 
@@ -2609,7 +2615,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="212">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3168,6 +3174,7 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4218,7 +4225,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="80">
-        <v>46291</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="12" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4336,7 +4343,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="79">
-        <v>105300</v>
+        <v>107500</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79"/>
@@ -4361,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="D16" s="79">
-        <v>91360</v>
+        <v>100960</v>
       </c>
       <c r="E16" s="78"/>
       <c r="F16" s="79"/>
@@ -4386,7 +4393,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="79">
-        <v>91360</v>
+        <v>97720</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79"/>
@@ -4443,8 +4450,12 @@
       <c r="N18" s="79">
         <v>86970</v>
       </c>
-      <c r="O18" s="78"/>
-      <c r="P18" s="79"/>
+      <c r="O18" s="78">
+        <v>93700</v>
+      </c>
+      <c r="P18" s="79">
+        <v>96800</v>
+      </c>
       <c r="Q18" s="78"/>
       <c r="R18" s="79"/>
     </row>
@@ -4456,7 +4467,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="79">
-        <v>52000</v>
+        <v>54250</v>
       </c>
       <c r="E19" s="78"/>
       <c r="F19" s="79"/>
@@ -4564,7 +4575,7 @@
         <v>50040</v>
       </c>
       <c r="R21" s="79">
-        <v>52000</v>
+        <v>54700</v>
       </c>
     </row>
     <row r="22" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4633,8 +4644,12 @@
       <c r="N23" s="79">
         <v>47010</v>
       </c>
-      <c r="O23" s="78"/>
-      <c r="P23" s="79"/>
+      <c r="O23" s="78">
+        <v>48000</v>
+      </c>
+      <c r="P23" s="79">
+        <v>50240</v>
+      </c>
       <c r="Q23" s="78"/>
       <c r="R23" s="79"/>
     </row>
@@ -4757,7 +4772,7 @@
         <v>23020</v>
       </c>
       <c r="H27" s="79">
-        <v>40086</v>
+        <v>44878</v>
       </c>
       <c r="I27" s="78"/>
       <c r="J27" s="79"/>
@@ -5447,55 +5462,55 @@
       <c r="J5" s="61"/>
       <c r="K5" s="61"/>
       <c r="L5" s="62">
-        <v>6.781286847493076E-2</v>
+        <v>5.9927423404253916E-2</v>
       </c>
       <c r="M5" s="62">
         <f t="shared" ref="M5:X5" si="1">M6-L6</f>
-        <v>8.2269783378556061E-2</v>
+        <v>7.7407601135277837E-2</v>
       </c>
       <c r="N5" s="62">
         <f t="shared" si="1"/>
-        <v>5.3316920765678344E-2</v>
+        <v>5.9545501372358367E-2</v>
       </c>
       <c r="O5" s="62">
         <f t="shared" si="1"/>
-        <v>5.6864394668070473E-2</v>
+        <v>5.6504819574451248E-2</v>
       </c>
       <c r="P5" s="62">
         <f t="shared" si="1"/>
-        <v>5.7008471646305681E-2</v>
+        <v>5.5049969779112196E-2</v>
       </c>
       <c r="Q5" s="62">
         <f t="shared" si="1"/>
-        <v>6.6847314390614532E-2</v>
+        <v>6.6879599404793266E-2</v>
       </c>
       <c r="R5" s="62">
         <f t="shared" si="1"/>
-        <v>6.5773175848752863E-2</v>
+        <v>6.4967958440981466E-2</v>
       </c>
       <c r="S5" s="62">
         <f t="shared" si="1"/>
-        <v>6.5830462848880944E-2</v>
+        <v>6.6572851489322904E-2</v>
       </c>
       <c r="T5" s="62">
         <f t="shared" si="1"/>
-        <v>7.5938391684603368E-2</v>
+        <v>7.5225278014127261E-2</v>
       </c>
       <c r="U5" s="62">
         <f t="shared" si="1"/>
-        <v>5.9193922251732256E-2</v>
+        <v>6.2034254747460493E-2</v>
       </c>
       <c r="V5" s="62">
         <f t="shared" si="1"/>
-        <v>5.5645243385036958E-2</v>
+        <v>5.7645965412102207E-2</v>
       </c>
       <c r="W5" s="62">
         <f t="shared" si="1"/>
-        <v>5.5815010446328528E-2</v>
+        <v>6.0092428488860095E-2</v>
       </c>
       <c r="X5" s="62">
         <f t="shared" si="1"/>
-        <v>4.743998030764196E-3</v>
+        <v>5.2865026797076498E-3</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -5513,43 +5528,43 @@
       <c r="J6" s="61"/>
       <c r="K6" s="61"/>
       <c r="L6" s="62">
-        <v>0.30051286847493075</v>
+        <v>0.29262742340425391</v>
       </c>
       <c r="M6" s="62">
-        <v>0.38278265185348681</v>
+        <v>0.37003502453953174</v>
       </c>
       <c r="N6" s="62">
-        <v>0.43609957261916515</v>
+        <v>0.42958052591189011</v>
       </c>
       <c r="O6" s="62">
-        <v>0.49296396728723563</v>
+        <v>0.48608534548634136</v>
       </c>
       <c r="P6" s="62">
-        <v>0.54997243893354131</v>
+        <v>0.54113531526545355</v>
       </c>
       <c r="Q6" s="62">
-        <v>0.61681975332415584</v>
+        <v>0.60801491467024682</v>
       </c>
       <c r="R6" s="62">
-        <v>0.6825929291729087</v>
+        <v>0.67298287311122829</v>
       </c>
       <c r="S6" s="62">
-        <v>0.74842339202178965</v>
+        <v>0.73955572460055119</v>
       </c>
       <c r="T6" s="62">
-        <v>0.82436178370639301</v>
+        <v>0.81478100261467845</v>
       </c>
       <c r="U6" s="62">
-        <v>0.88355570595812527</v>
+        <v>0.87681525736213894</v>
       </c>
       <c r="V6" s="62">
-        <v>0.93920094934316223</v>
+        <v>0.93446122277424115</v>
       </c>
       <c r="W6" s="62">
-        <v>0.99501595978949076</v>
+        <v>0.99455365126310125</v>
       </c>
       <c r="X6" s="62">
-        <v>0.99975995782025495</v>
+        <v>0.9998401539428089</v>
       </c>
       <c r="Y6" s="83">
         <v>1</v>
@@ -5590,7 +5605,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
       <c r="L7" s="62">
-        <v>3.2000000000000084E-3</v>
+        <v>1.3400000000000023E-2</v>
       </c>
       <c r="M7" s="62"/>
       <c r="N7" s="62"/>
@@ -5651,7 +5666,7 @@
       </c>
       <c r="L8" s="62">
         <f t="shared" si="2"/>
-        <v>0.2359</v>
+        <v>0.24610000000000001</v>
       </c>
       <c r="M8" s="62"/>
       <c r="N8" s="62"/>
@@ -5928,49 +5943,49 @@
       <c r="G14" s="61"/>
       <c r="H14" s="61"/>
       <c r="I14" s="62"/>
-      <c r="J14" s="62">
-        <v>4.1846289897626718E-2</v>
-      </c>
+      <c r="J14" s="62"/>
       <c r="K14" s="62">
-        <v>6.3208252221123126E-2</v>
+        <v>4.4954074588108996E-2</v>
       </c>
       <c r="L14" s="62">
-        <v>7.1195414356986897E-2</v>
+        <v>7.1648778434198451E-2</v>
       </c>
       <c r="M14" s="62">
-        <v>8.188176322115398E-2</v>
+        <v>7.7066110502763491E-2</v>
       </c>
       <c r="N14" s="62">
-        <v>4.8233907822541167E-2</v>
+        <v>5.7820745361437505E-2</v>
       </c>
       <c r="O14" s="62">
-        <v>5.7602435507203731E-2</v>
+        <v>6.0624254963656136E-2</v>
       </c>
       <c r="P14" s="62">
-        <v>5.9597632283525326E-2</v>
+        <v>6.2174397015389411E-2</v>
       </c>
       <c r="Q14" s="62">
-        <v>6.6399322145811235E-2</v>
+        <v>6.6099812139299413E-2</v>
       </c>
       <c r="R14" s="62">
-        <v>6.337337741019422E-2</v>
+        <v>6.4480911441211944E-2</v>
       </c>
       <c r="S14" s="62">
-        <v>6.5918181443970547E-2</v>
+        <v>6.8277429333762393E-2</v>
       </c>
       <c r="T14" s="62">
-        <v>7.6648971764140539E-2</v>
+        <v>7.2910649052511975E-2</v>
       </c>
       <c r="U14" s="62">
-        <v>5.8794301524071946E-2</v>
+        <v>5.2995525304215557E-2</v>
       </c>
       <c r="V14" s="62">
-        <v>5.350472654669014E-2</v>
+        <v>4.8646737309020624E-2</v>
       </c>
       <c r="W14" s="62">
-        <v>5.3740477450843316E-2</v>
-      </c>
-      <c r="X14" s="62"/>
+        <v>4.9575226371953732E-2</v>
+      </c>
+      <c r="X14" s="62">
+        <v>1.9554403958884619E-2</v>
+      </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -5984,65 +5999,61 @@
       <c r="G15" s="61"/>
       <c r="H15" s="61"/>
       <c r="I15" s="62"/>
-      <c r="J15" s="62">
-        <f>J14+I17</f>
-        <v>0.18317094428697323</v>
-      </c>
+      <c r="J15" s="62"/>
       <c r="K15" s="62">
-        <f t="shared" ref="K15:X15" si="3">K14+J15</f>
-        <v>0.24637919650809637</v>
+        <v>0.22812501887508221</v>
       </c>
       <c r="L15" s="62">
-        <f t="shared" si="3"/>
-        <v>0.31757461086508326</v>
+        <f t="shared" ref="K15:X15" si="3">L14+K15</f>
+        <v>0.29977379730928067</v>
       </c>
       <c r="M15" s="62">
         <f t="shared" si="3"/>
-        <v>0.39945637408623724</v>
+        <v>0.37683990781204413</v>
       </c>
       <c r="N15" s="62">
         <f t="shared" si="3"/>
-        <v>0.44769028190877841</v>
+        <v>0.43466065317348163</v>
       </c>
       <c r="O15" s="62">
         <f t="shared" si="3"/>
-        <v>0.50529271741598214</v>
+        <v>0.49528490813713777</v>
       </c>
       <c r="P15" s="62">
         <f t="shared" si="3"/>
-        <v>0.56489034969950747</v>
+        <v>0.55745930515252717</v>
       </c>
       <c r="Q15" s="62">
         <f t="shared" si="3"/>
-        <v>0.6312896718453187</v>
+        <v>0.62355911729182656</v>
       </c>
       <c r="R15" s="62">
         <f t="shared" si="3"/>
-        <v>0.69466304925551292</v>
+        <v>0.68804002873303849</v>
       </c>
       <c r="S15" s="62">
         <f t="shared" si="3"/>
-        <v>0.76058123069948347</v>
+        <v>0.75631745806680084</v>
       </c>
       <c r="T15" s="62">
         <f t="shared" si="3"/>
-        <v>0.83723020246362401</v>
+        <v>0.82922810711931283</v>
       </c>
       <c r="U15" s="62">
         <f t="shared" si="3"/>
-        <v>0.89602450398769595</v>
+        <v>0.88222363242352841</v>
       </c>
       <c r="V15" s="62">
         <f t="shared" si="3"/>
-        <v>0.94952923053438609</v>
+        <v>0.930870369732549</v>
       </c>
       <c r="W15" s="62">
         <f t="shared" si="3"/>
-        <v>1.0032697079852295</v>
+        <v>0.98044559610450277</v>
       </c>
       <c r="X15" s="62">
         <f t="shared" si="3"/>
-        <v>1.0032697079852295</v>
+        <v>1.0000000000633873</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
@@ -6076,7 +6087,9 @@
       <c r="J16" s="62">
         <v>4.1846289897626718E-2</v>
       </c>
-      <c r="K16" s="62"/>
+      <c r="K16" s="62">
+        <v>4.4954074588108996E-2</v>
+      </c>
       <c r="L16" s="62"/>
       <c r="M16" s="62"/>
       <c r="N16" s="62"/>
@@ -6131,7 +6144,9 @@
         <f t="shared" si="4"/>
         <v>0.18317094428697323</v>
       </c>
-      <c r="K17" s="62"/>
+      <c r="K17" s="62">
+        <v>0.22812501887508221</v>
+      </c>
       <c r="L17" s="62"/>
       <c r="M17" s="62"/>
       <c r="N17" s="62"/>
@@ -6363,7 +6378,9 @@
       <c r="K22" s="86">
         <v>229</v>
       </c>
-      <c r="L22" s="86"/>
+      <c r="L22" s="86">
+        <v>227</v>
+      </c>
       <c r="M22" s="62"/>
       <c r="N22" s="62"/>
       <c r="O22" s="62"/>
@@ -6595,7 +6612,9 @@
       <c r="K27" s="87">
         <v>115</v>
       </c>
-      <c r="L27" s="86"/>
+      <c r="L27" s="86">
+        <v>118</v>
+      </c>
       <c r="M27" s="62"/>
       <c r="N27" s="62"/>
       <c r="O27" s="62"/>
@@ -6827,7 +6846,9 @@
       <c r="K32" s="86">
         <v>49</v>
       </c>
-      <c r="L32" s="86"/>
+      <c r="L32" s="86">
+        <v>46</v>
+      </c>
       <c r="M32" s="62"/>
       <c r="N32" s="62"/>
       <c r="O32" s="62"/>
@@ -7059,7 +7080,9 @@
       <c r="K37" s="87">
         <v>46</v>
       </c>
-      <c r="L37" s="87"/>
+      <c r="L37" s="87">
+        <v>49</v>
+      </c>
       <c r="M37" s="62"/>
       <c r="N37" s="62"/>
       <c r="O37" s="62"/>
@@ -27482,7 +27505,7 @@
         <v>1265</v>
       </c>
       <c r="J5" s="68">
-        <v>147</v>
+        <v>345</v>
       </c>
       <c r="K5" s="68"/>
       <c r="L5" s="68"/>
@@ -27541,7 +27564,7 @@
         <v>23</v>
       </c>
       <c r="J6" s="69">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K6" s="69"/>
       <c r="L6" s="69"/>
@@ -27594,7 +27617,7 @@
       </c>
       <c r="J7" s="69">
         <f t="shared" si="2"/>
-        <v>49</v>
+        <v>43.125</v>
       </c>
       <c r="K7" s="69"/>
       <c r="L7" s="69"/>
@@ -27660,34 +27683,34 @@
         <v>1352.8999999999996</v>
       </c>
       <c r="J8" s="147">
-        <v>1406.5</v>
+        <v>1281.3999999999996</v>
       </c>
       <c r="K8" s="147">
-        <v>1259.5</v>
+        <v>1270.8000000000002</v>
       </c>
       <c r="L8" s="147">
-        <v>928.10000000000036</v>
+        <v>936.40000000000055</v>
       </c>
       <c r="M8" s="147">
-        <v>1259.5</v>
+        <v>1270.7999999999993</v>
       </c>
       <c r="N8" s="147">
-        <v>1325.7999999999993</v>
+        <v>1337.7000000000007</v>
       </c>
       <c r="O8" s="147">
-        <v>1524.7000000000007</v>
+        <v>1538.3999999999996</v>
       </c>
       <c r="P8" s="147">
-        <v>1458.3999999999996</v>
+        <v>1471.5</v>
       </c>
       <c r="Q8" s="147">
-        <v>1392.1000000000004</v>
+        <v>1404.6000000000004</v>
       </c>
       <c r="R8" s="147">
-        <v>1458.3999999999996</v>
+        <v>1471.4999999999982</v>
       </c>
       <c r="S8" s="147">
-        <v>1004.0999999999985</v>
+        <v>1034</v>
       </c>
       <c r="T8" s="147">
         <v>0</v>
@@ -27834,43 +27857,43 @@
       </c>
       <c r="J10" s="69">
         <f t="shared" si="5"/>
-        <v>52.092592592592595</v>
+        <v>47.459259259259248</v>
       </c>
       <c r="K10" s="69">
         <f t="shared" si="5"/>
-        <v>50.38</v>
+        <v>50.832000000000008</v>
       </c>
       <c r="L10" s="69">
         <f t="shared" si="5"/>
-        <v>58.006250000000023</v>
+        <v>58.525000000000034</v>
       </c>
       <c r="M10" s="69">
         <f t="shared" si="5"/>
-        <v>52.479166666666664</v>
+        <v>52.949999999999967</v>
       </c>
       <c r="N10" s="69">
         <f t="shared" si="5"/>
-        <v>55.241666666666639</v>
+        <v>55.737500000000033</v>
       </c>
       <c r="O10" s="69">
         <f t="shared" si="5"/>
-        <v>56.470370370370397</v>
+        <v>56.977777777777767</v>
       </c>
       <c r="P10" s="69">
         <f t="shared" si="5"/>
-        <v>56.092307692307678</v>
+        <v>56.596153846153847</v>
       </c>
       <c r="Q10" s="69">
         <f t="shared" si="5"/>
-        <v>53.542307692307709</v>
+        <v>54.023076923076935</v>
       </c>
       <c r="R10" s="69">
         <f t="shared" si="5"/>
-        <v>56.092307692307678</v>
+        <v>56.596153846153776</v>
       </c>
       <c r="S10" s="69">
         <f t="shared" si="5"/>
-        <v>37.188888888888833</v>
+        <v>38.296296296296298</v>
       </c>
       <c r="T10" s="69">
         <f t="shared" si="5"/>
@@ -28253,7 +28276,9 @@
       <c r="I16" s="153">
         <v>13615</v>
       </c>
-      <c r="J16" s="153"/>
+      <c r="J16" s="153">
+        <v>2200</v>
+      </c>
       <c r="K16" s="153"/>
       <c r="L16" s="153"/>
       <c r="M16" s="153"/>
@@ -28296,7 +28321,9 @@
       <c r="I17" s="69">
         <v>17</v>
       </c>
-      <c r="J17" s="69"/>
+      <c r="J17" s="69">
+        <v>4</v>
+      </c>
       <c r="K17" s="69"/>
       <c r="L17" s="69"/>
       <c r="M17" s="69"/>
@@ -28319,7 +28346,7 @@
         <v>150.33333333333334</v>
       </c>
       <c r="C18" s="69">
-        <f t="shared" ref="C18:I18" si="7">IFERROR(C16/C17,0)</f>
+        <f t="shared" ref="C18:J18" si="7">IFERROR(C16/C17,0)</f>
         <v>551.21428571428567</v>
       </c>
       <c r="D18" s="69">
@@ -28346,7 +28373,10 @@
         <f t="shared" si="7"/>
         <v>800.88235294117646</v>
       </c>
-      <c r="J18" s="69"/>
+      <c r="J18" s="69">
+        <f t="shared" si="7"/>
+        <v>550</v>
+      </c>
       <c r="K18" s="69"/>
       <c r="L18" s="69"/>
       <c r="M18" s="69"/>
@@ -28395,37 +28425,37 @@
         <v>13615</v>
       </c>
       <c r="J19" s="147">
-        <v>22273.800000000003</v>
+        <v>17270.899999999994</v>
       </c>
       <c r="K19" s="147">
-        <v>17983.499999999985</v>
+        <v>18600.5</v>
       </c>
       <c r="L19" s="147">
-        <v>12729.600000000006</v>
+        <v>12540.5</v>
       </c>
       <c r="M19" s="147">
-        <v>17684.899999999994</v>
+        <v>17578.5</v>
       </c>
       <c r="N19" s="147">
-        <v>18621.899999999994</v>
+        <v>18649.200000000012</v>
       </c>
       <c r="O19" s="147">
         <v>21409.799999999988</v>
       </c>
       <c r="P19" s="147">
-        <v>20509.700000000012</v>
+        <v>20501.299999999988</v>
       </c>
       <c r="Q19" s="147">
-        <v>19846.899999999994</v>
+        <v>19767.299999999988</v>
       </c>
       <c r="R19" s="147">
-        <v>20484.799999999988</v>
+        <v>20571.399999999994</v>
       </c>
       <c r="S19" s="147">
         <v>20484.799999999988</v>
       </c>
       <c r="T19" s="147">
-        <v>13594.799999999988</v>
+        <v>18250.299999999988</v>
       </c>
       <c r="U19" s="147">
         <v>0</v>
@@ -28548,23 +28578,23 @@
       </c>
       <c r="J21" s="69">
         <f t="shared" si="10"/>
-        <v>824.95555555555563</v>
+        <v>639.66296296296275</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="10"/>
-        <v>719.33999999999946</v>
+        <v>744.02</v>
       </c>
       <c r="L21" s="69">
         <f t="shared" si="10"/>
-        <v>795.60000000000036</v>
+        <v>783.78125</v>
       </c>
       <c r="M21" s="69">
         <f t="shared" si="10"/>
-        <v>736.87083333333305</v>
+        <v>732.4375</v>
       </c>
       <c r="N21" s="69">
         <f t="shared" si="10"/>
-        <v>775.9124999999998</v>
+        <v>777.05000000000052</v>
       </c>
       <c r="O21" s="69">
         <f t="shared" si="10"/>
@@ -28572,15 +28602,15 @@
       </c>
       <c r="P21" s="69">
         <f t="shared" si="10"/>
-        <v>788.83461538461586</v>
+        <v>788.51153846153807</v>
       </c>
       <c r="Q21" s="69">
         <f t="shared" si="10"/>
-        <v>763.34230769230749</v>
+        <v>760.28076923076878</v>
       </c>
       <c r="R21" s="69">
         <f t="shared" si="10"/>
-        <v>787.87692307692259</v>
+        <v>791.20769230769213</v>
       </c>
       <c r="S21" s="69">
         <f t="shared" si="10"/>
@@ -28588,7 +28618,7 @@
       </c>
       <c r="T21" s="69">
         <f t="shared" si="10"/>
-        <v>522.87692307692259</v>
+        <v>701.93461538461497</v>
       </c>
       <c r="U21" s="69">
         <f t="shared" si="10"/>
@@ -28922,7 +28952,7 @@
         <v>36285</v>
       </c>
       <c r="J27" s="68">
-        <v>7348</v>
+        <v>23447.999799999991</v>
       </c>
       <c r="K27" s="68" t="s">
         <v>196</v>
@@ -28991,7 +29021,7 @@
         <v>13</v>
       </c>
       <c r="J28" s="69">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K28" s="69"/>
       <c r="L28" s="69"/>
@@ -29044,7 +29074,7 @@
       </c>
       <c r="J29" s="69">
         <f t="shared" si="12"/>
-        <v>3674</v>
+        <v>3349.7142571428558</v>
       </c>
       <c r="K29" s="69"/>
       <c r="L29" s="69"/>
@@ -29094,40 +29124,40 @@
         <v>36285</v>
       </c>
       <c r="J30" s="147">
-        <v>55457.799999999988</v>
+        <v>52942.099799999996</v>
       </c>
       <c r="K30" s="147">
-        <v>45223.200000000012</v>
+        <v>40066.499999999971</v>
       </c>
       <c r="L30" s="147">
-        <v>36609.5</v>
+        <v>39282.099999999977</v>
       </c>
       <c r="M30" s="147">
-        <v>38266.299999999988</v>
+        <v>37845.799999999988</v>
       </c>
       <c r="N30" s="147">
-        <v>49823.700000000012</v>
+        <v>38516.099999999977</v>
       </c>
       <c r="O30" s="147">
-        <v>50217.700000000012</v>
+        <v>54697.099999999977</v>
       </c>
       <c r="P30" s="147">
-        <v>47717.900000000023</v>
+        <v>42693.400000000023</v>
       </c>
       <c r="Q30" s="147">
-        <v>52575.700000000012</v>
+        <v>56337.500000000058</v>
       </c>
       <c r="R30" s="147">
-        <v>48370.599999999977</v>
+        <v>50576.800000000047</v>
       </c>
       <c r="S30" s="147">
-        <v>36785.800000000047</v>
+        <v>38266.5</v>
       </c>
       <c r="T30" s="147">
-        <v>49910.900000000023</v>
+        <v>50911.800000000047</v>
       </c>
       <c r="U30" s="147">
-        <v>47310.799999999814</v>
+        <v>56134.200199999847</v>
       </c>
       <c r="V30" s="147">
         <v>0</v>
@@ -29247,51 +29277,51 @@
       </c>
       <c r="J32" s="69">
         <f t="shared" si="15"/>
-        <v>2053.9925925925922</v>
+        <v>1960.8185111111109</v>
       </c>
       <c r="K32" s="69">
         <f t="shared" si="15"/>
-        <v>1808.9280000000006</v>
+        <v>1602.6599999999989</v>
       </c>
       <c r="L32" s="69">
         <f t="shared" si="15"/>
-        <v>2288.09375</v>
+        <v>2455.1312499999985</v>
       </c>
       <c r="M32" s="69">
         <f t="shared" si="15"/>
-        <v>1594.4291666666661</v>
+        <v>1576.9083333333328</v>
       </c>
       <c r="N32" s="69">
         <f t="shared" si="15"/>
-        <v>2075.9875000000006</v>
+        <v>1604.837499999999</v>
       </c>
       <c r="O32" s="69">
         <f t="shared" si="15"/>
-        <v>1859.9148148148151</v>
+        <v>2025.8185185185177</v>
       </c>
       <c r="P32" s="69">
         <f t="shared" si="15"/>
-        <v>1835.303846153847</v>
+        <v>1642.053846153847</v>
       </c>
       <c r="Q32" s="69">
         <f t="shared" si="15"/>
-        <v>2022.1423076923081</v>
+        <v>2166.8269230769251</v>
       </c>
       <c r="R32" s="69">
         <f t="shared" si="15"/>
-        <v>1860.4076923076914</v>
+        <v>1945.2615384615403</v>
       </c>
       <c r="S32" s="69">
         <f t="shared" si="15"/>
-        <v>1362.4370370370389</v>
+        <v>1417.2777777777778</v>
       </c>
       <c r="T32" s="69">
         <f t="shared" si="15"/>
-        <v>1919.650000000001</v>
+        <v>1958.1461538461556</v>
       </c>
       <c r="U32" s="69">
         <f t="shared" si="15"/>
-        <v>1819.6461538461467</v>
+        <v>2159.0076999999942</v>
       </c>
       <c r="V32" s="69">
         <v>0</v>
@@ -29621,7 +29651,7 @@
         <v>119</v>
       </c>
       <c r="J38" s="68">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="K38" s="68" t="s">
         <v>196</v>
@@ -29690,7 +29720,7 @@
         <v>22</v>
       </c>
       <c r="J39" s="69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K39" s="69"/>
       <c r="L39" s="69"/>
@@ -29791,22 +29821,22 @@
         <v>132.20000000000005</v>
       </c>
       <c r="J41" s="147">
-        <v>272.79999999999995</v>
+        <v>272.5</v>
       </c>
       <c r="K41" s="147">
         <v>196.39999999999998</v>
       </c>
       <c r="L41" s="147">
-        <v>186.99999999999989</v>
+        <v>186.89999999999998</v>
       </c>
       <c r="M41" s="147">
-        <v>213.5</v>
+        <v>213.40000000000009</v>
       </c>
       <c r="N41" s="147">
-        <v>158.09999999999991</v>
+        <v>158.20000000000005</v>
       </c>
       <c r="O41" s="147">
-        <v>226.90000000000009</v>
+        <v>227</v>
       </c>
       <c r="P41" s="147">
         <v>261.69999999999982</v>
@@ -29818,16 +29848,16 @@
         <v>288.09999999999991</v>
       </c>
       <c r="S41" s="147">
-        <v>330.90000000000009</v>
+        <v>276.19999999999982</v>
       </c>
       <c r="T41" s="147">
-        <v>261.40000000000009</v>
+        <v>297.09999999999991</v>
       </c>
       <c r="U41" s="147">
-        <v>80.900000000000091</v>
+        <v>104.40000000000009</v>
       </c>
       <c r="V41" s="147">
-        <v>9.3000000000001819</v>
+        <v>5.3000000000001819</v>
       </c>
       <c r="X41" s="148"/>
     </row>
@@ -29944,7 +29974,7 @@
       </c>
       <c r="J43" s="69">
         <f t="shared" si="20"/>
-        <v>10.103703703703703</v>
+        <v>10.092592592592593</v>
       </c>
       <c r="K43" s="69">
         <f t="shared" si="20"/>
@@ -29952,19 +29982,19 @@
       </c>
       <c r="L43" s="69">
         <f t="shared" si="20"/>
-        <v>11.687499999999993</v>
+        <v>11.681249999999999</v>
       </c>
       <c r="M43" s="69">
         <f t="shared" si="20"/>
-        <v>8.8958333333333339</v>
+        <v>8.891666666666671</v>
       </c>
       <c r="N43" s="69">
         <f t="shared" si="20"/>
-        <v>6.5874999999999959</v>
+        <v>6.5916666666666686</v>
       </c>
       <c r="O43" s="69">
         <f t="shared" si="20"/>
-        <v>8.403703703703707</v>
+        <v>8.4074074074074066</v>
       </c>
       <c r="P43" s="69">
         <f t="shared" si="20"/>
@@ -29980,15 +30010,15 @@
       </c>
       <c r="S43" s="69">
         <f t="shared" si="20"/>
-        <v>12.255555555555558</v>
+        <v>10.229629629629622</v>
       </c>
       <c r="T43" s="69">
         <f t="shared" si="20"/>
-        <v>10.053846153846157</v>
+        <v>11.426923076923073</v>
       </c>
       <c r="U43" s="69">
         <f t="shared" si="20"/>
-        <v>3.1115384615384651</v>
+        <v>4.0153846153846189</v>
       </c>
       <c r="V43" s="69">
         <v>0</v>
@@ -30318,7 +30348,7 @@
         <v>18166</v>
       </c>
       <c r="J49" s="68">
-        <v>1450</v>
+        <v>5228</v>
       </c>
       <c r="K49" s="68" t="s">
         <v>196</v>
@@ -30387,7 +30417,7 @@
         <v>17</v>
       </c>
       <c r="J50" s="69">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K50" s="69"/>
       <c r="L50" s="69"/>
@@ -30440,7 +30470,7 @@
       </c>
       <c r="J51" s="69">
         <f t="shared" si="22"/>
-        <v>483.33333333333331</v>
+        <v>580.88888888888891</v>
       </c>
       <c r="K51" s="69"/>
       <c r="L51" s="69"/>
@@ -30490,40 +30520,40 @@
         <v>19854.100000000006</v>
       </c>
       <c r="J52" s="147">
-        <v>21512.800000000003</v>
+        <v>18746.699999999997</v>
       </c>
       <c r="K52" s="147">
-        <v>33846.800000000003</v>
+        <v>31552.5</v>
       </c>
       <c r="L52" s="147">
-        <v>17470.700000000012</v>
+        <v>17193.699999999997</v>
       </c>
       <c r="M52" s="147">
-        <v>10765.700000000012</v>
+        <v>11341.399999999994</v>
       </c>
       <c r="N52" s="147">
-        <v>12574.5</v>
+        <v>13326.5</v>
       </c>
       <c r="O52" s="147">
-        <v>18857.700000000012</v>
+        <v>17954.399999999994</v>
       </c>
       <c r="P52" s="147">
-        <v>19841.200000000012</v>
+        <v>16952.5</v>
       </c>
       <c r="Q52" s="147">
-        <v>21669.899999999994</v>
+        <v>24331.799999999988</v>
       </c>
       <c r="R52" s="147">
-        <v>23715.899999999994</v>
+        <v>22964</v>
       </c>
       <c r="S52" s="147">
-        <v>10968.200000000012</v>
+        <v>12742.899999999994</v>
       </c>
       <c r="T52" s="147">
-        <v>19240.699999999983</v>
+        <v>20111.599999999977</v>
       </c>
       <c r="U52" s="147">
-        <v>31189.099999999919</v>
+        <v>34435.200000000012</v>
       </c>
       <c r="V52" s="147"/>
       <c r="X52" s="148"/>
@@ -30641,51 +30671,51 @@
       </c>
       <c r="J54" s="69">
         <f t="shared" si="25"/>
-        <v>796.77037037037053</v>
+        <v>694.32222222222208</v>
       </c>
       <c r="K54" s="69">
         <f t="shared" si="25"/>
-        <v>1353.8720000000001</v>
+        <v>1262.0999999999999</v>
       </c>
       <c r="L54" s="69">
         <f t="shared" si="25"/>
-        <v>1091.9187500000007</v>
+        <v>1074.6062499999998</v>
       </c>
       <c r="M54" s="69">
         <f t="shared" si="25"/>
-        <v>448.57083333333384</v>
+        <v>472.55833333333311</v>
       </c>
       <c r="N54" s="69">
         <f t="shared" si="25"/>
-        <v>523.9375</v>
+        <v>555.27083333333337</v>
       </c>
       <c r="O54" s="69">
         <f t="shared" si="25"/>
-        <v>698.43333333333374</v>
+        <v>664.97777777777753</v>
       </c>
       <c r="P54" s="69">
         <f t="shared" si="25"/>
-        <v>763.12307692307741</v>
+        <v>652.01923076923072</v>
       </c>
       <c r="Q54" s="69">
         <f t="shared" si="25"/>
-        <v>833.45769230769213</v>
+        <v>935.83846153846105</v>
       </c>
       <c r="R54" s="69">
         <f t="shared" si="25"/>
-        <v>912.14999999999975</v>
+        <v>883.23076923076928</v>
       </c>
       <c r="S54" s="69">
         <f t="shared" si="25"/>
-        <v>406.22962962963004</v>
+        <v>471.95925925925906</v>
       </c>
       <c r="T54" s="69">
         <f t="shared" si="25"/>
-        <v>740.02692307692246</v>
+        <v>773.52307692307602</v>
       </c>
       <c r="U54" s="69">
         <f t="shared" si="25"/>
-        <v>1199.580769230766</v>
+        <v>1324.4307692307698</v>
       </c>
       <c r="V54" s="69">
         <f t="shared" si="25"/>
@@ -31016,7 +31046,7 @@
         <v>32756</v>
       </c>
       <c r="J60" s="68">
-        <v>2299</v>
+        <v>11884</v>
       </c>
       <c r="K60" s="68" t="s">
         <v>196</v>
@@ -31085,7 +31115,7 @@
         <v>15</v>
       </c>
       <c r="J61" s="69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K61" s="69"/>
       <c r="L61" s="69"/>
@@ -31137,7 +31167,7 @@
       </c>
       <c r="J62" s="69">
         <f>J60/J61</f>
-        <v>2299</v>
+        <v>1980.6666666666667</v>
       </c>
       <c r="K62" s="69"/>
       <c r="L62" s="69"/>
@@ -31186,43 +31216,43 @@
         <v>35224.199999999997</v>
       </c>
       <c r="J63" s="147">
-        <v>45728.5</v>
+        <v>45335.100000000006</v>
       </c>
       <c r="K63" s="147">
-        <v>50769.200000000012</v>
+        <v>50722.600000000006</v>
       </c>
       <c r="L63" s="147">
-        <v>39510.100000000006</v>
+        <v>39424.899999999994</v>
       </c>
       <c r="M63" s="147">
-        <v>44845.800000000017</v>
+        <v>44912.800000000017</v>
       </c>
       <c r="N63" s="147">
-        <v>34939.299999999988</v>
+        <v>35005.799999999988</v>
       </c>
       <c r="O63" s="147">
-        <v>44051.200000000012</v>
+        <v>44107.700000000012</v>
       </c>
       <c r="P63" s="147">
-        <v>47004.400000000023</v>
+        <v>47008</v>
       </c>
       <c r="Q63" s="147">
         <v>49998.700000000012</v>
       </c>
       <c r="R63" s="147">
-        <v>50818.5</v>
+        <v>50799.700000000012</v>
       </c>
       <c r="S63" s="147">
-        <v>52431.700000000012</v>
+        <v>52461</v>
       </c>
       <c r="T63" s="147">
-        <v>36387.700000000012</v>
+        <v>37247.099999999977</v>
       </c>
       <c r="U63" s="147">
-        <v>47263.099999999977</v>
+        <v>77263.099999999977</v>
       </c>
       <c r="V63" s="147">
-        <v>32415.79999999993</v>
+        <v>1877.9000000000233</v>
       </c>
       <c r="X63" s="148"/>
     </row>
@@ -31339,31 +31369,31 @@
       </c>
       <c r="J65" s="69">
         <f t="shared" si="29"/>
-        <v>1693.648148148148</v>
+        <v>1679.077777777778</v>
       </c>
       <c r="K65" s="69">
         <f t="shared" si="29"/>
-        <v>2030.7680000000005</v>
+        <v>2028.9040000000002</v>
       </c>
       <c r="L65" s="69">
         <f t="shared" si="29"/>
-        <v>2469.3812500000004</v>
+        <v>2464.0562499999996</v>
       </c>
       <c r="M65" s="69">
         <f t="shared" si="29"/>
-        <v>1868.5750000000007</v>
+        <v>1871.3666666666675</v>
       </c>
       <c r="N65" s="69">
         <f t="shared" si="29"/>
-        <v>1455.8041666666661</v>
+        <v>1458.5749999999996</v>
       </c>
       <c r="O65" s="69">
         <f t="shared" si="29"/>
-        <v>1631.5259259259265</v>
+        <v>1633.6185185185188</v>
       </c>
       <c r="P65" s="69">
         <f t="shared" si="29"/>
-        <v>1807.8615384615393</v>
+        <v>1808</v>
       </c>
       <c r="Q65" s="69">
         <f t="shared" si="29"/>
@@ -31371,19 +31401,19 @@
       </c>
       <c r="R65" s="69">
         <f t="shared" si="29"/>
-        <v>1954.5576923076924</v>
+        <v>1953.8346153846157</v>
       </c>
       <c r="S65" s="69">
         <f t="shared" si="29"/>
-        <v>1941.9148148148151</v>
+        <v>1943</v>
       </c>
       <c r="T65" s="69">
         <f t="shared" si="29"/>
-        <v>1399.5269230769236</v>
+        <v>1432.5807692307683</v>
       </c>
       <c r="U65" s="69">
         <f t="shared" si="29"/>
-        <v>1817.8115384615376</v>
+        <v>2971.6576923076914</v>
       </c>
       <c r="V65" s="69">
         <v>0</v>
@@ -31451,47 +31481,47 @@
       <c r="B2" s="46"/>
       <c r="C2" s="34">
         <f>SUM(C4:C733)</f>
-        <v>140861.58000000002</v>
+        <v>145839</v>
       </c>
       <c r="D2" s="35">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>140757.66000000006</v>
+        <v>142103.58000000007</v>
       </c>
       <c r="E2" s="36">
         <f t="shared" si="0"/>
-        <v>12503.916923076924</v>
+        <v>8038.2323076923085</v>
       </c>
       <c r="F2" s="34">
         <f t="shared" si="0"/>
-        <v>205357.03699999992</v>
+        <v>210259.08699999994</v>
       </c>
       <c r="G2" s="35">
         <f t="shared" si="0"/>
-        <v>203362.47999999998</v>
+        <v>208717.13999999998</v>
       </c>
       <c r="H2" s="36">
         <f t="shared" si="0"/>
-        <v>16958.866153846153</v>
+        <v>7537.2738461538447</v>
       </c>
       <c r="I2" s="34">
         <f t="shared" si="0"/>
-        <v>11968.449999999999</v>
+        <v>17301.32</v>
       </c>
       <c r="J2" s="35">
         <f t="shared" si="0"/>
-        <v>16608.355980999997</v>
+        <v>19955.665981000002</v>
       </c>
       <c r="K2" s="36">
         <f t="shared" si="0"/>
-        <v>579814.81481481565</v>
+        <v>573333.3333333343</v>
       </c>
       <c r="L2" s="34">
         <f t="shared" si="0"/>
-        <v>345297.78222199978</v>
+        <v>367929.76222199976</v>
       </c>
       <c r="M2" s="36">
         <f t="shared" si="0"/>
-        <v>662619.65655555553</v>
+        <v>647186.7336666669</v>
       </c>
       <c r="N2" s="29"/>
     </row>
@@ -31691,11 +31721,11 @@
       </c>
       <c r="Y5" s="5">
         <f t="shared" si="2"/>
-        <v>73069.385980999999</v>
+        <v>73254.095980999991</v>
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
-        <v>7568.1900000000005</v>
+        <v>17431.370000000003</v>
       </c>
       <c r="AA5" s="5">
         <f t="shared" si="2"/>
@@ -31782,7 +31812,7 @@
       </c>
       <c r="Z6" s="5">
         <f t="shared" si="4"/>
-        <v>59277.597891737882</v>
+        <v>38908.839487179481</v>
       </c>
       <c r="AA6" s="5">
         <f t="shared" si="4"/>
@@ -31909,7 +31939,7 @@
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="5"/>
-        <v>10778.059999999998</v>
+        <v>33410.039999999994</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="5"/>
@@ -31996,7 +32026,7 @@
       </c>
       <c r="Z9" s="5">
         <f t="shared" si="6"/>
-        <v>61731.691555555582</v>
+        <v>46298.768666666678</v>
       </c>
       <c r="AA9" s="5">
         <f t="shared" si="6"/>
@@ -32119,19 +32149,19 @@
       </c>
       <c r="Y11" s="5">
         <f t="shared" si="7"/>
-        <v>353160.30598099995</v>
+        <v>353345.01598099997</v>
       </c>
       <c r="Z11" s="5">
         <f t="shared" si="7"/>
-        <v>420006.09387273784</v>
+        <v>409685.22546817944</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="7"/>
-        <v>470006.09387273784</v>
+        <v>459685.22546817944</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="7"/>
-        <v>520006.09387273784</v>
+        <v>509685.22546817944</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
@@ -32210,15 +32240,15 @@
       </c>
       <c r="Z12" s="5">
         <f t="shared" si="8"/>
-        <v>407029.47377755563</v>
+        <v>414228.53088866669</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="8"/>
-        <v>474335.35877755558</v>
+        <v>481534.41588866664</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="8"/>
-        <v>510581.69377755554</v>
+        <v>517780.7508886666</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -32293,19 +32323,19 @@
       </c>
       <c r="Y13" s="5">
         <f t="shared" si="9"/>
-        <v>18640.583758999943</v>
+        <v>18825.293758999964</v>
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>12976.62009518221</v>
+        <v>-4543.305420487246</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
-        <v>-4329.2649048177409</v>
+        <v>-21849.190420487197</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>9424.4000951822964</v>
+        <v>-8095.5254204871599</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
@@ -42148,7 +42178,7 @@
       </c>
       <c r="H260" s="42"/>
       <c r="I260" s="39">
-        <v>1118</v>
+        <v>1210.6300000000001</v>
       </c>
       <c r="J260" s="40">
         <v>0</v>
@@ -42190,7 +42220,7 @@
       </c>
       <c r="H261" s="42"/>
       <c r="I261" s="39">
-        <v>445</v>
+        <v>537.63</v>
       </c>
       <c r="J261" s="40">
         <v>401.78</v>
@@ -42232,7 +42262,7 @@
       </c>
       <c r="H262" s="42"/>
       <c r="I262" s="39">
-        <v>722</v>
+        <v>814.63</v>
       </c>
       <c r="J262" s="40">
         <v>669.67598100000009</v>
@@ -42274,7 +42304,7 @@
       </c>
       <c r="H263" s="42"/>
       <c r="I263" s="39">
-        <v>925</v>
+        <v>1017.63</v>
       </c>
       <c r="J263" s="40">
         <v>987.55999999999983</v>
@@ -42316,7 +42346,7 @@
       </c>
       <c r="H264" s="42"/>
       <c r="I264" s="39">
-        <v>245</v>
+        <v>337.63</v>
       </c>
       <c r="J264" s="40">
         <v>771.46999999999991</v>
@@ -42442,7 +42472,7 @@
       </c>
       <c r="H267" s="42"/>
       <c r="I267" s="39">
-        <v>701</v>
+        <v>793.63</v>
       </c>
       <c r="J267" s="40">
         <v>229.29000000000002</v>
@@ -42484,7 +42514,7 @@
       </c>
       <c r="H268" s="42"/>
       <c r="I268" s="39">
-        <v>329</v>
+        <v>421.63</v>
       </c>
       <c r="J268" s="40">
         <v>833.75000000000023</v>
@@ -42526,7 +42556,7 @@
       </c>
       <c r="H269" s="42"/>
       <c r="I269" s="39">
-        <v>974</v>
+        <v>1066.6300000000001</v>
       </c>
       <c r="J269" s="40">
         <v>910.9699999999998</v>
@@ -42568,7 +42598,7 @@
       </c>
       <c r="H270" s="42"/>
       <c r="I270" s="39">
-        <v>455</v>
+        <v>547.63</v>
       </c>
       <c r="J270" s="40">
         <v>1356.5700000000004</v>
@@ -42610,7 +42640,7 @@
       </c>
       <c r="H271" s="42"/>
       <c r="I271" s="39">
-        <v>567.20000000000005</v>
+        <v>659.83</v>
       </c>
       <c r="J271" s="40">
         <v>1490.87</v>
@@ -42652,10 +42682,10 @@
       </c>
       <c r="H272" s="42"/>
       <c r="I272" s="39">
-        <v>507</v>
+        <v>599.63</v>
       </c>
       <c r="J272" s="40">
-        <v>706.05</v>
+        <v>857.18999999999994</v>
       </c>
       <c r="K272" s="5">
         <v>0</v>
@@ -42736,7 +42766,7 @@
       </c>
       <c r="H274" s="42"/>
       <c r="I274" s="39">
-        <v>782</v>
+        <v>874.63</v>
       </c>
       <c r="J274" s="40">
         <v>2330.4899999999993</v>
@@ -42778,7 +42808,7 @@
       </c>
       <c r="H275" s="42"/>
       <c r="I275" s="39">
-        <v>1344.9</v>
+        <v>1437.5300000000002</v>
       </c>
       <c r="J275" s="40">
         <v>1529.65</v>
@@ -42820,10 +42850,10 @@
       </c>
       <c r="H276" s="42"/>
       <c r="I276" s="39">
-        <v>922.7</v>
+        <v>1015.33</v>
       </c>
       <c r="J276" s="40">
-        <v>2063.6</v>
+        <v>2097.17</v>
       </c>
       <c r="K276" s="5">
         <v>0</v>
@@ -42862,7 +42892,7 @@
       </c>
       <c r="H277" s="42"/>
       <c r="I277" s="39">
-        <v>934.25</v>
+        <v>1026.8800000000001</v>
       </c>
       <c r="J277" s="40">
         <v>1286.47</v>
@@ -42904,7 +42934,7 @@
       </c>
       <c r="H278" s="42"/>
       <c r="I278" s="39">
-        <v>70</v>
+        <v>162.63</v>
       </c>
       <c r="J278" s="40">
         <v>654.12</v>
@@ -42997,9 +43027,7 @@
         <v>0</v>
       </c>
       <c r="L280" s="157"/>
-      <c r="M280" s="41">
-        <v>0</v>
-      </c>
+      <c r="M280" s="41"/>
       <c r="O280" s="29"/>
       <c r="P280" s="5"/>
       <c r="R280" s="5"/>
@@ -43030,7 +43058,7 @@
       </c>
       <c r="H281" s="42"/>
       <c r="I281" s="39">
-        <v>0</v>
+        <v>1014.6</v>
       </c>
       <c r="J281" s="40">
         <v>0</v>
@@ -43038,10 +43066,10 @@
       <c r="K281" s="5">
         <v>0</v>
       </c>
-      <c r="L281" s="157"/>
-      <c r="M281" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+      <c r="L281" s="157">
+        <v>2032.1799999999998</v>
+      </c>
+      <c r="M281" s="41"/>
       <c r="O281" s="29"/>
       <c r="P281" s="5"/>
       <c r="R281" s="5"/>
@@ -43057,25 +43085,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C282" s="39"/>
-      <c r="D282" s="40"/>
-      <c r="E282" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F282" s="39"/>
-      <c r="G282" s="40"/>
-      <c r="H282" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I282" s="39"/>
-      <c r="J282" s="40"/>
+      <c r="C282" s="39">
+        <v>1424.12</v>
+      </c>
+      <c r="D282" s="40">
+        <v>1135.1600000000001</v>
+      </c>
+      <c r="E282" s="42"/>
+      <c r="F282" s="39">
+        <v>762.54</v>
+      </c>
+      <c r="G282" s="40">
+        <v>1122.8799999999999</v>
+      </c>
+      <c r="H282" s="42"/>
+      <c r="I282" s="39">
+        <v>479</v>
+      </c>
+      <c r="J282" s="40">
+        <v>655.45000000000016</v>
+      </c>
       <c r="K282" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L282" s="157"/>
-      <c r="M282" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L282" s="157">
+        <v>5231.96</v>
+      </c>
+      <c r="M282" s="41"/>
       <c r="O282" s="29"/>
       <c r="P282" s="5"/>
       <c r="R282" s="5"/>
@@ -43091,25 +43127,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C283" s="39"/>
-      <c r="D283" s="40"/>
-      <c r="E283" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F283" s="39"/>
-      <c r="G283" s="40"/>
-      <c r="H283" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I283" s="39"/>
-      <c r="J283" s="40"/>
+      <c r="C283" s="39">
+        <v>1847</v>
+      </c>
+      <c r="D283" s="40">
+        <v>210.76</v>
+      </c>
+      <c r="E283" s="42"/>
+      <c r="F283" s="39">
+        <v>872.65</v>
+      </c>
+      <c r="G283" s="40">
+        <v>1839.6199999999997</v>
+      </c>
+      <c r="H283" s="42"/>
+      <c r="I283" s="39">
+        <v>173.4</v>
+      </c>
+      <c r="J283" s="40">
+        <v>1106.1799999999998</v>
+      </c>
       <c r="K283" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L283" s="157"/>
-      <c r="M283" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L283" s="157">
+        <v>0</v>
+      </c>
+      <c r="M283" s="41"/>
       <c r="O283" s="29"/>
       <c r="P283" s="5"/>
       <c r="R283" s="5"/>
@@ -43125,25 +43169,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C284" s="39"/>
-      <c r="D284" s="40"/>
-      <c r="E284" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F284" s="39"/>
-      <c r="G284" s="40"/>
-      <c r="H284" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I284" s="39"/>
-      <c r="J284" s="40"/>
+      <c r="C284" s="39">
+        <v>557.92999999999995</v>
+      </c>
+      <c r="D284" s="40">
+        <v>0</v>
+      </c>
+      <c r="E284" s="42"/>
+      <c r="F284" s="39">
+        <v>1658.45</v>
+      </c>
+      <c r="G284" s="40">
+        <v>770.12000000000012</v>
+      </c>
+      <c r="H284" s="42"/>
+      <c r="I284" s="39">
+        <v>1006.27</v>
+      </c>
+      <c r="J284" s="40">
+        <v>481.00000000000011</v>
+      </c>
       <c r="K284" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L284" s="157"/>
-      <c r="M284" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L284" s="157">
+        <v>6780.4199999999992</v>
+      </c>
+      <c r="M284" s="41"/>
       <c r="O284" s="29"/>
       <c r="P284" s="5"/>
       <c r="R284" s="5"/>
@@ -43159,25 +43211,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C285" s="39"/>
-      <c r="D285" s="40"/>
-      <c r="E285" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F285" s="39"/>
-      <c r="G285" s="40"/>
-      <c r="H285" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I285" s="39"/>
-      <c r="J285" s="40"/>
+      <c r="C285" s="39">
+        <v>511.58</v>
+      </c>
+      <c r="D285" s="40">
+        <v>0</v>
+      </c>
+      <c r="E285" s="42"/>
+      <c r="F285" s="39">
+        <v>1189.27</v>
+      </c>
+      <c r="G285" s="40">
+        <v>700.99999999999989</v>
+      </c>
+      <c r="H285" s="42"/>
+      <c r="I285" s="39">
+        <v>679.1</v>
+      </c>
+      <c r="J285" s="40">
+        <v>519.79000000000008</v>
+      </c>
       <c r="K285" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L285" s="157"/>
-      <c r="M285" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L285" s="157">
+        <v>764.5</v>
+      </c>
+      <c r="M285" s="41"/>
       <c r="O285" s="29"/>
       <c r="P285" s="5"/>
       <c r="R285" s="5"/>
@@ -43193,25 +43253,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C286" s="39"/>
-      <c r="D286" s="40"/>
-      <c r="E286" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F286" s="39"/>
-      <c r="G286" s="40"/>
-      <c r="H286" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I286" s="39"/>
-      <c r="J286" s="40"/>
+      <c r="C286" s="39">
+        <v>636.79</v>
+      </c>
+      <c r="D286" s="40">
+        <v>0</v>
+      </c>
+      <c r="E286" s="42"/>
+      <c r="F286" s="39">
+        <v>419.14</v>
+      </c>
+      <c r="G286" s="40">
+        <v>921.04</v>
+      </c>
+      <c r="H286" s="42"/>
+      <c r="I286" s="39">
+        <v>498.42</v>
+      </c>
+      <c r="J286" s="40">
+        <v>400.18000000000006</v>
+      </c>
       <c r="K286" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L286" s="157"/>
-      <c r="M286" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L286" s="157">
+        <v>7822.9199999999992</v>
+      </c>
+      <c r="M286" s="41"/>
       <c r="O286" s="29"/>
       <c r="P286" s="5"/>
       <c r="R286" s="5"/>
@@ -58600,6 +58668,8 @@
     <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.5703125" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -58689,11 +58759,11 @@
         <v>38572.915000000001</v>
       </c>
       <c r="N2" s="72">
-        <v>9061.92</v>
+        <v>9480.9599999999991</v>
       </c>
       <c r="O2" s="29">
         <f>M2-N2</f>
-        <v>29510.995000000003</v>
+        <v>29091.955000000002</v>
       </c>
       <c r="P2" s="29"/>
       <c r="S2">
@@ -58745,18 +58815,21 @@
         <v>509033</v>
       </c>
       <c r="M3" s="72">
-        <v>292226</v>
+        <v>305602</v>
       </c>
       <c r="N3" s="72">
-        <v>178376</v>
+        <v>180194</v>
       </c>
       <c r="O3" s="29">
         <f t="shared" ref="O3:O15" si="0">M3-N3</f>
-        <v>113850</v>
+        <v>125408</v>
       </c>
       <c r="P3" s="29"/>
+      <c r="Q3" s="211" t="s">
+        <v>396</v>
+      </c>
       <c r="R3">
-        <v>6293</v>
+        <v>6584</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -58801,23 +58874,30 @@
       </c>
       <c r="N4" s="72">
         <f>M3*4</f>
-        <v>1168904</v>
+        <v>1222408</v>
       </c>
       <c r="O4" s="29">
         <f t="shared" si="0"/>
-        <v>118954</v>
+        <v>65450</v>
       </c>
       <c r="P4" s="29"/>
-      <c r="R4">
+      <c r="Q4" s="211" t="s">
+        <v>397</v>
+      </c>
+      <c r="R4" s="194">
+        <f>W4</f>
+        <v>9480.9599999999991</v>
+      </c>
+      <c r="T4">
         <v>9659</v>
       </c>
       <c r="V4" s="193">
         <f>U2*R3</f>
-        <v>9061920</v>
+        <v>9480960</v>
       </c>
       <c r="W4" s="194">
         <f>V4/1000</f>
-        <v>9061.92</v>
+        <v>9480.9599999999991</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -58869,7 +58949,7 @@
       </c>
       <c r="P5" s="29"/>
       <c r="V5" s="193">
-        <f>U2*R4</f>
+        <f>U2*T4</f>
         <v>13908960</v>
       </c>
     </row>
@@ -59350,14 +59430,14 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <v>324336.21000000002</v>
+        <v>373978.08</v>
       </c>
       <c r="N15" s="72">
-        <v>309493.43</v>
+        <v>372154.01</v>
       </c>
       <c r="O15" s="29">
         <f t="shared" si="0"/>
-        <v>14842.780000000028</v>
+        <v>1824.070000000007</v>
       </c>
       <c r="P15" s="29"/>
     </row>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-10-15T09:06:28.249-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="705" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CA3825A-27A6-4FBC-8C10-9D42E986BEAC}"/>
+  <xr:revisionPtr revIDLastSave="717" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384F435E-F3A3-4F14-8920-EA7F9CAC9DB8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1670,6 +1670,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="24">
@@ -3142,6 +3143,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3174,7 +3176,6 @@
     <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4163,56 +4164,56 @@
   <sheetData>
     <row r="1" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:18" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="195" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="196"/>
-      <c r="D2" s="196"/>
-      <c r="E2" s="196"/>
-      <c r="F2" s="196"/>
-      <c r="G2" s="196"/>
+      <c r="B2" s="196" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="197"/>
+      <c r="D2" s="197"/>
+      <c r="E2" s="197"/>
+      <c r="F2" s="197"/>
+      <c r="G2" s="197"/>
     </row>
     <row r="3" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="197" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="198"/>
-      <c r="D3" s="198"/>
-      <c r="E3" s="198"/>
-      <c r="F3" s="198"/>
-      <c r="G3" s="199"/>
+      <c r="B3" s="198" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="199"/>
+      <c r="D3" s="199"/>
+      <c r="E3" s="199"/>
+      <c r="F3" s="199"/>
+      <c r="G3" s="200"/>
     </row>
     <row r="4" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="200"/>
-      <c r="C4" s="196"/>
-      <c r="D4" s="196"/>
-      <c r="E4" s="196"/>
-      <c r="F4" s="196"/>
-      <c r="G4" s="201"/>
+      <c r="B4" s="201"/>
+      <c r="C4" s="197"/>
+      <c r="D4" s="197"/>
+      <c r="E4" s="197"/>
+      <c r="F4" s="197"/>
+      <c r="G4" s="202"/>
     </row>
     <row r="5" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="200"/>
-      <c r="C5" s="196"/>
-      <c r="D5" s="196"/>
-      <c r="E5" s="196"/>
-      <c r="F5" s="196"/>
-      <c r="G5" s="201"/>
+      <c r="B5" s="201"/>
+      <c r="C5" s="197"/>
+      <c r="D5" s="197"/>
+      <c r="E5" s="197"/>
+      <c r="F5" s="197"/>
+      <c r="G5" s="202"/>
     </row>
     <row r="6" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="200"/>
-      <c r="C6" s="196"/>
-      <c r="D6" s="196"/>
-      <c r="E6" s="196"/>
-      <c r="F6" s="196"/>
-      <c r="G6" s="201"/>
+      <c r="B6" s="201"/>
+      <c r="C6" s="197"/>
+      <c r="D6" s="197"/>
+      <c r="E6" s="197"/>
+      <c r="F6" s="197"/>
+      <c r="G6" s="202"/>
     </row>
     <row r="7" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="202"/>
-      <c r="C7" s="203"/>
-      <c r="D7" s="203"/>
-      <c r="E7" s="203"/>
-      <c r="F7" s="203"/>
-      <c r="G7" s="204"/>
+      <c r="B7" s="203"/>
+      <c r="C7" s="204"/>
+      <c r="D7" s="204"/>
+      <c r="E7" s="204"/>
+      <c r="F7" s="204"/>
+      <c r="G7" s="205"/>
     </row>
     <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4225,7 +4226,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="80">
-        <v>46305</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="12" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4343,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="79">
-        <v>107500</v>
+        <v>108140</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79"/>
@@ -4393,7 +4394,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="79">
-        <v>97720</v>
+        <v>99130</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79"/>
@@ -4454,7 +4455,7 @@
         <v>93700</v>
       </c>
       <c r="P18" s="79">
-        <v>96800</v>
+        <v>98220</v>
       </c>
       <c r="Q18" s="78"/>
       <c r="R18" s="79"/>
@@ -4469,8 +4470,12 @@
       <c r="D19" s="79">
         <v>54250</v>
       </c>
-      <c r="E19" s="78"/>
-      <c r="F19" s="79"/>
+      <c r="E19" s="78">
+        <v>57320</v>
+      </c>
+      <c r="F19" s="79">
+        <v>59880</v>
+      </c>
       <c r="G19" s="78"/>
       <c r="H19" s="79"/>
       <c r="I19" s="78"/>
@@ -4642,7 +4647,7 @@
         <v>41500</v>
       </c>
       <c r="N23" s="79">
-        <v>47010</v>
+        <v>47800</v>
       </c>
       <c r="O23" s="78">
         <v>48000</v>
@@ -6004,7 +6009,7 @@
         <v>0.22812501887508221</v>
       </c>
       <c r="L15" s="62">
-        <f t="shared" ref="K15:X15" si="3">L14+K15</f>
+        <f t="shared" ref="L15:X15" si="3">L14+K15</f>
         <v>0.29977379730928067</v>
       </c>
       <c r="M15" s="62">
@@ -12726,7 +12731,7 @@
       <c r="O34" s="15"/>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A35" s="205" t="s">
+      <c r="A35" s="206" t="s">
         <v>97</v>
       </c>
       <c r="B35" s="89">
@@ -12892,7 +12897,7 @@
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A36" s="206"/>
+      <c r="A36" s="207"/>
       <c r="B36" s="96" t="s">
         <v>63</v>
       </c>
@@ -20330,7 +20335,7 @@
       <c r="O80" s="15"/>
     </row>
     <row r="81" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A81" s="205" t="s">
+      <c r="A81" s="206" t="s">
         <v>140</v>
       </c>
       <c r="B81" s="89">
@@ -20496,7 +20501,7 @@
       </c>
     </row>
     <row r="82" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A82" s="207"/>
+      <c r="A82" s="208"/>
       <c r="B82" s="96" t="s">
         <v>63</v>
       </c>
@@ -22146,7 +22151,7 @@
       <c r="O91" s="15"/>
     </row>
     <row r="92" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A92" s="205" t="s">
+      <c r="A92" s="206" t="s">
         <v>145</v>
       </c>
       <c r="B92" s="89">
@@ -22312,7 +22317,7 @@
       </c>
     </row>
     <row r="93" spans="1:70" x14ac:dyDescent="0.25">
-      <c r="A93" s="206"/>
+      <c r="A93" s="207"/>
       <c r="B93" s="96" t="s">
         <v>63</v>
       </c>
@@ -58756,14 +58761,14 @@
         <v>37087.89</v>
       </c>
       <c r="M2" s="72">
-        <v>38572.915000000001</v>
+        <v>21970.61</v>
       </c>
       <c r="N2" s="72">
         <v>9480.9599999999991</v>
       </c>
       <c r="O2" s="29">
         <f>M2-N2</f>
-        <v>29091.955000000002</v>
+        <v>12489.650000000001</v>
       </c>
       <c r="P2" s="29"/>
       <c r="S2">
@@ -58825,7 +58830,7 @@
         <v>125408</v>
       </c>
       <c r="P3" s="29"/>
-      <c r="Q3" s="211" t="s">
+      <c r="Q3" s="195" t="s">
         <v>396</v>
       </c>
       <c r="R3">
@@ -58881,7 +58886,7 @@
         <v>65450</v>
       </c>
       <c r="P4" s="29"/>
-      <c r="Q4" s="211" t="s">
+      <c r="Q4" s="195" t="s">
         <v>397</v>
       </c>
       <c r="R4" s="194">
@@ -59465,25 +59470,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="208" t="s">
+      <c r="A1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="B1" s="208" t="s">
+      <c r="B1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="C1" s="208" t="s">
+      <c r="C1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="D1" s="208" t="s">
+      <c r="D1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="208" t="s">
+      <c r="E1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="F1" s="208" t="s">
+      <c r="F1" s="209" t="s">
         <v>251</v>
       </c>
-      <c r="G1" s="208" t="s">
+      <c r="G1" s="209" t="s">
         <v>251</v>
       </c>
     </row>
@@ -60018,43 +60023,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="209" t="s">
+      <c r="A1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="B1" s="209" t="s">
+      <c r="B1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="C1" s="209" t="s">
+      <c r="C1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="D1" s="209" t="s">
+      <c r="D1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="E1" s="209" t="s">
+      <c r="E1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="F1" s="209" t="s">
+      <c r="F1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="G1" s="209" t="s">
+      <c r="G1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="H1" s="209" t="s">
+      <c r="H1" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="J1" s="210" t="s">
+      <c r="J1" s="211" t="s">
         <v>320</v>
       </c>
-      <c r="K1" s="210" t="s">
+      <c r="K1" s="211" t="s">
         <v>320</v>
       </c>
-      <c r="L1" s="210" t="s">
+      <c r="L1" s="211" t="s">
         <v>320</v>
       </c>
-      <c r="M1" s="210" t="s">
+      <c r="M1" s="211" t="s">
         <v>320</v>
       </c>
-      <c r="N1" s="210" t="s">
+      <c r="N1" s="211" t="s">
         <v>320</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-10-20T10:18:48.622-03:00
Responsável: MARCO AURÉLIO GOMES ABREU
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/0. Superestrutura/0. Premissas de Planejamento/00 - Controles de Obra/04 - Unifilar Superestrutura/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="717" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{384F435E-F3A3-4F14-8920-EA7F9CAC9DB8}"/>
+  <xr:revisionPtr revIDLastSave="821" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6042F85-CE8A-4D3D-9D98-C4A3EBED436B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1093" uniqueCount="398">
   <si>
     <t>ACOMPANHAMENTO SUPERESTRUTURA — FOLHA DE ENTRADA</t>
   </si>
@@ -4151,7 +4151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:R61"/>
+  <dimension ref="B1:V61"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -4160,10 +4160,12 @@
     <col min="6" max="6" width="22.42578125" style="4" customWidth="1"/>
     <col min="7" max="12" width="22.42578125" customWidth="1"/>
     <col min="13" max="19" width="22.140625" customWidth="1"/>
+    <col min="20" max="20" width="19.85546875" customWidth="1"/>
+    <col min="21" max="22" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:18" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:22" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:22" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="196" t="s">
         <v>0</v>
       </c>
@@ -4173,7 +4175,7 @@
       <c r="F2" s="197"/>
       <c r="G2" s="197"/>
     </row>
-    <row r="3" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="198" t="s">
         <v>1</v>
       </c>
@@ -4183,7 +4185,7 @@
       <c r="F3" s="199"/>
       <c r="G3" s="200"/>
     </row>
-    <row r="4" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="201"/>
       <c r="C4" s="197"/>
       <c r="D4" s="197"/>
@@ -4191,7 +4193,7 @@
       <c r="F4" s="197"/>
       <c r="G4" s="202"/>
     </row>
-    <row r="5" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="201"/>
       <c r="C5" s="197"/>
       <c r="D5" s="197"/>
@@ -4199,7 +4201,7 @@
       <c r="F5" s="197"/>
       <c r="G5" s="202"/>
     </row>
-    <row r="6" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="201"/>
       <c r="C6" s="197"/>
       <c r="D6" s="197"/>
@@ -4207,7 +4209,7 @@
       <c r="F6" s="197"/>
       <c r="G6" s="202"/>
     </row>
-    <row r="7" spans="2:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="203"/>
       <c r="C7" s="204"/>
       <c r="D7" s="204"/>
@@ -4215,26 +4217,26 @@
       <c r="F7" s="204"/>
       <c r="G7" s="205"/>
     </row>
-    <row r="8" spans="2:18" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="80">
-        <v>46308</v>
-      </c>
-    </row>
-    <row r="12" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>46312</v>
+      </c>
+    </row>
+    <row r="12" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="73" t="s">
         <v>5</v>
       </c>
@@ -4286,8 +4288,20 @@
       <c r="R13" s="75" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S13" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="T13" s="75" t="s">
+        <v>7</v>
+      </c>
+      <c r="U13" s="76" t="s">
+        <v>6</v>
+      </c>
+      <c r="V13" s="75" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="77" t="s">
         <v>8</v>
       </c>
@@ -4335,8 +4349,12 @@
       </c>
       <c r="Q14" s="78"/>
       <c r="R14" s="79"/>
-    </row>
-    <row r="15" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S14" s="78"/>
+      <c r="T14" s="79"/>
+      <c r="U14" s="78"/>
+      <c r="V14" s="79"/>
+    </row>
+    <row r="15" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="77" t="s">
         <v>9</v>
       </c>
@@ -4344,7 +4362,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="79">
-        <v>108140</v>
+        <v>110800</v>
       </c>
       <c r="E15" s="78"/>
       <c r="F15" s="79"/>
@@ -4360,8 +4378,12 @@
       <c r="P15" s="79"/>
       <c r="Q15" s="78"/>
       <c r="R15" s="79"/>
-    </row>
-    <row r="16" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S15" s="78"/>
+      <c r="T15" s="79"/>
+      <c r="U15" s="78"/>
+      <c r="V15" s="79"/>
+    </row>
+    <row r="16" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="77" t="s">
         <v>10</v>
       </c>
@@ -4385,8 +4407,12 @@
       <c r="P16" s="79"/>
       <c r="Q16" s="78"/>
       <c r="R16" s="79"/>
-    </row>
-    <row r="17" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S16" s="78"/>
+      <c r="T16" s="79"/>
+      <c r="U16" s="78"/>
+      <c r="V16" s="79"/>
+    </row>
+    <row r="17" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="77" t="s">
         <v>11</v>
       </c>
@@ -4394,7 +4420,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="79">
-        <v>99130</v>
+        <v>100960</v>
       </c>
       <c r="E17" s="78"/>
       <c r="F17" s="79"/>
@@ -4410,8 +4436,12 @@
       <c r="P17" s="79"/>
       <c r="Q17" s="78"/>
       <c r="R17" s="79"/>
-    </row>
-    <row r="18" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S17" s="78"/>
+      <c r="T17" s="79"/>
+      <c r="U17" s="78"/>
+      <c r="V17" s="79"/>
+    </row>
+    <row r="18" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="77" t="s">
         <v>12</v>
       </c>
@@ -4455,12 +4485,16 @@
         <v>93700</v>
       </c>
       <c r="P18" s="79">
-        <v>98220</v>
+        <v>100900</v>
       </c>
       <c r="Q18" s="78"/>
       <c r="R18" s="79"/>
-    </row>
-    <row r="19" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S18" s="78"/>
+      <c r="T18" s="79"/>
+      <c r="U18" s="78"/>
+      <c r="V18" s="79"/>
+    </row>
+    <row r="19" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="77" t="s">
         <v>13</v>
       </c>
@@ -4476,8 +4510,12 @@
       <c r="F19" s="79">
         <v>59880</v>
       </c>
-      <c r="G19" s="78"/>
-      <c r="H19" s="79"/>
+      <c r="G19" s="78">
+        <v>61900</v>
+      </c>
+      <c r="H19" s="79">
+        <v>66270</v>
+      </c>
       <c r="I19" s="78"/>
       <c r="J19" s="79"/>
       <c r="K19" s="78"/>
@@ -4488,8 +4526,12 @@
       <c r="P19" s="79"/>
       <c r="Q19" s="78"/>
       <c r="R19" s="79"/>
-    </row>
-    <row r="20" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S19" s="78"/>
+      <c r="T19" s="79"/>
+      <c r="U19" s="78"/>
+      <c r="V19" s="79"/>
+    </row>
+    <row r="20" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="77" t="s">
         <v>14</v>
       </c>
@@ -4523,14 +4565,22 @@
       <c r="L20" s="79">
         <v>77400</v>
       </c>
-      <c r="M20" s="78"/>
-      <c r="N20" s="79"/>
+      <c r="M20" s="78">
+        <v>57660</v>
+      </c>
+      <c r="N20" s="79">
+        <v>58440</v>
+      </c>
       <c r="O20" s="78"/>
       <c r="P20" s="79"/>
       <c r="Q20" s="78"/>
       <c r="R20" s="79"/>
-    </row>
-    <row r="21" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S20" s="78"/>
+      <c r="T20" s="79"/>
+      <c r="U20" s="78"/>
+      <c r="V20" s="79"/>
+    </row>
+    <row r="21" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="77" t="s">
         <v>15</v>
       </c>
@@ -4571,7 +4621,7 @@
         <v>50000</v>
       </c>
       <c r="O21" s="78">
-        <v>61300</v>
+        <v>60000</v>
       </c>
       <c r="P21" s="79">
         <v>61700</v>
@@ -4580,10 +4630,22 @@
         <v>50040</v>
       </c>
       <c r="R21" s="79">
-        <v>54700</v>
-      </c>
-    </row>
-    <row r="22" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>57660</v>
+      </c>
+      <c r="S21" s="78">
+        <v>58560</v>
+      </c>
+      <c r="T21" s="79">
+        <v>59860</v>
+      </c>
+      <c r="U21" s="78">
+        <v>61950</v>
+      </c>
+      <c r="V21" s="79">
+        <v>62200</v>
+      </c>
+    </row>
+    <row r="22" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="77" t="s">
         <v>16</v>
       </c>
@@ -4607,8 +4669,12 @@
       <c r="P22" s="79"/>
       <c r="Q22" s="78"/>
       <c r="R22" s="79"/>
-    </row>
-    <row r="23" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S22" s="78"/>
+      <c r="T22" s="79"/>
+      <c r="U22" s="78"/>
+      <c r="V22" s="79"/>
+    </row>
+    <row r="23" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="77" t="s">
         <v>17</v>
       </c>
@@ -4641,24 +4707,28 @@
         <v>40100</v>
       </c>
       <c r="L23" s="79">
-        <v>41500</v>
+        <v>50260</v>
       </c>
       <c r="M23" s="78">
-        <v>41500</v>
+        <v>50540</v>
       </c>
       <c r="N23" s="79">
-        <v>47800</v>
+        <v>52260</v>
       </c>
       <c r="O23" s="78">
-        <v>48000</v>
+        <v>60000</v>
       </c>
       <c r="P23" s="79">
-        <v>50240</v>
+        <v>61340</v>
       </c>
       <c r="Q23" s="78"/>
       <c r="R23" s="79"/>
-    </row>
-    <row r="24" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S23" s="78"/>
+      <c r="T23" s="79"/>
+      <c r="U23" s="78"/>
+      <c r="V23" s="79"/>
+    </row>
+    <row r="24" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="77" t="s">
         <v>18</v>
       </c>
@@ -4686,8 +4756,12 @@
       <c r="P24" s="79"/>
       <c r="Q24" s="78"/>
       <c r="R24" s="79"/>
-    </row>
-    <row r="25" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S24" s="78"/>
+      <c r="T24" s="79"/>
+      <c r="U24" s="78"/>
+      <c r="V24" s="79"/>
+    </row>
+    <row r="25" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="77" t="s">
         <v>19</v>
       </c>
@@ -4727,8 +4801,12 @@
       <c r="P25" s="79"/>
       <c r="Q25" s="78"/>
       <c r="R25" s="79"/>
-    </row>
-    <row r="26" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S25" s="78"/>
+      <c r="T25" s="79"/>
+      <c r="U25" s="78"/>
+      <c r="V25" s="79"/>
+    </row>
+    <row r="26" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="77" t="s">
         <v>20</v>
       </c>
@@ -4756,8 +4834,12 @@
       <c r="P26" s="79"/>
       <c r="Q26" s="78"/>
       <c r="R26" s="79"/>
-    </row>
-    <row r="27" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S26" s="78"/>
+      <c r="T26" s="79"/>
+      <c r="U26" s="78"/>
+      <c r="V26" s="79"/>
+    </row>
+    <row r="27" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="77" t="s">
         <v>21</v>
       </c>
@@ -4777,7 +4859,7 @@
         <v>23020</v>
       </c>
       <c r="H27" s="79">
-        <v>44878</v>
+        <v>47754</v>
       </c>
       <c r="I27" s="78"/>
       <c r="J27" s="79"/>
@@ -4789,13 +4871,17 @@
       <c r="P27" s="79"/>
       <c r="Q27" s="78"/>
       <c r="R27" s="79"/>
-    </row>
-    <row r="29" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S27" s="78"/>
+      <c r="T27" s="79"/>
+      <c r="U27" s="78"/>
+      <c r="V27" s="79"/>
+    </row>
+    <row r="29" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
         <v>23</v>
       </c>
@@ -4803,12 +4889,12 @@
         <v>131260</v>
       </c>
     </row>
-    <row r="31" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="191" t="s">
         <v>25</v>
       </c>
@@ -5471,51 +5557,51 @@
       </c>
       <c r="M5" s="62">
         <f t="shared" ref="M5:X5" si="1">M6-L6</f>
-        <v>7.7407601135277837E-2</v>
+        <v>8.0760796683505109E-2</v>
       </c>
       <c r="N5" s="62">
         <f t="shared" si="1"/>
-        <v>5.9545501372358367E-2</v>
+        <v>5.7544614609517597E-2</v>
       </c>
       <c r="O5" s="62">
         <f t="shared" si="1"/>
-        <v>5.6504819574451248E-2</v>
+        <v>5.7556545481491084E-2</v>
       </c>
       <c r="P5" s="62">
         <f t="shared" si="1"/>
-        <v>5.5049969779112196E-2</v>
+        <v>5.5648513874657857E-2</v>
       </c>
       <c r="Q5" s="62">
         <f t="shared" si="1"/>
-        <v>6.6879599404793266E-2</v>
+        <v>6.5950744922580129E-2</v>
       </c>
       <c r="R5" s="62">
         <f t="shared" si="1"/>
-        <v>6.4967958440981466E-2</v>
+        <v>6.4162942140209567E-2</v>
       </c>
       <c r="S5" s="62">
         <f t="shared" si="1"/>
-        <v>6.6572851489322904E-2</v>
+        <v>6.6605864908650725E-2</v>
       </c>
       <c r="T5" s="62">
         <f t="shared" si="1"/>
-        <v>7.5225278014127261E-2</v>
+        <v>7.5634717087211367E-2</v>
       </c>
       <c r="U5" s="62">
         <f t="shared" si="1"/>
-        <v>6.2034254747460493E-2</v>
+        <v>6.3685692355299861E-2</v>
       </c>
       <c r="V5" s="62">
         <f t="shared" si="1"/>
-        <v>5.7645965412102207E-2</v>
+        <v>5.797165093240042E-2</v>
       </c>
       <c r="W5" s="62">
         <f t="shared" si="1"/>
-        <v>6.0092428488860095E-2</v>
+        <v>5.8422499538519745E-2</v>
       </c>
       <c r="X5" s="62">
         <f t="shared" si="1"/>
-        <v>5.2865026797076498E-3</v>
+        <v>4.8980331980249536E-3</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -5533,43 +5619,43 @@
       <c r="J6" s="61"/>
       <c r="K6" s="61"/>
       <c r="L6" s="62">
-        <v>0.29262742340425391</v>
+        <v>0.29115738426793158</v>
       </c>
       <c r="M6" s="62">
-        <v>0.37003502453953174</v>
+        <v>0.37191818095143669</v>
       </c>
       <c r="N6" s="62">
-        <v>0.42958052591189011</v>
+        <v>0.42946279556095429</v>
       </c>
       <c r="O6" s="62">
-        <v>0.48608534548634136</v>
+        <v>0.48701934104244538</v>
       </c>
       <c r="P6" s="62">
-        <v>0.54113531526545355</v>
+        <v>0.54266785491710323</v>
       </c>
       <c r="Q6" s="62">
-        <v>0.60801491467024682</v>
+        <v>0.60861859983968336</v>
       </c>
       <c r="R6" s="62">
-        <v>0.67298287311122829</v>
+        <v>0.67278154197989293</v>
       </c>
       <c r="S6" s="62">
-        <v>0.73955572460055119</v>
+        <v>0.73938740688854365</v>
       </c>
       <c r="T6" s="62">
-        <v>0.81478100261467845</v>
+        <v>0.81502212397575502</v>
       </c>
       <c r="U6" s="62">
-        <v>0.87681525736213894</v>
+        <v>0.87870781633105488</v>
       </c>
       <c r="V6" s="62">
-        <v>0.93446122277424115</v>
+        <v>0.9366794672634553</v>
       </c>
       <c r="W6" s="62">
-        <v>0.99455365126310125</v>
+        <v>0.99510196680197505</v>
       </c>
       <c r="X6" s="62">
-        <v>0.9998401539428089</v>
+        <v>1</v>
       </c>
       <c r="Y6" s="83">
         <v>1</v>
@@ -5610,7 +5696,7 @@
         <v>4.7600000000000003E-2</v>
       </c>
       <c r="L7" s="62">
-        <v>1.3400000000000023E-2</v>
+        <v>2.2900000000000004E-2</v>
       </c>
       <c r="M7" s="62"/>
       <c r="N7" s="62"/>
@@ -5671,7 +5757,7 @@
       </c>
       <c r="L8" s="62">
         <f t="shared" si="2"/>
-        <v>0.24610000000000001</v>
+        <v>0.25559999999999999</v>
       </c>
       <c r="M8" s="62"/>
       <c r="N8" s="62"/>
@@ -6384,6 +6470,7 @@
         <v>229</v>
       </c>
       <c r="L22" s="86">
+        <f>HISTOGRAMA!W33</f>
         <v>227</v>
       </c>
       <c r="M22" s="62"/>
@@ -6618,6 +6705,7 @@
         <v>115</v>
       </c>
       <c r="L27" s="86">
+        <f>HISTOGRAMA!W79</f>
         <v>118</v>
       </c>
       <c r="M27" s="62"/>
@@ -6852,6 +6940,7 @@
         <v>49</v>
       </c>
       <c r="L32" s="86">
+        <f>HISTOGRAMA!W116</f>
         <v>46</v>
       </c>
       <c r="M32" s="62"/>
@@ -7086,6 +7175,7 @@
         <v>46</v>
       </c>
       <c r="L37" s="87">
+        <f>HISTOGRAMA!W90</f>
         <v>49</v>
       </c>
       <c r="M37" s="62"/>
@@ -8052,7 +8142,7 @@
         <v>3</v>
       </c>
       <c r="W6" s="103">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X6" s="102">
         <v>2</v>
@@ -9040,7 +9130,7 @@
         <v>3</v>
       </c>
       <c r="W12" s="103">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X12" s="102">
         <v>3</v>
@@ -9866,7 +9956,7 @@
         <v>23</v>
       </c>
       <c r="W17" s="13">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="X17" s="12">
         <v>23</v>
@@ -10198,7 +10288,7 @@
         <v>22</v>
       </c>
       <c r="W19" s="13">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X19" s="12">
         <v>22</v>
@@ -14654,7 +14744,7 @@
         <v>6</v>
       </c>
       <c r="W46" s="103">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X46" s="102">
         <v>5</v>
@@ -19622,7 +19712,7 @@
         <v>6</v>
       </c>
       <c r="W76" s="103">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X76" s="102">
         <v>6</v>
@@ -27510,7 +27600,7 @@
         <v>1265</v>
       </c>
       <c r="J5" s="68">
-        <v>345</v>
+        <v>429</v>
       </c>
       <c r="K5" s="68"/>
       <c r="L5" s="68"/>
@@ -27569,7 +27659,7 @@
         <v>23</v>
       </c>
       <c r="J6" s="69">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K6" s="69"/>
       <c r="L6" s="69"/>
@@ -27622,7 +27712,7 @@
       </c>
       <c r="J7" s="69">
         <f t="shared" si="2"/>
-        <v>43.125</v>
+        <v>39</v>
       </c>
       <c r="K7" s="69"/>
       <c r="L7" s="69"/>
@@ -27688,34 +27778,34 @@
         <v>1352.8999999999996</v>
       </c>
       <c r="J8" s="147">
-        <v>1281.3999999999996</v>
+        <v>1106.8000000000002</v>
       </c>
       <c r="K8" s="147">
-        <v>1270.8000000000002</v>
+        <v>1287.6999999999998</v>
       </c>
       <c r="L8" s="147">
-        <v>936.40000000000055</v>
+        <v>948.89999999999964</v>
       </c>
       <c r="M8" s="147">
-        <v>1270.7999999999993</v>
+        <v>1287.7000000000007</v>
       </c>
       <c r="N8" s="147">
-        <v>1337.7000000000007</v>
+        <v>1355.5</v>
       </c>
       <c r="O8" s="147">
-        <v>1538.3999999999996</v>
+        <v>1558.7999999999993</v>
       </c>
       <c r="P8" s="147">
-        <v>1471.5</v>
+        <v>1491.1000000000004</v>
       </c>
       <c r="Q8" s="147">
-        <v>1404.6000000000004</v>
+        <v>1423.2999999999993</v>
       </c>
       <c r="R8" s="147">
-        <v>1471.4999999999982</v>
+        <v>1491.0999999999985</v>
       </c>
       <c r="S8" s="147">
-        <v>1034</v>
+        <v>1066.2999999999993</v>
       </c>
       <c r="T8" s="147">
         <v>0</v>
@@ -27862,43 +27952,43 @@
       </c>
       <c r="J10" s="69">
         <f t="shared" si="5"/>
-        <v>47.459259259259248</v>
+        <v>40.992592592592601</v>
       </c>
       <c r="K10" s="69">
         <f t="shared" si="5"/>
-        <v>50.832000000000008</v>
+        <v>51.507999999999996</v>
       </c>
       <c r="L10" s="69">
         <f t="shared" si="5"/>
-        <v>58.525000000000034</v>
+        <v>59.306249999999977</v>
       </c>
       <c r="M10" s="69">
         <f t="shared" si="5"/>
-        <v>52.949999999999967</v>
+        <v>53.654166666666697</v>
       </c>
       <c r="N10" s="69">
         <f t="shared" si="5"/>
-        <v>55.737500000000033</v>
+        <v>56.479166666666664</v>
       </c>
       <c r="O10" s="69">
         <f t="shared" si="5"/>
-        <v>56.977777777777767</v>
+        <v>57.733333333333306</v>
       </c>
       <c r="P10" s="69">
         <f t="shared" si="5"/>
-        <v>56.596153846153847</v>
+        <v>57.350000000000016</v>
       </c>
       <c r="Q10" s="69">
         <f t="shared" si="5"/>
-        <v>54.023076923076935</v>
+        <v>54.742307692307662</v>
       </c>
       <c r="R10" s="69">
         <f t="shared" si="5"/>
-        <v>56.596153846153776</v>
+        <v>57.349999999999945</v>
       </c>
       <c r="S10" s="69">
         <f t="shared" si="5"/>
-        <v>38.296296296296298</v>
+        <v>39.492592592592565</v>
       </c>
       <c r="T10" s="69">
         <f t="shared" si="5"/>
@@ -28282,7 +28372,7 @@
         <v>13615</v>
       </c>
       <c r="J16" s="153">
-        <v>2200</v>
+        <v>5500</v>
       </c>
       <c r="K16" s="153"/>
       <c r="L16" s="153"/>
@@ -28327,7 +28417,7 @@
         <v>17</v>
       </c>
       <c r="J17" s="69">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K17" s="69"/>
       <c r="L17" s="69"/>
@@ -28380,7 +28470,7 @@
       </c>
       <c r="J18" s="69">
         <f t="shared" si="7"/>
-        <v>550</v>
+        <v>687.5</v>
       </c>
       <c r="K18" s="69"/>
       <c r="L18" s="69"/>
@@ -28430,37 +28520,37 @@
         <v>13615</v>
       </c>
       <c r="J19" s="147">
-        <v>17270.899999999994</v>
+        <v>17883.300000000003</v>
       </c>
       <c r="K19" s="147">
-        <v>18600.5</v>
+        <v>18572.599999999991</v>
       </c>
       <c r="L19" s="147">
-        <v>12540.5</v>
+        <v>12565.700000000012</v>
       </c>
       <c r="M19" s="147">
-        <v>17578.5</v>
+        <v>17592.700000000012</v>
       </c>
       <c r="N19" s="147">
-        <v>18649.200000000012</v>
+        <v>18645.5</v>
       </c>
       <c r="O19" s="147">
         <v>21409.799999999988</v>
       </c>
       <c r="P19" s="147">
-        <v>20501.299999999988</v>
+        <v>20502.5</v>
       </c>
       <c r="Q19" s="147">
-        <v>19767.299999999988</v>
+        <v>19778.399999999994</v>
       </c>
       <c r="R19" s="147">
-        <v>20571.399999999994</v>
+        <v>20559.400000000023</v>
       </c>
       <c r="S19" s="147">
         <v>20484.799999999988</v>
       </c>
       <c r="T19" s="147">
-        <v>18250.299999999988</v>
+        <v>17629.79999999993</v>
       </c>
       <c r="U19" s="147">
         <v>0</v>
@@ -28583,23 +28673,23 @@
       </c>
       <c r="J21" s="69">
         <f t="shared" si="10"/>
-        <v>639.66296296296275</v>
+        <v>662.34444444444455</v>
       </c>
       <c r="K21" s="69">
         <f t="shared" si="10"/>
-        <v>744.02</v>
+        <v>742.90399999999966</v>
       </c>
       <c r="L21" s="69">
         <f t="shared" si="10"/>
-        <v>783.78125</v>
+        <v>785.35625000000073</v>
       </c>
       <c r="M21" s="69">
         <f t="shared" si="10"/>
-        <v>732.4375</v>
+        <v>733.02916666666715</v>
       </c>
       <c r="N21" s="69">
         <f t="shared" si="10"/>
-        <v>777.05000000000052</v>
+        <v>776.89583333333337</v>
       </c>
       <c r="O21" s="69">
         <f t="shared" si="10"/>
@@ -28607,15 +28697,15 @@
       </c>
       <c r="P21" s="69">
         <f t="shared" si="10"/>
-        <v>788.51153846153807</v>
+        <v>788.55769230769226</v>
       </c>
       <c r="Q21" s="69">
         <f t="shared" si="10"/>
-        <v>760.28076923076878</v>
+        <v>760.70769230769213</v>
       </c>
       <c r="R21" s="69">
         <f t="shared" si="10"/>
-        <v>791.20769230769213</v>
+        <v>790.7461538461547</v>
       </c>
       <c r="S21" s="69">
         <f t="shared" si="10"/>
@@ -28623,7 +28713,7 @@
       </c>
       <c r="T21" s="69">
         <f t="shared" si="10"/>
-        <v>701.93461538461497</v>
+        <v>678.06923076922806</v>
       </c>
       <c r="U21" s="69">
         <f t="shared" si="10"/>
@@ -28957,7 +29047,7 @@
         <v>36285</v>
       </c>
       <c r="J27" s="68">
-        <v>23447.999799999991</v>
+        <v>35107</v>
       </c>
       <c r="K27" s="68" t="s">
         <v>196</v>
@@ -29026,7 +29116,7 @@
         <v>13</v>
       </c>
       <c r="J28" s="69">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K28" s="69"/>
       <c r="L28" s="69"/>
@@ -29079,7 +29169,7 @@
       </c>
       <c r="J29" s="69">
         <f t="shared" si="12"/>
-        <v>3349.7142571428558</v>
+        <v>2925.5833333333335</v>
       </c>
       <c r="K29" s="69"/>
       <c r="L29" s="69"/>
@@ -29129,40 +29219,40 @@
         <v>36285</v>
       </c>
       <c r="J30" s="147">
-        <v>52942.099799999996</v>
+        <v>86171.799999999988</v>
       </c>
       <c r="K30" s="147">
-        <v>40066.499999999971</v>
+        <v>47896.799999999988</v>
       </c>
       <c r="L30" s="147">
-        <v>39282.099999999977</v>
+        <v>28221.5</v>
       </c>
       <c r="M30" s="147">
-        <v>37845.799999999988</v>
+        <v>28266.299999999988</v>
       </c>
       <c r="N30" s="147">
-        <v>38516.099999999977</v>
+        <v>31935.299999999988</v>
       </c>
       <c r="O30" s="147">
-        <v>54697.099999999977</v>
+        <v>51662.900000000023</v>
       </c>
       <c r="P30" s="147">
-        <v>42693.400000000023</v>
+        <v>37808.400000000023</v>
       </c>
       <c r="Q30" s="147">
-        <v>56337.500000000058</v>
+        <v>56204.199999999953</v>
       </c>
       <c r="R30" s="147">
-        <v>50576.800000000047</v>
+        <v>50229.5</v>
       </c>
       <c r="S30" s="147">
-        <v>38266.5</v>
+        <v>33918.199999999953</v>
       </c>
       <c r="T30" s="147">
-        <v>50911.800000000047</v>
+        <v>52176.900000000023</v>
       </c>
       <c r="U30" s="147">
-        <v>56134.200199999847</v>
+        <v>53778.099999999977</v>
       </c>
       <c r="V30" s="147">
         <v>0</v>
@@ -29282,51 +29372,51 @@
       </c>
       <c r="J32" s="69">
         <f t="shared" si="15"/>
-        <v>1960.8185111111109</v>
+        <v>3191.5481481481479</v>
       </c>
       <c r="K32" s="69">
         <f t="shared" si="15"/>
-        <v>1602.6599999999989</v>
+        <v>1915.8719999999996</v>
       </c>
       <c r="L32" s="69">
         <f t="shared" si="15"/>
-        <v>2455.1312499999985</v>
+        <v>1763.84375</v>
       </c>
       <c r="M32" s="69">
         <f t="shared" si="15"/>
-        <v>1576.9083333333328</v>
+        <v>1177.7624999999996</v>
       </c>
       <c r="N32" s="69">
         <f t="shared" si="15"/>
-        <v>1604.837499999999</v>
+        <v>1330.6374999999996</v>
       </c>
       <c r="O32" s="69">
         <f t="shared" si="15"/>
-        <v>2025.8185185185177</v>
+        <v>1913.4407407407416</v>
       </c>
       <c r="P32" s="69">
         <f t="shared" si="15"/>
-        <v>1642.053846153847</v>
+        <v>1454.1692307692317</v>
       </c>
       <c r="Q32" s="69">
         <f t="shared" si="15"/>
-        <v>2166.8269230769251</v>
+        <v>2161.699999999998</v>
       </c>
       <c r="R32" s="69">
         <f t="shared" si="15"/>
-        <v>1945.2615384615403</v>
+        <v>1931.9038461538462</v>
       </c>
       <c r="S32" s="69">
         <f t="shared" si="15"/>
-        <v>1417.2777777777778</v>
+        <v>1256.2296296296279</v>
       </c>
       <c r="T32" s="69">
         <f t="shared" si="15"/>
-        <v>1958.1461538461556</v>
+        <v>2006.803846153847</v>
       </c>
       <c r="U32" s="69">
         <f t="shared" si="15"/>
-        <v>2159.0076999999942</v>
+        <v>2068.3884615384604</v>
       </c>
       <c r="V32" s="69">
         <v>0</v>
@@ -29656,7 +29746,7 @@
         <v>119</v>
       </c>
       <c r="J38" s="68">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="K38" s="68" t="s">
         <v>196</v>
@@ -29725,7 +29815,7 @@
         <v>22</v>
       </c>
       <c r="J39" s="69">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K39" s="69"/>
       <c r="L39" s="69"/>
@@ -29826,43 +29916,43 @@
         <v>132.20000000000005</v>
       </c>
       <c r="J41" s="147">
-        <v>272.5</v>
+        <v>244</v>
       </c>
       <c r="K41" s="147">
-        <v>196.39999999999998</v>
+        <v>192.5</v>
       </c>
       <c r="L41" s="147">
-        <v>186.89999999999998</v>
+        <v>178.09999999999991</v>
       </c>
       <c r="M41" s="147">
-        <v>213.40000000000009</v>
+        <v>219.79999999999995</v>
       </c>
       <c r="N41" s="147">
-        <v>158.20000000000005</v>
+        <v>164.29999999999995</v>
       </c>
       <c r="O41" s="147">
-        <v>227</v>
+        <v>220.59999999999991</v>
       </c>
       <c r="P41" s="147">
-        <v>261.69999999999982</v>
+        <v>263.90000000000009</v>
       </c>
       <c r="Q41" s="147">
-        <v>267.80000000000018</v>
+        <v>268.59999999999991</v>
       </c>
       <c r="R41" s="147">
-        <v>288.09999999999991</v>
+        <v>279.09999999999991</v>
       </c>
       <c r="S41" s="147">
-        <v>276.19999999999982</v>
+        <v>325.30000000000018</v>
       </c>
       <c r="T41" s="147">
-        <v>297.09999999999991</v>
+        <v>297</v>
       </c>
       <c r="U41" s="147">
-        <v>104.40000000000009</v>
+        <v>98.300000000000182</v>
       </c>
       <c r="V41" s="147">
-        <v>5.3000000000001819</v>
+        <v>3.4000000000000909</v>
       </c>
       <c r="X41" s="148"/>
     </row>
@@ -29979,51 +30069,51 @@
       </c>
       <c r="J43" s="69">
         <f t="shared" si="20"/>
-        <v>10.092592592592593</v>
+        <v>9.0370370370370363</v>
       </c>
       <c r="K43" s="69">
         <f t="shared" si="20"/>
-        <v>7.855999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="L43" s="69">
         <f t="shared" si="20"/>
-        <v>11.681249999999999</v>
+        <v>11.131249999999994</v>
       </c>
       <c r="M43" s="69">
         <f t="shared" si="20"/>
-        <v>8.891666666666671</v>
+        <v>9.1583333333333314</v>
       </c>
       <c r="N43" s="69">
         <f t="shared" si="20"/>
-        <v>6.5916666666666686</v>
+        <v>6.8458333333333314</v>
       </c>
       <c r="O43" s="69">
         <f t="shared" si="20"/>
-        <v>8.4074074074074066</v>
+        <v>8.1703703703703674</v>
       </c>
       <c r="P43" s="69">
         <f t="shared" si="20"/>
-        <v>10.065384615384609</v>
+        <v>10.150000000000004</v>
       </c>
       <c r="Q43" s="69">
         <f t="shared" si="20"/>
-        <v>10.300000000000008</v>
+        <v>10.330769230769228</v>
       </c>
       <c r="R43" s="69">
         <f t="shared" si="20"/>
-        <v>11.080769230769228</v>
+        <v>10.734615384615381</v>
       </c>
       <c r="S43" s="69">
         <f t="shared" si="20"/>
-        <v>10.229629629629622</v>
+        <v>12.048148148148154</v>
       </c>
       <c r="T43" s="69">
         <f t="shared" si="20"/>
-        <v>11.426923076923073</v>
+        <v>11.423076923076923</v>
       </c>
       <c r="U43" s="69">
         <f t="shared" si="20"/>
-        <v>4.0153846153846189</v>
+        <v>3.7807692307692378</v>
       </c>
       <c r="V43" s="69">
         <v>0</v>
@@ -30353,7 +30443,7 @@
         <v>18166</v>
       </c>
       <c r="J49" s="68">
-        <v>5228</v>
+        <v>10174</v>
       </c>
       <c r="K49" s="68" t="s">
         <v>196</v>
@@ -30422,7 +30512,7 @@
         <v>17</v>
       </c>
       <c r="J50" s="69">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="K50" s="69"/>
       <c r="L50" s="69"/>
@@ -30475,7 +30565,7 @@
       </c>
       <c r="J51" s="69">
         <f t="shared" si="22"/>
-        <v>580.88888888888891</v>
+        <v>678.26666666666665</v>
       </c>
       <c r="K51" s="69"/>
       <c r="L51" s="69"/>
@@ -30525,40 +30615,40 @@
         <v>19854.100000000006</v>
       </c>
       <c r="J52" s="147">
-        <v>18746.699999999997</v>
+        <v>19345.100000000006</v>
       </c>
       <c r="K52" s="147">
-        <v>31552.5</v>
+        <v>22372.300000000003</v>
       </c>
       <c r="L52" s="147">
-        <v>17193.699999999997</v>
+        <v>16204.100000000006</v>
       </c>
       <c r="M52" s="147">
-        <v>11341.399999999994</v>
+        <v>11686.300000000003</v>
       </c>
       <c r="N52" s="147">
-        <v>13326.5</v>
+        <v>18486.200000000012</v>
       </c>
       <c r="O52" s="147">
-        <v>17954.399999999994</v>
+        <v>17583</v>
       </c>
       <c r="P52" s="147">
-        <v>16952.5</v>
+        <v>21629.399999999994</v>
       </c>
       <c r="Q52" s="147">
-        <v>24331.799999999988</v>
+        <v>24342.700000000012</v>
       </c>
       <c r="R52" s="147">
-        <v>22964</v>
+        <v>23209.700000000012</v>
       </c>
       <c r="S52" s="147">
-        <v>12742.899999999994</v>
+        <v>22639.700000000012</v>
       </c>
       <c r="T52" s="147">
-        <v>20111.599999999977</v>
+        <v>21052.5</v>
       </c>
       <c r="U52" s="147">
-        <v>34435.200000000012</v>
+        <v>23102.199999999895</v>
       </c>
       <c r="V52" s="147"/>
       <c r="X52" s="148"/>
@@ -30676,51 +30766,51 @@
       </c>
       <c r="J54" s="69">
         <f t="shared" si="25"/>
-        <v>694.32222222222208</v>
+        <v>716.4851851851854</v>
       </c>
       <c r="K54" s="69">
         <f t="shared" si="25"/>
-        <v>1262.0999999999999</v>
+        <v>894.89200000000017</v>
       </c>
       <c r="L54" s="69">
         <f t="shared" si="25"/>
-        <v>1074.6062499999998</v>
+        <v>1012.7562500000004</v>
       </c>
       <c r="M54" s="69">
         <f t="shared" si="25"/>
-        <v>472.55833333333311</v>
+        <v>486.92916666666679</v>
       </c>
       <c r="N54" s="69">
         <f t="shared" si="25"/>
-        <v>555.27083333333337</v>
+        <v>770.25833333333378</v>
       </c>
       <c r="O54" s="69">
         <f t="shared" si="25"/>
-        <v>664.97777777777753</v>
+        <v>651.22222222222217</v>
       </c>
       <c r="P54" s="69">
         <f t="shared" si="25"/>
-        <v>652.01923076923072</v>
+        <v>831.89999999999975</v>
       </c>
       <c r="Q54" s="69">
         <f t="shared" si="25"/>
-        <v>935.83846153846105</v>
+        <v>936.25769230769276</v>
       </c>
       <c r="R54" s="69">
         <f t="shared" si="25"/>
-        <v>883.23076923076928</v>
+        <v>892.68076923076967</v>
       </c>
       <c r="S54" s="69">
         <f t="shared" si="25"/>
-        <v>471.95925925925906</v>
+        <v>838.50740740740787</v>
       </c>
       <c r="T54" s="69">
         <f t="shared" si="25"/>
-        <v>773.52307692307602</v>
+        <v>809.71153846153845</v>
       </c>
       <c r="U54" s="69">
         <f t="shared" si="25"/>
-        <v>1324.4307692307698</v>
+        <v>888.54615384614976</v>
       </c>
       <c r="V54" s="69">
         <f t="shared" si="25"/>
@@ -31051,7 +31141,7 @@
         <v>32756</v>
       </c>
       <c r="J60" s="68">
-        <v>11884</v>
+        <v>17635</v>
       </c>
       <c r="K60" s="68" t="s">
         <v>196</v>
@@ -31120,7 +31210,7 @@
         <v>15</v>
       </c>
       <c r="J61" s="69">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K61" s="69"/>
       <c r="L61" s="69"/>
@@ -31172,7 +31262,7 @@
       </c>
       <c r="J62" s="69">
         <f>J60/J61</f>
-        <v>1980.6666666666667</v>
+        <v>1959.4444444444443</v>
       </c>
       <c r="K62" s="69"/>
       <c r="L62" s="69"/>
@@ -31221,43 +31311,43 @@
         <v>35224.199999999997</v>
       </c>
       <c r="J63" s="147">
-        <v>45335.100000000006</v>
+        <v>52250.7</v>
       </c>
       <c r="K63" s="147">
-        <v>50722.600000000006</v>
+        <v>51537.8</v>
       </c>
       <c r="L63" s="147">
-        <v>39424.899999999994</v>
+        <v>40915</v>
       </c>
       <c r="M63" s="147">
-        <v>44912.800000000017</v>
+        <v>40980.600000000006</v>
       </c>
       <c r="N63" s="147">
-        <v>35005.799999999988</v>
+        <v>41880.300000000017</v>
       </c>
       <c r="O63" s="147">
-        <v>44107.700000000012</v>
+        <v>43797.200000000012</v>
       </c>
       <c r="P63" s="147">
-        <v>47008</v>
+        <v>46988.200000000012</v>
       </c>
       <c r="Q63" s="147">
         <v>49998.700000000012</v>
       </c>
       <c r="R63" s="147">
-        <v>50799.700000000012</v>
+        <v>50903.400000000023</v>
       </c>
       <c r="S63" s="147">
-        <v>52461</v>
+        <v>52299.700000000012</v>
       </c>
       <c r="T63" s="147">
-        <v>37247.099999999977</v>
+        <v>47349.400000000023</v>
       </c>
       <c r="U63" s="147">
-        <v>77263.099999999977</v>
+        <v>57263.099999999977</v>
       </c>
       <c r="V63" s="147">
-        <v>1877.9000000000233</v>
+        <v>0</v>
       </c>
       <c r="X63" s="148"/>
     </row>
@@ -31374,31 +31464,31 @@
       </c>
       <c r="J65" s="69">
         <f t="shared" si="29"/>
-        <v>1679.077777777778</v>
+        <v>1935.211111111111</v>
       </c>
       <c r="K65" s="69">
         <f t="shared" si="29"/>
-        <v>2028.9040000000002</v>
+        <v>2061.5120000000002</v>
       </c>
       <c r="L65" s="69">
         <f t="shared" si="29"/>
-        <v>2464.0562499999996</v>
+        <v>2557.1875</v>
       </c>
       <c r="M65" s="69">
         <f t="shared" si="29"/>
-        <v>1871.3666666666675</v>
+        <v>1707.5250000000003</v>
       </c>
       <c r="N65" s="69">
         <f t="shared" si="29"/>
-        <v>1458.5749999999996</v>
+        <v>1745.0125000000007</v>
       </c>
       <c r="O65" s="69">
         <f t="shared" si="29"/>
-        <v>1633.6185185185188</v>
+        <v>1622.1185185185188</v>
       </c>
       <c r="P65" s="69">
         <f t="shared" si="29"/>
-        <v>1808</v>
+        <v>1807.2384615384619</v>
       </c>
       <c r="Q65" s="69">
         <f t="shared" si="29"/>
@@ -31406,19 +31496,19 @@
       </c>
       <c r="R65" s="69">
         <f t="shared" si="29"/>
-        <v>1953.8346153846157</v>
+        <v>1957.8230769230779</v>
       </c>
       <c r="S65" s="69">
         <f t="shared" si="29"/>
-        <v>1943</v>
+        <v>1937.0259259259265</v>
       </c>
       <c r="T65" s="69">
         <f t="shared" si="29"/>
-        <v>1432.5807692307683</v>
+        <v>1821.1307692307701</v>
       </c>
       <c r="U65" s="69">
         <f t="shared" si="29"/>
-        <v>2971.6576923076914</v>
+        <v>2202.4269230769223</v>
       </c>
       <c r="V65" s="69">
         <v>0</v>
@@ -31436,6 +31526,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -31486,47 +31577,47 @@
       <c r="B2" s="46"/>
       <c r="C2" s="34">
         <f>SUM(C4:C733)</f>
-        <v>145839</v>
+        <v>151671.87999999998</v>
       </c>
       <c r="D2" s="35">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>142103.58000000007</v>
+        <v>145434.64000000007</v>
       </c>
       <c r="E2" s="36">
         <f t="shared" si="0"/>
-        <v>8038.2323076923085</v>
+        <v>2679.4107692307689</v>
       </c>
       <c r="F2" s="34">
         <f t="shared" si="0"/>
-        <v>210259.08699999994</v>
+        <v>217078.07699999996</v>
       </c>
       <c r="G2" s="35">
         <f t="shared" si="0"/>
-        <v>208717.13999999998</v>
+        <v>215263.65999999997</v>
       </c>
       <c r="H2" s="36">
         <f t="shared" si="0"/>
-        <v>7537.2738461538447</v>
+        <v>0</v>
       </c>
       <c r="I2" s="34">
         <f t="shared" si="0"/>
-        <v>17301.32</v>
+        <v>22935.920000000002</v>
       </c>
       <c r="J2" s="35">
         <f t="shared" si="0"/>
-        <v>19955.665981000002</v>
+        <v>26827.705980999999</v>
       </c>
       <c r="K2" s="36">
         <f t="shared" si="0"/>
-        <v>573333.3333333343</v>
+        <v>565555.55555555667</v>
       </c>
       <c r="L2" s="34">
         <f t="shared" si="0"/>
-        <v>367929.76222199976</v>
+        <v>384135.77222199977</v>
       </c>
       <c r="M2" s="36">
         <f t="shared" si="0"/>
-        <v>647186.7336666669</v>
+        <v>631753.81077777827</v>
       </c>
       <c r="N2" s="29"/>
     </row>
@@ -31730,7 +31821,7 @@
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
-        <v>17431.370000000003</v>
+        <v>34180.990000000005</v>
       </c>
       <c r="AA5" s="5">
         <f t="shared" si="2"/>
@@ -31817,7 +31908,7 @@
       </c>
       <c r="Z6" s="5">
         <f t="shared" si="4"/>
-        <v>38908.839487179481</v>
+        <v>18234.966324786321</v>
       </c>
       <c r="AA6" s="5">
         <f t="shared" si="4"/>
@@ -31944,7 +32035,7 @@
       </c>
       <c r="Z8" s="5">
         <f t="shared" si="5"/>
-        <v>33410.039999999994</v>
+        <v>49616.049999999996</v>
       </c>
       <c r="AA8" s="5">
         <f t="shared" si="5"/>
@@ -32031,7 +32122,7 @@
       </c>
       <c r="Z9" s="5">
         <f t="shared" si="6"/>
-        <v>46298.768666666678</v>
+        <v>30865.845777777777</v>
       </c>
       <c r="AA9" s="5">
         <f t="shared" si="6"/>
@@ -32158,15 +32249,15 @@
       </c>
       <c r="Z11" s="5">
         <f t="shared" si="7"/>
-        <v>409685.22546817944</v>
+        <v>405760.97230578633</v>
       </c>
       <c r="AA11" s="5">
         <f t="shared" si="7"/>
-        <v>459685.22546817944</v>
+        <v>455760.97230578633</v>
       </c>
       <c r="AB11" s="5">
         <f t="shared" si="7"/>
-        <v>509685.22546817944</v>
+        <v>505760.97230578633</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
@@ -32245,15 +32336,15 @@
       </c>
       <c r="Z12" s="5">
         <f t="shared" si="8"/>
-        <v>414228.53088866669</v>
+        <v>415001.61799977778</v>
       </c>
       <c r="AA12" s="5">
         <f t="shared" si="8"/>
-        <v>481534.41588866664</v>
+        <v>482307.50299977773</v>
       </c>
       <c r="AB12" s="5">
         <f t="shared" si="8"/>
-        <v>517780.7508886666</v>
+        <v>518553.83799977769</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
@@ -32332,15 +32423,15 @@
       </c>
       <c r="Z13" s="5">
         <f t="shared" si="9"/>
-        <v>-4543.305420487246</v>
+        <v>-9240.6456939914497</v>
       </c>
       <c r="AA13" s="5">
         <f t="shared" si="9"/>
-        <v>-21849.190420487197</v>
+        <v>-26546.530693991401</v>
       </c>
       <c r="AB13" s="5">
         <f t="shared" si="9"/>
-        <v>-8095.5254204871599</v>
+        <v>-12792.865693991364</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
@@ -43300,25 +43391,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C287" s="39"/>
-      <c r="D287" s="40"/>
-      <c r="E287" s="182">
-        <v>0</v>
-      </c>
-      <c r="F287" s="39"/>
-      <c r="G287" s="40"/>
-      <c r="H287" s="182">
-        <v>0</v>
-      </c>
-      <c r="I287" s="39"/>
-      <c r="J287" s="40"/>
+      <c r="C287" s="39">
+        <v>0</v>
+      </c>
+      <c r="D287" s="40">
+        <v>0</v>
+      </c>
+      <c r="E287" s="42"/>
+      <c r="F287" s="39">
+        <v>259.38</v>
+      </c>
+      <c r="G287" s="40">
+        <v>0</v>
+      </c>
+      <c r="H287" s="42"/>
+      <c r="I287" s="39">
+        <v>0</v>
+      </c>
+      <c r="J287" s="40">
+        <v>0</v>
+      </c>
       <c r="K287" s="5">
         <v>0</v>
       </c>
-      <c r="L287" s="157"/>
-      <c r="M287" s="41">
-        <v>0</v>
-      </c>
+      <c r="L287" s="157">
+        <v>0</v>
+      </c>
+      <c r="M287" s="41"/>
       <c r="O287" s="29"/>
       <c r="P287" s="5"/>
       <c r="R287" s="5"/>
@@ -43334,25 +43433,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C288" s="39"/>
-      <c r="D288" s="40"/>
-      <c r="E288" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F288" s="39"/>
-      <c r="G288" s="40"/>
-      <c r="H288" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I288" s="39"/>
-      <c r="J288" s="40"/>
+      <c r="C288" s="39">
+        <v>661.52</v>
+      </c>
+      <c r="D288" s="40">
+        <v>0</v>
+      </c>
+      <c r="E288" s="42"/>
+      <c r="F288" s="39">
+        <v>447.92</v>
+      </c>
+      <c r="G288" s="40">
+        <v>972.3</v>
+      </c>
+      <c r="H288" s="42"/>
+      <c r="I288" s="39">
+        <v>0</v>
+      </c>
+      <c r="J288" s="40">
+        <v>0</v>
+      </c>
       <c r="K288" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L288" s="157"/>
-      <c r="M288" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L288" s="157">
+        <v>764.5</v>
+      </c>
+      <c r="M288" s="41"/>
       <c r="O288" s="29"/>
       <c r="P288" s="5"/>
       <c r="R288" s="5"/>
@@ -43368,25 +43475,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C289" s="39"/>
-      <c r="D289" s="40"/>
-      <c r="E289" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F289" s="39"/>
-      <c r="G289" s="40"/>
-      <c r="H289" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I289" s="39"/>
-      <c r="J289" s="40"/>
+      <c r="C289" s="39">
+        <v>1321.81</v>
+      </c>
+      <c r="D289" s="40">
+        <v>0</v>
+      </c>
+      <c r="E289" s="42"/>
+      <c r="F289" s="39">
+        <v>1916.98</v>
+      </c>
+      <c r="G289" s="40">
+        <v>802.1400000000001</v>
+      </c>
+      <c r="H289" s="42"/>
+      <c r="I289" s="39">
+        <v>1313.4</v>
+      </c>
+      <c r="J289" s="40">
+        <v>1356.25</v>
+      </c>
       <c r="K289" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L289" s="157"/>
-      <c r="M289" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L289" s="157">
+        <v>6421.7999999999993</v>
+      </c>
+      <c r="M289" s="41"/>
       <c r="O289" s="29"/>
       <c r="P289" s="5"/>
       <c r="R289" s="5"/>
@@ -43402,25 +43517,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C290" s="39"/>
-      <c r="D290" s="40"/>
-      <c r="E290" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F290" s="39"/>
-      <c r="G290" s="40"/>
-      <c r="H290" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I290" s="39"/>
-      <c r="J290" s="40"/>
+      <c r="C290" s="39">
+        <v>1212.81</v>
+      </c>
+      <c r="D290" s="40">
+        <v>155.33999999999997</v>
+      </c>
+      <c r="E290" s="42"/>
+      <c r="F290" s="39">
+        <v>1903.8</v>
+      </c>
+      <c r="G290" s="40">
+        <v>1897.0200000000004</v>
+      </c>
+      <c r="H290" s="42"/>
+      <c r="I290" s="39">
+        <v>1379.3</v>
+      </c>
+      <c r="J290" s="40">
+        <v>1630.1699999999998</v>
+      </c>
       <c r="K290" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L290" s="157"/>
-      <c r="M290" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L290" s="157">
+        <v>1078.6399999999999</v>
+      </c>
+      <c r="M290" s="41"/>
       <c r="O290" s="29"/>
       <c r="P290" s="5"/>
       <c r="R290" s="5"/>
@@ -43436,25 +43559,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C291" s="39"/>
-      <c r="D291" s="40"/>
-      <c r="E291" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F291" s="39"/>
-      <c r="G291" s="40"/>
-      <c r="H291" s="182">
-        <v>1884.3184615384612</v>
-      </c>
-      <c r="I291" s="39"/>
-      <c r="J291" s="40"/>
+      <c r="C291" s="39">
+        <v>759.55</v>
+      </c>
+      <c r="D291" s="40">
+        <v>393.82</v>
+      </c>
+      <c r="E291" s="42"/>
+      <c r="F291" s="39">
+        <v>937.73</v>
+      </c>
+      <c r="G291" s="40">
+        <v>996.12000000000012</v>
+      </c>
+      <c r="H291" s="42"/>
+      <c r="I291" s="39">
+        <v>1605.7</v>
+      </c>
+      <c r="J291" s="40">
+        <v>1942.64</v>
+      </c>
       <c r="K291" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L291" s="157"/>
-      <c r="M291" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L291" s="157">
+        <v>0</v>
+      </c>
+      <c r="M291" s="41"/>
       <c r="O291" s="29"/>
       <c r="P291" s="5"/>
       <c r="R291" s="5"/>
@@ -43470,25 +43601,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C292" s="39"/>
-      <c r="D292" s="40"/>
-      <c r="E292" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F292" s="39"/>
-      <c r="G292" s="40"/>
-      <c r="H292" s="182">
-        <v>0</v>
-      </c>
-      <c r="I292" s="39"/>
-      <c r="J292" s="40"/>
+      <c r="C292" s="39">
+        <v>1392.37</v>
+      </c>
+      <c r="D292" s="40">
+        <v>1533.9599999999998</v>
+      </c>
+      <c r="E292" s="42"/>
+      <c r="F292" s="39">
+        <v>824.47</v>
+      </c>
+      <c r="G292" s="40">
+        <v>850.65999999999985</v>
+      </c>
+      <c r="H292" s="42"/>
+      <c r="I292" s="39">
+        <v>735.2</v>
+      </c>
+      <c r="J292" s="40">
+        <v>1092.6399999999999</v>
+      </c>
       <c r="K292" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L292" s="157"/>
-      <c r="M292" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L292" s="157">
+        <v>6014.53</v>
+      </c>
+      <c r="M292" s="41"/>
       <c r="O292" s="29"/>
       <c r="P292" s="5"/>
       <c r="R292" s="5"/>
@@ -43504,25 +43643,33 @@
         <f t="shared" si="17"/>
         <v>out/26</v>
       </c>
-      <c r="C293" s="39"/>
-      <c r="D293" s="40"/>
-      <c r="E293" s="182">
-        <v>893.13692307692304</v>
-      </c>
-      <c r="F293" s="39"/>
-      <c r="G293" s="40"/>
-      <c r="H293" s="182">
-        <v>0</v>
-      </c>
-      <c r="I293" s="39"/>
-      <c r="J293" s="40"/>
+      <c r="C293" s="39">
+        <v>484.82</v>
+      </c>
+      <c r="D293" s="40">
+        <v>1247.9399999999998</v>
+      </c>
+      <c r="E293" s="42"/>
+      <c r="F293" s="39">
+        <v>528.71</v>
+      </c>
+      <c r="G293" s="40">
+        <v>1028.28</v>
+      </c>
+      <c r="H293" s="42"/>
+      <c r="I293" s="39">
+        <v>601</v>
+      </c>
+      <c r="J293" s="40">
+        <v>850.33999999999992</v>
+      </c>
       <c r="K293" s="5">
-        <v>1296.2962962962963</v>
-      </c>
-      <c r="L293" s="157"/>
-      <c r="M293" s="41">
-        <v>2572.1538148148152</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L293" s="157">
+        <v>1926.54</v>
+      </c>
+      <c r="M293" s="41"/>
       <c r="O293" s="29"/>
       <c r="P293" s="5"/>
       <c r="R293" s="5"/>
@@ -58764,11 +58911,11 @@
         <v>21970.61</v>
       </c>
       <c r="N2" s="72">
-        <v>9480.9599999999991</v>
+        <v>9537.1200000000008</v>
       </c>
       <c r="O2" s="29">
         <f>M2-N2</f>
-        <v>12489.650000000001</v>
+        <v>12433.49</v>
       </c>
       <c r="P2" s="29"/>
       <c r="S2">
@@ -58823,18 +58970,18 @@
         <v>305602</v>
       </c>
       <c r="N3" s="72">
-        <v>180194</v>
+        <v>185168</v>
       </c>
       <c r="O3" s="29">
         <f t="shared" ref="O3:O15" si="0">M3-N3</f>
-        <v>125408</v>
+        <v>120434</v>
       </c>
       <c r="P3" s="29"/>
       <c r="Q3" s="195" t="s">
         <v>396</v>
       </c>
       <c r="R3">
-        <v>6584</v>
+        <v>6623</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -58891,18 +59038,18 @@
       </c>
       <c r="R4" s="194">
         <f>W4</f>
-        <v>9480.9599999999991</v>
+        <v>9537.1200000000008</v>
       </c>
       <c r="T4">
         <v>9659</v>
       </c>
       <c r="V4" s="193">
         <f>U2*R3</f>
-        <v>9480960</v>
+        <v>9537120</v>
       </c>
       <c r="W4" s="194">
         <f>V4/1000</f>
-        <v>9480.9599999999991</v>
+        <v>9537.1200000000008</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -59389,11 +59536,11 @@
         <v>1592</v>
       </c>
       <c r="N14" s="72">
-        <v>483</v>
+        <v>603</v>
       </c>
       <c r="O14" s="29">
         <f t="shared" si="0"/>
-        <v>1109</v>
+        <v>989</v>
       </c>
       <c r="P14" s="29"/>
     </row>
@@ -59435,14 +59582,14 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="72">
-        <v>373978.08</v>
+        <v>392805.34</v>
       </c>
       <c r="N15" s="72">
-        <v>372154.01</v>
+        <v>389206.69</v>
       </c>
       <c r="O15" s="29">
         <f t="shared" si="0"/>
-        <v>1824.070000000007</v>
+        <v>3598.6500000000233</v>
       </c>
       <c r="P15" s="29"/>
     </row>

</xml_diff>